<commit_message>
chore: monitoring 13/09/2026 12:42
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 82j (04/12/2026)</t>
+          <t>Valide 81j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>82j</t>
+          <t>81j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 173j (05/03/2027)</t>
+          <t>Valide 172j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>12/09/2026 11:31</t>
+          <t>13/09/2026 12:36</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 328j (07/08/2027)</t>
+          <t>Valide 327j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>12/09/2026 11:31</t>
+          <t>13/09/2026 12:36</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 50j (02/11/2026)</t>
+          <t>Valide 49j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>50j</t>
+          <t>49j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 135j (26/01/2027)</t>
+          <t>Valide 134j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>12/09/2026 11:31</t>
+          <t>13/09/2026 12:36</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 69j (20/11/2026)</t>
+          <t>Valide 68j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>69j</t>
+          <t>68j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 51j (02/11/2026)</t>
+          <t>Valide 49j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>12/09/2026 11:31</t>
+          <t>13/09/2026 12:36</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 150j (09/02/2027)</t>
+          <t>Valide 149j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>150j</t>
+          <t>149j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 168j (28/02/2027)</t>
+          <t>Valide 167j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>12/09/2026 11:31</t>
+          <t>13/09/2026 12:36</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 148j (07/02/2027)</t>
+          <t>Valide 147j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>148j</t>
+          <t>147j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 312j (22/07/2027)</t>
+          <t>Valide 311j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>12/09/2026 11:31</t>
+          <t>13/09/2026 12:36</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 32j (14/10/2026)</t>
+          <t>Valide 31j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>32j</t>
+          <t>31j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>12/09/2026 11:31</t>
+          <t>13/09/2026 12:36</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 47j (29/10/2026)</t>
+          <t>Valide 46j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>47j</t>
+          <t>46j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 86j (07/12/2026)</t>
+          <t>Valide 85j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>12/09/2026 11:31</t>
+          <t>13/09/2026 12:36</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 47j (29/10/2026)</t>
+          <t>Valide 46j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>47j</t>
+          <t>46j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 86j (07/12/2026)</t>
+          <t>Valide 85j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>12/09/2026 11:31</t>
+          <t>13/09/2026 12:36</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 27j (09/10/2026)</t>
+          <t>Expire dans 26j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>27j</t>
+          <t>26j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 79j (30/11/2026)</t>
+          <t>Valide 78j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>12/09/2026 11:31</t>
+          <t>13/09/2026 12:36</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 27j (09/10/2026)</t>
+          <t>Expire dans 26j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>27j</t>
+          <t>26j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 79j (30/11/2026)</t>
+          <t>Valide 78j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>12/09/2026 11:31</t>
+          <t>13/09/2026 12:36</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 150j (09/02/2027)</t>
+          <t>Valide 149j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>150j</t>
+          <t>149j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 69j (20/11/2026)</t>
+          <t>Valide 68j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>12/09/2026 11:31</t>
+          <t>13/09/2026 12:36</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 150j (09/02/2027)</t>
+          <t>Valide 149j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>150j</t>
+          <t>149j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 69j (20/11/2026)</t>
+          <t>Valide 68j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>12/09/2026 11:31</t>
+          <t>13/09/2026 12:36</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 98j (19/12/2026)</t>
+          <t>Valide 97j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>98j</t>
+          <t>97j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 321j (31/07/2027)</t>
+          <t>Valide 320j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>12/09/2026 11:31</t>
+          <t>13/09/2026 12:36</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 98j (19/12/2026)</t>
+          <t>Valide 97j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>98j</t>
+          <t>97j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 321j (31/07/2027)</t>
+          <t>Valide 320j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>12/09/2026 11:31</t>
+          <t>13/09/2026 12:36</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,25 +2725,29 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 31j (13/10/2026)</t>
+          <t>Expire dans 30j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>31j</t>
+          <t>30j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 28j (10/10/2026)</t>
+          <t>Expire dans 27j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>12/09/2026 11:31</t>
-        </is>
-      </c>
-      <c r="P49" t="inlineStr"/>
+          <t>13/09/2026 12:36</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1" s="34">
       <c r="A50" s="3" t="inlineStr">

</xml_diff>

<commit_message>
chore: monitoring 14/09/2026 13:51
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 81j (04/12/2026)</t>
+          <t>Valide 80j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>81j</t>
+          <t>80j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 172j (05/03/2027)</t>
+          <t>Valide 171j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>13/09/2026 12:36</t>
+          <t>14/09/2026 13:45</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 146j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>146j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 327j (07/08/2027)</t>
+          <t>Valide 326j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>13/09/2026 12:36</t>
+          <t>14/09/2026 13:45</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 49j (02/11/2026)</t>
+          <t>Valide 48j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>49j</t>
+          <t>48j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 134j (26/01/2027)</t>
+          <t>Valide 133j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>13/09/2026 12:36</t>
+          <t>14/09/2026 13:45</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 68j (20/11/2026)</t>
+          <t>Valide 67j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>68j</t>
+          <t>67j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 49j (02/11/2026)</t>
+          <t>Valide 48j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>13/09/2026 12:36</t>
+          <t>14/09/2026 13:45</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 149j (09/02/2027)</t>
+          <t>Valide 148j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>149j</t>
+          <t>148j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 167j (28/02/2027)</t>
+          <t>Valide 166j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>13/09/2026 12:36</t>
+          <t>14/09/2026 13:45</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 147j (07/02/2027)</t>
+          <t>Valide 146j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>147j</t>
+          <t>146j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 311j (22/07/2027)</t>
+          <t>Valide 310j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>13/09/2026 12:36</t>
+          <t>14/09/2026 13:45</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 31j (14/10/2026)</t>
+          <t>Expire dans 30j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>31j</t>
+          <t>30j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,10 +1665,14 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>13/09/2026 12:36</t>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr"/>
+          <t>14/09/2026 13:45</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
       <c r="R23" t="inlineStr">
         <is>
           <t>x</t>
@@ -1745,22 +1749,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 46j (29/10/2026)</t>
+          <t>Valide 45j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>46j</t>
+          <t>45j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 85j (07/12/2026)</t>
+          <t>Valide 84j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>13/09/2026 12:36</t>
+          <t>14/09/2026 13:45</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1815,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 46j (29/10/2026)</t>
+          <t>Valide 45j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>46j</t>
+          <t>45j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 85j (07/12/2026)</t>
+          <t>Valide 84j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>13/09/2026 12:36</t>
+          <t>14/09/2026 13:45</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1961,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 26j (09/10/2026)</t>
+          <t>Expire dans 25j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>26j</t>
+          <t>25j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 78j (30/11/2026)</t>
+          <t>Valide 77j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>13/09/2026 12:36</t>
+          <t>14/09/2026 13:45</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2011,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 26j (09/10/2026)</t>
+          <t>Expire dans 25j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>26j</t>
+          <t>25j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 78j (30/11/2026)</t>
+          <t>Valide 77j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>13/09/2026 12:36</t>
+          <t>14/09/2026 13:45</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2189,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 149j (09/02/2027)</t>
+          <t>Valide 148j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>149j</t>
+          <t>148j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 68j (20/11/2026)</t>
+          <t>Valide 67j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>13/09/2026 12:36</t>
+          <t>14/09/2026 13:45</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2251,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 149j (09/02/2027)</t>
+          <t>Valide 148j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>149j</t>
+          <t>148j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 68j (20/11/2026)</t>
+          <t>Valide 67j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>13/09/2026 12:36</t>
+          <t>14/09/2026 13:45</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2461,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 97j (19/12/2026)</t>
+          <t>Valide 96j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>97j</t>
+          <t>96j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 320j (31/07/2027)</t>
+          <t>Valide 319j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>13/09/2026 12:36</t>
+          <t>14/09/2026 13:45</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2515,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 97j (19/12/2026)</t>
+          <t>Valide 96j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>97j</t>
+          <t>96j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 320j (31/07/2027)</t>
+          <t>Valide 319j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>13/09/2026 12:36</t>
+          <t>14/09/2026 13:45</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,29 +2729,25 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 30j (13/10/2026)</t>
+          <t>Expire dans 29j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>30j</t>
+          <t>29j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 27j (10/10/2026)</t>
+          <t>Expire dans 25j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>13/09/2026 12:36</t>
-        </is>
-      </c>
-      <c r="P49" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>14/09/2026 13:45</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr"/>
     </row>
     <row r="50" ht="18" customHeight="1" s="34">
       <c r="A50" s="3" t="inlineStr">

</xml_diff>

<commit_message>
chore: monitoring 15/09/2026 12:39
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 80j (04/12/2026)</t>
+          <t>Valide 79j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>80j</t>
+          <t>79j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 171j (05/03/2027)</t>
+          <t>Valide 170j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>14/09/2026 13:45</t>
+          <t>15/09/2026 12:31</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 146j (07/02/2027)</t>
+          <t>Valide 145j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>146j</t>
+          <t>145j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 326j (07/08/2027)</t>
+          <t>Valide 325j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>14/09/2026 13:45</t>
+          <t>15/09/2026 12:31</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 48j (02/11/2026)</t>
+          <t>Valide 47j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>48j</t>
+          <t>47j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 133j (26/01/2027)</t>
+          <t>Valide 132j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>14/09/2026 13:45</t>
+          <t>15/09/2026 12:31</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 67j (20/11/2026)</t>
+          <t>Valide 66j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>67j</t>
+          <t>66j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 48j (02/11/2026)</t>
+          <t>Valide 47j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>14/09/2026 13:45</t>
+          <t>15/09/2026 12:31</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 148j (09/02/2027)</t>
+          <t>Valide 147j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>148j</t>
+          <t>147j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 166j (28/02/2027)</t>
+          <t>Valide 165j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>14/09/2026 13:45</t>
+          <t>15/09/2026 12:31</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 146j (07/02/2027)</t>
+          <t>Valide 145j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>146j</t>
+          <t>145j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 310j (22/07/2027)</t>
+          <t>Valide 309j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>14/09/2026 13:45</t>
+          <t>15/09/2026 12:31</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 30j (14/10/2026)</t>
+          <t>Expire dans 29j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>30j</t>
+          <t>29j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,14 +1665,10 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>14/09/2026 13:45</t>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>15/09/2026 12:31</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
           <t>x</t>
@@ -1749,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 45j (29/10/2026)</t>
+          <t>Valide 44j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>45j</t>
+          <t>44j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 84j (07/12/2026)</t>
+          <t>Valide 83j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>14/09/2026 13:45</t>
+          <t>15/09/2026 12:31</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1815,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 45j (29/10/2026)</t>
+          <t>Valide 44j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>45j</t>
+          <t>44j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 84j (07/12/2026)</t>
+          <t>Valide 83j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>14/09/2026 13:45</t>
+          <t>15/09/2026 12:31</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1961,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 25j (09/10/2026)</t>
+          <t>Expire dans 24j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>25j</t>
+          <t>24j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 77j (30/11/2026)</t>
+          <t>Valide 76j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>14/09/2026 13:45</t>
+          <t>15/09/2026 12:31</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2011,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 25j (09/10/2026)</t>
+          <t>Expire dans 24j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>25j</t>
+          <t>24j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 77j (30/11/2026)</t>
+          <t>Valide 76j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>14/09/2026 13:45</t>
+          <t>15/09/2026 12:31</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2189,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 148j (09/02/2027)</t>
+          <t>Valide 147j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>148j</t>
+          <t>147j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 67j (20/11/2026)</t>
+          <t>Valide 66j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>14/09/2026 13:45</t>
+          <t>15/09/2026 12:31</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2251,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 148j (09/02/2027)</t>
+          <t>Valide 147j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>148j</t>
+          <t>147j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 67j (20/11/2026)</t>
+          <t>Valide 66j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>14/09/2026 13:45</t>
+          <t>15/09/2026 12:31</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2461,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 96j (19/12/2026)</t>
+          <t>Valide 95j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>96j</t>
+          <t>95j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 319j (31/07/2027)</t>
+          <t>Valide 318j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>14/09/2026 13:45</t>
+          <t>15/09/2026 12:31</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2515,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 96j (19/12/2026)</t>
+          <t>Valide 95j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>96j</t>
+          <t>95j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 319j (31/07/2027)</t>
+          <t>Valide 318j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>14/09/2026 13:45</t>
+          <t>15/09/2026 12:31</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2729,12 +2725,12 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 29j (13/10/2026)</t>
+          <t>Expire dans 28j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>29j</t>
+          <t>28j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
@@ -2744,7 +2740,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>14/09/2026 13:45</t>
+          <t>15/09/2026 12:31</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 16/09/2026 12:36
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 79j (04/12/2026)</t>
+          <t>Valide 78j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>79j</t>
+          <t>78j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 170j (05/03/2027)</t>
+          <t>Valide 169j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>15/09/2026 12:31</t>
+          <t>16/09/2026 12:29</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 145j (07/02/2027)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>145j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 325j (07/08/2027)</t>
+          <t>Valide 324j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>15/09/2026 12:31</t>
+          <t>16/09/2026 12:29</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 47j (02/11/2026)</t>
+          <t>Valide 46j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>47j</t>
+          <t>46j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 132j (26/01/2027)</t>
+          <t>Valide 131j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>15/09/2026 12:31</t>
+          <t>16/09/2026 12:29</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 66j (20/11/2026)</t>
+          <t>Valide 65j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>66j</t>
+          <t>65j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 47j (02/11/2026)</t>
+          <t>Valide 46j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>15/09/2026 12:31</t>
+          <t>16/09/2026 12:29</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 147j (09/02/2027)</t>
+          <t>Valide 146j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>147j</t>
+          <t>146j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 165j (28/02/2027)</t>
+          <t>Valide 164j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>15/09/2026 12:31</t>
+          <t>16/09/2026 12:29</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 145j (07/02/2027)</t>
+          <t>Valide 144j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>145j</t>
+          <t>144j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 309j (22/07/2027)</t>
+          <t>Valide 308j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>15/09/2026 12:31</t>
+          <t>16/09/2026 12:29</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 29j (14/10/2026)</t>
+          <t>Expire dans 28j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>29j</t>
+          <t>28j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>15/09/2026 12:31</t>
+          <t>16/09/2026 12:29</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 44j (29/10/2026)</t>
+          <t>Valide 43j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>44j</t>
+          <t>43j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 83j (07/12/2026)</t>
+          <t>Valide 82j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>15/09/2026 12:31</t>
+          <t>16/09/2026 12:29</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 44j (29/10/2026)</t>
+          <t>Valide 43j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>44j</t>
+          <t>43j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 83j (07/12/2026)</t>
+          <t>Valide 82j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>15/09/2026 12:31</t>
+          <t>16/09/2026 12:29</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 24j (09/10/2026)</t>
+          <t>Expire dans 23j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>24j</t>
+          <t>23j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 76j (30/11/2026)</t>
+          <t>Valide 75j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>15/09/2026 12:31</t>
+          <t>16/09/2026 12:29</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 24j (09/10/2026)</t>
+          <t>Expire dans 23j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>24j</t>
+          <t>23j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 76j (30/11/2026)</t>
+          <t>Valide 75j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>15/09/2026 12:31</t>
+          <t>16/09/2026 12:29</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 147j (09/02/2027)</t>
+          <t>Valide 146j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>147j</t>
+          <t>146j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 66j (20/11/2026)</t>
+          <t>Valide 65j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>15/09/2026 12:31</t>
+          <t>16/09/2026 12:29</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 147j (09/02/2027)</t>
+          <t>Valide 146j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>147j</t>
+          <t>146j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 66j (20/11/2026)</t>
+          <t>Valide 65j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>15/09/2026 12:31</t>
+          <t>16/09/2026 12:29</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 95j (19/12/2026)</t>
+          <t>Valide 94j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>95j</t>
+          <t>94j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 318j (31/07/2027)</t>
+          <t>Valide 317j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>15/09/2026 12:31</t>
+          <t>16/09/2026 12:29</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 95j (19/12/2026)</t>
+          <t>Valide 94j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>95j</t>
+          <t>94j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 318j (31/07/2027)</t>
+          <t>Valide 317j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>15/09/2026 12:31</t>
+          <t>16/09/2026 12:29</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 28j (13/10/2026)</t>
+          <t>Expire dans 27j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>28j</t>
+          <t>27j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 25j (10/10/2026)</t>
+          <t>Expire dans 24j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>15/09/2026 12:31</t>
+          <t>16/09/2026 12:29</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 17/09/2026 12:36
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 78j (04/12/2026)</t>
+          <t>Valide 77j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>78j</t>
+          <t>77j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 169j (05/03/2027)</t>
+          <t>Valide 168j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>16/09/2026 12:29</t>
+          <t>17/09/2026 12:29</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 324j (07/08/2027)</t>
+          <t>Valide 323j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>16/09/2026 12:29</t>
+          <t>17/09/2026 12:29</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 46j (02/11/2026)</t>
+          <t>Valide 45j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>46j</t>
+          <t>45j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 131j (26/01/2027)</t>
+          <t>Valide 130j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>16/09/2026 12:29</t>
+          <t>17/09/2026 12:29</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 65j (20/11/2026)</t>
+          <t>Valide 64j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>65j</t>
+          <t>64j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 46j (02/11/2026)</t>
+          <t>Valide 45j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>16/09/2026 12:29</t>
+          <t>17/09/2026 12:29</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 146j (09/02/2027)</t>
+          <t>Valide 145j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>146j</t>
+          <t>145j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 164j (28/02/2027)</t>
+          <t>Valide 163j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>16/09/2026 12:29</t>
+          <t>17/09/2026 12:29</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 144j (07/02/2027)</t>
+          <t>Valide 143j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>144j</t>
+          <t>143j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 308j (22/07/2027)</t>
+          <t>Valide 307j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>16/09/2026 12:29</t>
+          <t>17/09/2026 12:29</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 28j (14/10/2026)</t>
+          <t>Expire dans 27j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>28j</t>
+          <t>27j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>16/09/2026 12:29</t>
+          <t>17/09/2026 12:29</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 43j (29/10/2026)</t>
+          <t>Valide 42j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>43j</t>
+          <t>42j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 82j (07/12/2026)</t>
+          <t>Valide 81j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>16/09/2026 12:29</t>
+          <t>17/09/2026 12:29</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 43j (29/10/2026)</t>
+          <t>Valide 42j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>43j</t>
+          <t>42j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 82j (07/12/2026)</t>
+          <t>Valide 81j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>16/09/2026 12:29</t>
+          <t>17/09/2026 12:29</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 23j (09/10/2026)</t>
+          <t>Expire dans 22j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>23j</t>
+          <t>22j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 75j (30/11/2026)</t>
+          <t>Valide 74j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>16/09/2026 12:29</t>
+          <t>17/09/2026 12:29</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 23j (09/10/2026)</t>
+          <t>Expire dans 22j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>23j</t>
+          <t>22j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 75j (30/11/2026)</t>
+          <t>Valide 74j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>16/09/2026 12:29</t>
+          <t>17/09/2026 12:29</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 146j (09/02/2027)</t>
+          <t>Valide 145j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>146j</t>
+          <t>145j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 65j (20/11/2026)</t>
+          <t>Valide 64j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>16/09/2026 12:29</t>
+          <t>17/09/2026 12:29</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 146j (09/02/2027)</t>
+          <t>Valide 145j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>146j</t>
+          <t>145j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 65j (20/11/2026)</t>
+          <t>Valide 64j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>16/09/2026 12:29</t>
+          <t>17/09/2026 12:29</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 94j (19/12/2026)</t>
+          <t>Valide 93j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>94j</t>
+          <t>93j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 317j (31/07/2027)</t>
+          <t>Valide 316j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>16/09/2026 12:29</t>
+          <t>17/09/2026 12:29</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 94j (19/12/2026)</t>
+          <t>Valide 93j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>94j</t>
+          <t>93j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 317j (31/07/2027)</t>
+          <t>Valide 316j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>16/09/2026 12:29</t>
+          <t>17/09/2026 12:29</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 27j (13/10/2026)</t>
+          <t>Expire dans 26j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>27j</t>
+          <t>26j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 24j (10/10/2026)</t>
+          <t>Valide 388j (10/10/2027)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>16/09/2026 12:29</t>
+          <t>17/09/2026 12:29</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 18/09/2026 12:15
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 77j (04/12/2026)</t>
+          <t>Valide 76j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>77j</t>
+          <t>76j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 168j (05/03/2027)</t>
+          <t>Valide 167j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>17/09/2026 12:29</t>
+          <t>18/09/2026 12:07</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 142j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>142j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 323j (07/08/2027)</t>
+          <t>Valide 322j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>17/09/2026 12:29</t>
+          <t>18/09/2026 12:07</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 45j (02/11/2026)</t>
+          <t>Valide 44j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>45j</t>
+          <t>44j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 130j (26/01/2027)</t>
+          <t>Valide 129j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>17/09/2026 12:29</t>
+          <t>18/09/2026 12:07</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,12 +1152,12 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 64j (20/11/2026)</t>
+          <t>Valide 63j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>64j</t>
+          <t>63j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>17/09/2026 12:29</t>
+          <t>18/09/2026 12:07</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 145j (09/02/2027)</t>
+          <t>Valide 144j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>145j</t>
+          <t>144j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 163j (28/02/2027)</t>
+          <t>Valide 162j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>17/09/2026 12:29</t>
+          <t>18/09/2026 12:07</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 143j (07/02/2027)</t>
+          <t>Valide 142j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>143j</t>
+          <t>142j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 307j (22/07/2027)</t>
+          <t>Valide 306j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>17/09/2026 12:29</t>
+          <t>18/09/2026 12:07</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 27j (14/10/2026)</t>
+          <t>Expire dans 26j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>27j</t>
+          <t>26j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>17/09/2026 12:29</t>
+          <t>18/09/2026 12:07</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 42j (29/10/2026)</t>
+          <t>Valide 41j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>42j</t>
+          <t>41j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 81j (07/12/2026)</t>
+          <t>Valide 80j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>17/09/2026 12:29</t>
+          <t>18/09/2026 12:07</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 42j (29/10/2026)</t>
+          <t>Valide 41j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>42j</t>
+          <t>41j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 81j (07/12/2026)</t>
+          <t>Valide 80j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>17/09/2026 12:29</t>
+          <t>18/09/2026 12:07</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 22j (09/10/2026)</t>
+          <t>Expire dans 21j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>22j</t>
+          <t>21j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 74j (30/11/2026)</t>
+          <t>Valide 73j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>17/09/2026 12:29</t>
+          <t>18/09/2026 12:07</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 22j (09/10/2026)</t>
+          <t>Expire dans 21j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>22j</t>
+          <t>21j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 74j (30/11/2026)</t>
+          <t>Valide 73j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>17/09/2026 12:29</t>
+          <t>18/09/2026 12:07</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 145j (09/02/2027)</t>
+          <t>Valide 144j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>145j</t>
+          <t>144j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 64j (20/11/2026)</t>
+          <t>Valide 63j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>17/09/2026 12:29</t>
+          <t>18/09/2026 12:07</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 145j (09/02/2027)</t>
+          <t>Valide 144j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>145j</t>
+          <t>144j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 64j (20/11/2026)</t>
+          <t>Valide 63j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>17/09/2026 12:29</t>
+          <t>18/09/2026 12:07</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 93j (19/12/2026)</t>
+          <t>Valide 92j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>93j</t>
+          <t>92j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 316j (31/07/2027)</t>
+          <t>Valide 315j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>17/09/2026 12:29</t>
+          <t>18/09/2026 12:07</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 93j (19/12/2026)</t>
+          <t>Valide 92j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>93j</t>
+          <t>92j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 316j (31/07/2027)</t>
+          <t>Valide 315j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>17/09/2026 12:29</t>
+          <t>18/09/2026 12:07</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 26j (13/10/2026)</t>
+          <t>Expire dans 25j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>26j</t>
+          <t>25j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 388j (10/10/2027)</t>
+          <t>Valide 387j (10/10/2027)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>17/09/2026 12:29</t>
+          <t>18/09/2026 12:07</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 19/09/2026 11:57
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 76j (04/12/2026)</t>
+          <t>Valide 75j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>76j</t>
+          <t>75j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 167j (05/03/2027)</t>
+          <t>Valide 166j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>18/09/2026 12:07</t>
+          <t>19/09/2026 11:50</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 142j (07/02/2027)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>142j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 322j (07/08/2027)</t>
+          <t>Valide 321j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>18/09/2026 12:07</t>
+          <t>19/09/2026 11:50</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 44j (02/11/2026)</t>
+          <t>Valide 43j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>44j</t>
+          <t>43j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 129j (26/01/2027)</t>
+          <t>Valide 128j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>18/09/2026 12:07</t>
+          <t>19/09/2026 11:50</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 63j (20/11/2026)</t>
+          <t>Valide 62j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>63j</t>
+          <t>62j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 45j (02/11/2026)</t>
+          <t>Valide 44j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>18/09/2026 12:07</t>
+          <t>19/09/2026 11:50</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 144j (09/02/2027)</t>
+          <t>Valide 143j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>144j</t>
+          <t>143j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 162j (28/02/2027)</t>
+          <t>Valide 161j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>18/09/2026 12:07</t>
+          <t>19/09/2026 11:50</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 142j (07/02/2027)</t>
+          <t>Valide 141j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>142j</t>
+          <t>141j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 306j (22/07/2027)</t>
+          <t>Valide 305j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>18/09/2026 12:07</t>
+          <t>19/09/2026 11:50</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 26j (14/10/2026)</t>
+          <t>Expire dans 25j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>26j</t>
+          <t>25j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>18/09/2026 12:07</t>
+          <t>19/09/2026 11:50</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 41j (29/10/2026)</t>
+          <t>Valide 40j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>41j</t>
+          <t>40j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 80j (07/12/2026)</t>
+          <t>Valide 79j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>18/09/2026 12:07</t>
+          <t>19/09/2026 11:50</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 41j (29/10/2026)</t>
+          <t>Valide 40j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>41j</t>
+          <t>40j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 80j (07/12/2026)</t>
+          <t>Valide 79j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>18/09/2026 12:07</t>
+          <t>19/09/2026 11:50</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 21j (09/10/2026)</t>
+          <t>Expire dans 20j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>21j</t>
+          <t>20j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 73j (30/11/2026)</t>
+          <t>Valide 72j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>18/09/2026 12:07</t>
+          <t>19/09/2026 11:50</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 21j (09/10/2026)</t>
+          <t>Expire dans 20j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>21j</t>
+          <t>20j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 73j (30/11/2026)</t>
+          <t>Valide 72j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>18/09/2026 12:07</t>
+          <t>19/09/2026 11:50</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 144j (09/02/2027)</t>
+          <t>Valide 143j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>144j</t>
+          <t>143j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 63j (20/11/2026)</t>
+          <t>Valide 62j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>18/09/2026 12:07</t>
+          <t>19/09/2026 11:50</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 144j (09/02/2027)</t>
+          <t>Valide 143j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>144j</t>
+          <t>143j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 63j (20/11/2026)</t>
+          <t>Valide 62j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>18/09/2026 12:07</t>
+          <t>19/09/2026 11:50</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 92j (19/12/2026)</t>
+          <t>Valide 91j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>92j</t>
+          <t>91j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 315j (31/07/2027)</t>
+          <t>Valide 314j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>18/09/2026 12:07</t>
+          <t>19/09/2026 11:50</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 92j (19/12/2026)</t>
+          <t>Valide 91j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>92j</t>
+          <t>91j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 315j (31/07/2027)</t>
+          <t>Valide 314j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>18/09/2026 12:07</t>
+          <t>19/09/2026 11:50</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 25j (13/10/2026)</t>
+          <t>Expire dans 24j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>25j</t>
+          <t>24j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 387j (10/10/2027)</t>
+          <t>Valide 386j (10/10/2027)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>18/09/2026 12:07</t>
+          <t>19/09/2026 11:50</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 20/09/2026 12:13
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 75j (04/12/2026)</t>
+          <t>Valide 74j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>75j</t>
+          <t>74j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 166j (05/03/2027)</t>
+          <t>Valide 165j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>19/09/2026 11:50</t>
+          <t>20/09/2026 12:07</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 321j (07/08/2027)</t>
+          <t>Valide 320j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>19/09/2026 11:50</t>
+          <t>20/09/2026 12:07</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 43j (02/11/2026)</t>
+          <t>Valide 42j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>43j</t>
+          <t>42j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 128j (26/01/2027)</t>
+          <t>Valide 127j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>19/09/2026 11:50</t>
+          <t>20/09/2026 12:07</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 62j (20/11/2026)</t>
+          <t>Valide 61j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>62j</t>
+          <t>61j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 44j (02/11/2026)</t>
+          <t>Valide 43j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>19/09/2026 11:50</t>
+          <t>20/09/2026 12:07</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 143j (09/02/2027)</t>
+          <t>Valide 142j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>143j</t>
+          <t>142j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 161j (28/02/2027)</t>
+          <t>Valide 160j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>19/09/2026 11:50</t>
+          <t>20/09/2026 12:07</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 141j (07/02/2027)</t>
+          <t>Valide 140j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>141j</t>
+          <t>140j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 305j (22/07/2027)</t>
+          <t>Valide 304j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>19/09/2026 11:50</t>
+          <t>20/09/2026 12:07</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 25j (14/10/2026)</t>
+          <t>Expire dans 24j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>25j</t>
+          <t>24j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>19/09/2026 11:50</t>
+          <t>20/09/2026 12:07</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 40j (29/10/2026)</t>
+          <t>Valide 39j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>40j</t>
+          <t>39j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 79j (07/12/2026)</t>
+          <t>Valide 78j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>19/09/2026 11:50</t>
+          <t>20/09/2026 12:07</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 40j (29/10/2026)</t>
+          <t>Valide 39j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>40j</t>
+          <t>39j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 79j (07/12/2026)</t>
+          <t>Valide 78j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>19/09/2026 11:50</t>
+          <t>20/09/2026 12:07</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 20j (09/10/2026)</t>
+          <t>Expire dans 19j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>20j</t>
+          <t>19j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 72j (30/11/2026)</t>
+          <t>Valide 71j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>19/09/2026 11:50</t>
+          <t>20/09/2026 12:07</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 20j (09/10/2026)</t>
+          <t>Expire dans 19j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>20j</t>
+          <t>19j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 72j (30/11/2026)</t>
+          <t>Valide 71j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>19/09/2026 11:50</t>
+          <t>20/09/2026 12:07</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 143j (09/02/2027)</t>
+          <t>Valide 142j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>143j</t>
+          <t>142j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 62j (20/11/2026)</t>
+          <t>Valide 61j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>19/09/2026 11:50</t>
+          <t>20/09/2026 12:07</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 143j (09/02/2027)</t>
+          <t>Valide 142j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>143j</t>
+          <t>142j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 62j (20/11/2026)</t>
+          <t>Valide 61j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>19/09/2026 11:50</t>
+          <t>20/09/2026 12:07</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 91j (19/12/2026)</t>
+          <t>Valide 90j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>91j</t>
+          <t>90j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 314j (31/07/2027)</t>
+          <t>Valide 313j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>19/09/2026 11:50</t>
+          <t>20/09/2026 12:07</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 91j (19/12/2026)</t>
+          <t>Valide 90j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>91j</t>
+          <t>90j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 314j (31/07/2027)</t>
+          <t>Valide 313j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>19/09/2026 11:50</t>
+          <t>20/09/2026 12:07</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 24j (13/10/2026)</t>
+          <t>Expire dans 23j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>24j</t>
+          <t>23j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 386j (10/10/2027)</t>
+          <t>Valide 385j (10/10/2027)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>19/09/2026 11:50</t>
+          <t>20/09/2026 12:07</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 21/09/2026 13:52
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 74j (04/12/2026)</t>
+          <t>Valide 73j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>74j</t>
+          <t>73j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 165j (05/03/2027)</t>
+          <t>Valide 164j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>20/09/2026 12:07</t>
+          <t>21/09/2026 13:45</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 320j (07/08/2027)</t>
+          <t>Valide 319j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>20/09/2026 12:07</t>
+          <t>21/09/2026 13:45</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 42j (02/11/2026)</t>
+          <t>Valide 41j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>42j</t>
+          <t>41j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 127j (26/01/2027)</t>
+          <t>Valide 126j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>20/09/2026 12:07</t>
+          <t>21/09/2026 13:45</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 61j (20/11/2026)</t>
+          <t>Valide 60j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>61j</t>
+          <t>60j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 43j (02/11/2026)</t>
+          <t>Valide 41j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>20/09/2026 12:07</t>
+          <t>21/09/2026 13:45</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 142j (09/02/2027)</t>
+          <t>Valide 141j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>142j</t>
+          <t>141j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 160j (28/02/2027)</t>
+          <t>Valide 159j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>20/09/2026 12:07</t>
+          <t>21/09/2026 13:45</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 140j (07/02/2027)</t>
+          <t>Valide 139j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>140j</t>
+          <t>139j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 304j (22/07/2027)</t>
+          <t>Valide 303j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>20/09/2026 12:07</t>
+          <t>21/09/2026 13:45</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 24j (14/10/2026)</t>
+          <t>Expire dans 23j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>24j</t>
+          <t>23j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>20/09/2026 12:07</t>
+          <t>21/09/2026 13:45</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 39j (29/10/2026)</t>
+          <t>Valide 38j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>39j</t>
+          <t>38j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 78j (07/12/2026)</t>
+          <t>Valide 77j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>20/09/2026 12:07</t>
+          <t>21/09/2026 13:45</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 39j (29/10/2026)</t>
+          <t>Valide 38j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>39j</t>
+          <t>38j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 78j (07/12/2026)</t>
+          <t>Valide 77j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>20/09/2026 12:07</t>
+          <t>21/09/2026 13:45</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 19j (09/10/2026)</t>
+          <t>Expire dans 18j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>19j</t>
+          <t>18j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 71j (30/11/2026)</t>
+          <t>Valide 70j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>20/09/2026 12:07</t>
+          <t>21/09/2026 13:45</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 19j (09/10/2026)</t>
+          <t>Expire dans 18j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>19j</t>
+          <t>18j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 71j (30/11/2026)</t>
+          <t>Valide 70j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>20/09/2026 12:07</t>
+          <t>21/09/2026 13:45</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 142j (09/02/2027)</t>
+          <t>Valide 141j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>142j</t>
+          <t>141j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 61j (20/11/2026)</t>
+          <t>Valide 60j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>20/09/2026 12:07</t>
+          <t>21/09/2026 13:45</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 142j (09/02/2027)</t>
+          <t>Valide 141j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>142j</t>
+          <t>141j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 61j (20/11/2026)</t>
+          <t>Valide 60j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>20/09/2026 12:07</t>
+          <t>21/09/2026 13:45</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 90j (19/12/2026)</t>
+          <t>Valide 89j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>90j</t>
+          <t>89j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 313j (31/07/2027)</t>
+          <t>Valide 312j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>20/09/2026 12:07</t>
+          <t>21/09/2026 13:45</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 90j (19/12/2026)</t>
+          <t>Valide 89j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>90j</t>
+          <t>89j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 313j (31/07/2027)</t>
+          <t>Valide 312j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>20/09/2026 12:07</t>
+          <t>21/09/2026 13:45</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 23j (13/10/2026)</t>
+          <t>Expire dans 22j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>23j</t>
+          <t>22j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 385j (10/10/2027)</t>
+          <t>Valide 383j (10/10/2027)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>20/09/2026 12:07</t>
+          <t>21/09/2026 13:45</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 22/09/2026 12:33
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 73j (04/12/2026)</t>
+          <t>Valide 72j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>73j</t>
+          <t>72j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 164j (05/03/2027)</t>
+          <t>Valide 163j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>21/09/2026 13:45</t>
+          <t>22/09/2026 12:28</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 138j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>138j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 319j (07/08/2027)</t>
+          <t>Valide 318j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>21/09/2026 13:45</t>
+          <t>22/09/2026 12:28</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 41j (02/11/2026)</t>
+          <t>Valide 40j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>41j</t>
+          <t>40j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 126j (26/01/2027)</t>
+          <t>Valide 125j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>21/09/2026 13:45</t>
+          <t>22/09/2026 12:28</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 60j (20/11/2026)</t>
+          <t>Valide 59j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>60j</t>
+          <t>59j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 41j (02/11/2026)</t>
+          <t>Valide 40j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>21/09/2026 13:45</t>
+          <t>22/09/2026 12:28</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 141j (09/02/2027)</t>
+          <t>Valide 140j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>141j</t>
+          <t>140j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 159j (28/02/2027)</t>
+          <t>Valide 158j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>21/09/2026 13:45</t>
+          <t>22/09/2026 12:28</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 139j (07/02/2027)</t>
+          <t>Valide 138j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>139j</t>
+          <t>138j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 303j (22/07/2027)</t>
+          <t>Valide 302j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>21/09/2026 13:45</t>
+          <t>22/09/2026 12:28</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 23j (14/10/2026)</t>
+          <t>Expire dans 22j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>23j</t>
+          <t>22j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>21/09/2026 13:45</t>
+          <t>22/09/2026 12:28</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 38j (29/10/2026)</t>
+          <t>Valide 37j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>38j</t>
+          <t>37j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 77j (07/12/2026)</t>
+          <t>Valide 76j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>21/09/2026 13:45</t>
+          <t>22/09/2026 12:28</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 38j (29/10/2026)</t>
+          <t>Valide 37j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>38j</t>
+          <t>37j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 77j (07/12/2026)</t>
+          <t>Valide 76j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>21/09/2026 13:45</t>
+          <t>22/09/2026 12:28</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 18j (09/10/2026)</t>
+          <t>Expire dans 17j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>18j</t>
+          <t>17j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 70j (30/11/2026)</t>
+          <t>Valide 69j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>21/09/2026 13:45</t>
+          <t>22/09/2026 12:28</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 18j (09/10/2026)</t>
+          <t>Expire dans 17j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>18j</t>
+          <t>17j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 70j (30/11/2026)</t>
+          <t>Valide 69j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>21/09/2026 13:45</t>
+          <t>22/09/2026 12:28</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 141j (09/02/2027)</t>
+          <t>Valide 140j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>141j</t>
+          <t>140j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 60j (20/11/2026)</t>
+          <t>Valide 59j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>21/09/2026 13:45</t>
+          <t>22/09/2026 12:28</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 141j (09/02/2027)</t>
+          <t>Valide 140j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>141j</t>
+          <t>140j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 60j (20/11/2026)</t>
+          <t>Valide 59j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>21/09/2026 13:45</t>
+          <t>22/09/2026 12:28</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 89j (19/12/2026)</t>
+          <t>Valide 88j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>89j</t>
+          <t>88j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 312j (31/07/2027)</t>
+          <t>Valide 311j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>21/09/2026 13:45</t>
+          <t>22/09/2026 12:28</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 89j (19/12/2026)</t>
+          <t>Valide 88j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>89j</t>
+          <t>88j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 312j (31/07/2027)</t>
+          <t>Valide 311j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>21/09/2026 13:45</t>
+          <t>22/09/2026 12:28</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,12 +2725,12 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 22j (13/10/2026)</t>
+          <t>Expire dans 21j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>22j</t>
+          <t>21j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
@@ -2740,7 +2740,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>21/09/2026 13:45</t>
+          <t>22/09/2026 12:28</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 23/09/2026 12:46
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 72j (04/12/2026)</t>
+          <t>Valide 71j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>72j</t>
+          <t>71j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 163j (05/03/2027)</t>
+          <t>Valide 162j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>22/09/2026 12:28</t>
+          <t>23/09/2026 12:38</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 138j (07/02/2027)</t>
+          <t>Valide 137j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>138j</t>
+          <t>137j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 318j (07/08/2027)</t>
+          <t>Valide 317j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>22/09/2026 12:28</t>
+          <t>23/09/2026 12:38</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 40j (02/11/2026)</t>
+          <t>Valide 39j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>40j</t>
+          <t>39j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 125j (26/01/2027)</t>
+          <t>Valide 124j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>22/09/2026 12:28</t>
+          <t>23/09/2026 12:38</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 59j (20/11/2026)</t>
+          <t>Valide 58j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>59j</t>
+          <t>58j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 40j (02/11/2026)</t>
+          <t>Valide 39j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>22/09/2026 12:28</t>
+          <t>23/09/2026 12:38</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 140j (09/02/2027)</t>
+          <t>Valide 139j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>140j</t>
+          <t>139j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 158j (28/02/2027)</t>
+          <t>Valide 157j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>22/09/2026 12:28</t>
+          <t>23/09/2026 12:38</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 138j (07/02/2027)</t>
+          <t>Valide 137j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>138j</t>
+          <t>137j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 302j (22/07/2027)</t>
+          <t>Valide 301j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>22/09/2026 12:28</t>
+          <t>23/09/2026 12:38</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 22j (14/10/2026)</t>
+          <t>Expire dans 21j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>22j</t>
+          <t>21j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>22/09/2026 12:28</t>
+          <t>23/09/2026 12:38</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 37j (29/10/2026)</t>
+          <t>Valide 36j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>37j</t>
+          <t>36j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 76j (07/12/2026)</t>
+          <t>Valide 75j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>22/09/2026 12:28</t>
+          <t>23/09/2026 12:38</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 37j (29/10/2026)</t>
+          <t>Valide 36j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>37j</t>
+          <t>36j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 76j (07/12/2026)</t>
+          <t>Valide 75j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>22/09/2026 12:28</t>
+          <t>23/09/2026 12:38</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 17j (09/10/2026)</t>
+          <t>Expire dans 16j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>17j</t>
+          <t>16j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 69j (30/11/2026)</t>
+          <t>Valide 68j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>22/09/2026 12:28</t>
+          <t>23/09/2026 12:38</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 17j (09/10/2026)</t>
+          <t>Expire dans 16j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>17j</t>
+          <t>16j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 69j (30/11/2026)</t>
+          <t>Valide 68j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>22/09/2026 12:28</t>
+          <t>23/09/2026 12:38</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 140j (09/02/2027)</t>
+          <t>Valide 139j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>140j</t>
+          <t>139j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 59j (20/11/2026)</t>
+          <t>Valide 58j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>22/09/2026 12:28</t>
+          <t>23/09/2026 12:38</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 140j (09/02/2027)</t>
+          <t>Valide 139j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>140j</t>
+          <t>139j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 59j (20/11/2026)</t>
+          <t>Valide 58j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>22/09/2026 12:28</t>
+          <t>23/09/2026 12:38</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 88j (19/12/2026)</t>
+          <t>Valide 87j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>88j</t>
+          <t>87j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 311j (31/07/2027)</t>
+          <t>Valide 310j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>22/09/2026 12:28</t>
+          <t>23/09/2026 12:38</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 88j (19/12/2026)</t>
+          <t>Valide 87j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>88j</t>
+          <t>87j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 311j (31/07/2027)</t>
+          <t>Valide 310j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>22/09/2026 12:28</t>
+          <t>23/09/2026 12:38</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 21j (13/10/2026)</t>
+          <t>Expire dans 20j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>21j</t>
+          <t>20j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 383j (10/10/2027)</t>
+          <t>Valide 382j (10/10/2027)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>22/09/2026 12:28</t>
+          <t>23/09/2026 12:38</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 24/09/2026 12:44
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 71j (04/12/2026)</t>
+          <t>Valide 70j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>71j</t>
+          <t>70j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 162j (05/03/2027)</t>
+          <t>Valide 161j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>23/09/2026 12:38</t>
+          <t>24/09/2026 12:37</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 137j (07/02/2027)</t>
+          <t>Valide 136j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>137j</t>
+          <t>136j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 317j (07/08/2027)</t>
+          <t>Valide 316j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>23/09/2026 12:38</t>
+          <t>24/09/2026 12:37</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 39j (02/11/2026)</t>
+          <t>Valide 38j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>39j</t>
+          <t>38j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 124j (26/01/2027)</t>
+          <t>Valide 123j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>23/09/2026 12:38</t>
+          <t>24/09/2026 12:37</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 58j (20/11/2026)</t>
+          <t>Valide 57j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>58j</t>
+          <t>57j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 39j (02/11/2026)</t>
+          <t>Valide 38j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>23/09/2026 12:38</t>
+          <t>24/09/2026 12:37</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 139j (09/02/2027)</t>
+          <t>Valide 138j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>139j</t>
+          <t>138j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 157j (28/02/2027)</t>
+          <t>Valide 156j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>23/09/2026 12:38</t>
+          <t>24/09/2026 12:37</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 137j (07/02/2027)</t>
+          <t>Valide 136j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>137j</t>
+          <t>136j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 301j (22/07/2027)</t>
+          <t>Valide 300j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>23/09/2026 12:38</t>
+          <t>24/09/2026 12:37</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 21j (14/10/2026)</t>
+          <t>Expire dans 20j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>21j</t>
+          <t>20j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>23/09/2026 12:38</t>
+          <t>24/09/2026 12:37</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 36j (29/10/2026)</t>
+          <t>Valide 35j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>36j</t>
+          <t>35j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 75j (07/12/2026)</t>
+          <t>Valide 74j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>23/09/2026 12:38</t>
+          <t>24/09/2026 12:37</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 36j (29/10/2026)</t>
+          <t>Valide 35j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>36j</t>
+          <t>35j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 75j (07/12/2026)</t>
+          <t>Valide 74j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>23/09/2026 12:38</t>
+          <t>24/09/2026 12:37</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,25 +1957,29 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 16j (09/10/2026)</t>
+          <t>Expire dans 15j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>16j</t>
+          <t>15j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 68j (30/11/2026)</t>
+          <t>Valide 67j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>23/09/2026 12:38</t>
-        </is>
-      </c>
-      <c r="P29" t="inlineStr"/>
+          <t>24/09/2026 12:37</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1" s="34">
       <c r="A30" s="3" t="inlineStr">
@@ -2007,25 +2011,29 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 16j (09/10/2026)</t>
+          <t>Expire dans 15j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>16j</t>
+          <t>15j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 68j (30/11/2026)</t>
+          <t>Valide 67j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>23/09/2026 12:38</t>
-        </is>
-      </c>
-      <c r="P30" t="inlineStr"/>
+          <t>24/09/2026 12:37</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="31" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A31" s="8" t="inlineStr">
@@ -2185,22 +2193,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 139j (09/02/2027)</t>
+          <t>Valide 138j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>139j</t>
+          <t>138j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 58j (20/11/2026)</t>
+          <t>Valide 57j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>23/09/2026 12:38</t>
+          <t>24/09/2026 12:37</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2255,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 139j (09/02/2027)</t>
+          <t>Valide 138j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>139j</t>
+          <t>138j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 58j (20/11/2026)</t>
+          <t>Valide 57j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>23/09/2026 12:38</t>
+          <t>24/09/2026 12:37</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2465,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 87j (19/12/2026)</t>
+          <t>Valide 86j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>87j</t>
+          <t>86j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 310j (31/07/2027)</t>
+          <t>Valide 309j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>23/09/2026 12:38</t>
+          <t>24/09/2026 12:37</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2519,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 87j (19/12/2026)</t>
+          <t>Valide 86j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>87j</t>
+          <t>86j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 310j (31/07/2027)</t>
+          <t>Valide 309j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>23/09/2026 12:38</t>
+          <t>24/09/2026 12:37</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2733,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 20j (13/10/2026)</t>
+          <t>Expire dans 19j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>20j</t>
+          <t>19j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 382j (10/10/2027)</t>
+          <t>Valide 381j (10/10/2027)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>23/09/2026 12:38</t>
+          <t>24/09/2026 12:37</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 25/09/2026 12:46
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 70j (04/12/2026)</t>
+          <t>Valide 69j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>70j</t>
+          <t>69j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 161j (05/03/2027)</t>
+          <t>Valide 160j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>24/09/2026 12:37</t>
+          <t>25/09/2026 12:38</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 136j (07/02/2027)</t>
+          <t>Valide 135j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>136j</t>
+          <t>135j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 316j (07/08/2027)</t>
+          <t>Valide 315j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>24/09/2026 12:37</t>
+          <t>25/09/2026 12:38</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 38j (02/11/2026)</t>
+          <t>Valide 37j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>38j</t>
+          <t>37j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 123j (26/01/2027)</t>
+          <t>Valide 122j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>24/09/2026 12:37</t>
+          <t>25/09/2026 12:38</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 57j (20/11/2026)</t>
+          <t>Valide 56j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>57j</t>
+          <t>56j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 38j (02/11/2026)</t>
+          <t>Valide 37j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>24/09/2026 12:37</t>
+          <t>25/09/2026 12:38</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 138j (09/02/2027)</t>
+          <t>Valide 137j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>138j</t>
+          <t>137j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 156j (28/02/2027)</t>
+          <t>Valide 155j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>24/09/2026 12:37</t>
+          <t>25/09/2026 12:38</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 136j (07/02/2027)</t>
+          <t>Valide 135j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>136j</t>
+          <t>135j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 300j (22/07/2027)</t>
+          <t>Valide 299j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>24/09/2026 12:37</t>
+          <t>25/09/2026 12:38</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 20j (14/10/2026)</t>
+          <t>Expire dans 19j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>20j</t>
+          <t>19j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>24/09/2026 12:37</t>
+          <t>25/09/2026 12:38</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 35j (29/10/2026)</t>
+          <t>Valide 34j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>35j</t>
+          <t>34j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 74j (07/12/2026)</t>
+          <t>Valide 73j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>24/09/2026 12:37</t>
+          <t>25/09/2026 12:38</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 35j (29/10/2026)</t>
+          <t>Valide 34j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>35j</t>
+          <t>34j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 74j (07/12/2026)</t>
+          <t>Valide 73j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>24/09/2026 12:37</t>
+          <t>25/09/2026 12:38</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,29 +1957,25 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 15j (09/10/2026)</t>
+          <t>Expire dans 14j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>15j</t>
+          <t>14j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 67j (30/11/2026)</t>
+          <t>Valide 66j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>24/09/2026 12:37</t>
-        </is>
-      </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>25/09/2026 12:38</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr"/>
     </row>
     <row r="30" ht="18" customHeight="1" s="34">
       <c r="A30" s="3" t="inlineStr">
@@ -2011,29 +2007,25 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 15j (09/10/2026)</t>
+          <t>Expire dans 14j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>15j</t>
+          <t>14j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 67j (30/11/2026)</t>
+          <t>Valide 66j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>24/09/2026 12:37</t>
-        </is>
-      </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>25/09/2026 12:38</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr"/>
     </row>
     <row r="31" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A31" s="8" t="inlineStr">
@@ -2193,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 138j (09/02/2027)</t>
+          <t>Valide 137j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>138j</t>
+          <t>137j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 57j (20/11/2026)</t>
+          <t>Valide 56j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>24/09/2026 12:37</t>
+          <t>25/09/2026 12:38</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2255,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 138j (09/02/2027)</t>
+          <t>Valide 137j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>138j</t>
+          <t>137j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 57j (20/11/2026)</t>
+          <t>Valide 56j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>24/09/2026 12:37</t>
+          <t>25/09/2026 12:38</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2465,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 86j (19/12/2026)</t>
+          <t>Valide 85j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>86j</t>
+          <t>85j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 309j (31/07/2027)</t>
+          <t>Valide 308j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>24/09/2026 12:37</t>
+          <t>25/09/2026 12:38</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2519,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 86j (19/12/2026)</t>
+          <t>Valide 85j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>86j</t>
+          <t>85j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 309j (31/07/2027)</t>
+          <t>Valide 308j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>24/09/2026 12:37</t>
+          <t>25/09/2026 12:38</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2733,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 19j (13/10/2026)</t>
+          <t>Expire dans 18j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>19j</t>
+          <t>18j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 381j (10/10/2027)</t>
+          <t>Valide 380j (10/10/2027)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>24/09/2026 12:37</t>
+          <t>25/09/2026 12:38</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 26/09/2026 12:12
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 69j (04/12/2026)</t>
+          <t>Valide 68j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>69j</t>
+          <t>68j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 160j (05/03/2027)</t>
+          <t>Valide 159j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>25/09/2026 12:38</t>
+          <t>26/09/2026 12:07</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 135j (07/02/2027)</t>
+          <t>Valide 134j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>135j</t>
+          <t>134j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 315j (07/08/2027)</t>
+          <t>Valide 314j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>25/09/2026 12:38</t>
+          <t>26/09/2026 12:07</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 37j (02/11/2026)</t>
+          <t>Valide 36j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>37j</t>
+          <t>36j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 122j (26/01/2027)</t>
+          <t>Valide 121j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>25/09/2026 12:38</t>
+          <t>26/09/2026 12:07</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,12 +1152,12 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 56j (20/11/2026)</t>
+          <t>Valide 55j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>56j</t>
+          <t>55j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>25/09/2026 12:38</t>
+          <t>26/09/2026 12:07</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 137j (09/02/2027)</t>
+          <t>Valide 136j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>137j</t>
+          <t>136j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 155j (28/02/2027)</t>
+          <t>Valide 154j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>25/09/2026 12:38</t>
+          <t>26/09/2026 12:07</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 135j (07/02/2027)</t>
+          <t>Valide 134j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>135j</t>
+          <t>134j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 299j (22/07/2027)</t>
+          <t>Valide 298j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>25/09/2026 12:38</t>
+          <t>26/09/2026 12:07</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 19j (14/10/2026)</t>
+          <t>Expire dans 18j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>19j</t>
+          <t>18j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>25/09/2026 12:38</t>
+          <t>26/09/2026 12:07</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 34j (29/10/2026)</t>
+          <t>Valide 33j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>34j</t>
+          <t>33j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 73j (07/12/2026)</t>
+          <t>Valide 72j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>25/09/2026 12:38</t>
+          <t>26/09/2026 12:07</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 34j (29/10/2026)</t>
+          <t>Valide 33j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>34j</t>
+          <t>33j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 73j (07/12/2026)</t>
+          <t>Valide 72j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>25/09/2026 12:38</t>
+          <t>26/09/2026 12:07</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 14j (09/10/2026)</t>
+          <t>Expire dans 13j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>14j</t>
+          <t>13j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 66j (30/11/2026)</t>
+          <t>Valide 65j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>25/09/2026 12:38</t>
+          <t>26/09/2026 12:07</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 14j (09/10/2026)</t>
+          <t>Expire dans 13j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>14j</t>
+          <t>13j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 66j (30/11/2026)</t>
+          <t>Valide 65j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>25/09/2026 12:38</t>
+          <t>26/09/2026 12:07</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 137j (09/02/2027)</t>
+          <t>Valide 136j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>137j</t>
+          <t>136j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 56j (20/11/2026)</t>
+          <t>Valide 55j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>25/09/2026 12:38</t>
+          <t>26/09/2026 12:07</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 137j (09/02/2027)</t>
+          <t>Valide 136j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>137j</t>
+          <t>136j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 56j (20/11/2026)</t>
+          <t>Valide 55j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>25/09/2026 12:38</t>
+          <t>26/09/2026 12:07</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 85j (19/12/2026)</t>
+          <t>Valide 84j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>85j</t>
+          <t>84j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 308j (31/07/2027)</t>
+          <t>Valide 307j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>25/09/2026 12:38</t>
+          <t>26/09/2026 12:07</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 85j (19/12/2026)</t>
+          <t>Valide 84j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>85j</t>
+          <t>84j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 308j (31/07/2027)</t>
+          <t>Valide 307j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>25/09/2026 12:38</t>
+          <t>26/09/2026 12:07</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 18j (13/10/2026)</t>
+          <t>Expire dans 17j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>18j</t>
+          <t>17j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 380j (10/10/2027)</t>
+          <t>Valide 379j (10/10/2027)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>25/09/2026 12:38</t>
+          <t>26/09/2026 12:07</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 27/09/2026 12:58
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 68j (04/12/2026)</t>
+          <t>Valide 67j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>68j</t>
+          <t>67j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 159j (05/03/2027)</t>
+          <t>Valide 158j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>26/09/2026 12:07</t>
+          <t>27/09/2026 12:52</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 134j (07/02/2027)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>134j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 314j (07/08/2027)</t>
+          <t>Valide 313j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>26/09/2026 12:07</t>
+          <t>27/09/2026 12:52</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 36j (02/11/2026)</t>
+          <t>Valide 35j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>36j</t>
+          <t>35j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 121j (26/01/2027)</t>
+          <t>Valide 120j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>26/09/2026 12:07</t>
+          <t>27/09/2026 12:52</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 55j (20/11/2026)</t>
+          <t>Valide 54j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>55j</t>
+          <t>54j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 37j (02/11/2026)</t>
+          <t>Valide 35j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>26/09/2026 12:07</t>
+          <t>27/09/2026 12:52</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 136j (09/02/2027)</t>
+          <t>Valide 135j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>136j</t>
+          <t>135j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 154j (28/02/2027)</t>
+          <t>Valide 153j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>26/09/2026 12:07</t>
+          <t>27/09/2026 12:52</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 134j (07/02/2027)</t>
+          <t>Valide 133j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>134j</t>
+          <t>133j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 298j (22/07/2027)</t>
+          <t>Valide 297j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>26/09/2026 12:07</t>
+          <t>27/09/2026 12:52</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 18j (14/10/2026)</t>
+          <t>Expire dans 17j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>18j</t>
+          <t>17j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>26/09/2026 12:07</t>
+          <t>27/09/2026 12:52</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 33j (29/10/2026)</t>
+          <t>Valide 32j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>33j</t>
+          <t>32j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 72j (07/12/2026)</t>
+          <t>Valide 71j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>26/09/2026 12:07</t>
+          <t>27/09/2026 12:52</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 33j (29/10/2026)</t>
+          <t>Valide 32j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>33j</t>
+          <t>32j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 72j (07/12/2026)</t>
+          <t>Valide 71j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>26/09/2026 12:07</t>
+          <t>27/09/2026 12:52</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 13j (09/10/2026)</t>
+          <t>Expire dans 12j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>13j</t>
+          <t>12j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 65j (30/11/2026)</t>
+          <t>Valide 64j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>26/09/2026 12:07</t>
+          <t>27/09/2026 12:52</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 13j (09/10/2026)</t>
+          <t>Expire dans 12j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>13j</t>
+          <t>12j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 65j (30/11/2026)</t>
+          <t>Valide 64j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>26/09/2026 12:07</t>
+          <t>27/09/2026 12:52</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 136j (09/02/2027)</t>
+          <t>Valide 135j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>136j</t>
+          <t>135j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 55j (20/11/2026)</t>
+          <t>Valide 54j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>26/09/2026 12:07</t>
+          <t>27/09/2026 12:52</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 136j (09/02/2027)</t>
+          <t>Valide 135j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>136j</t>
+          <t>135j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 55j (20/11/2026)</t>
+          <t>Valide 54j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>26/09/2026 12:07</t>
+          <t>27/09/2026 12:52</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 84j (19/12/2026)</t>
+          <t>Valide 83j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>84j</t>
+          <t>83j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 307j (31/07/2027)</t>
+          <t>Valide 306j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>26/09/2026 12:07</t>
+          <t>27/09/2026 12:52</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 84j (19/12/2026)</t>
+          <t>Valide 83j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>84j</t>
+          <t>83j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 307j (31/07/2027)</t>
+          <t>Valide 306j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>26/09/2026 12:07</t>
+          <t>27/09/2026 12:52</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 17j (13/10/2026)</t>
+          <t>Expire dans 16j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>17j</t>
+          <t>16j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 379j (10/10/2027)</t>
+          <t>Valide 378j (10/10/2027)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>26/09/2026 12:07</t>
+          <t>27/09/2026 12:52</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 28/09/2026 15:17
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 67j (04/12/2026)</t>
+          <t>Valide 66j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>67j</t>
+          <t>66j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 158j (05/03/2027)</t>
+          <t>Valide 157j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>27/09/2026 12:52</t>
+          <t>28/09/2026 15:07</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 313j (07/08/2027)</t>
+          <t>Valide 312j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>27/09/2026 12:52</t>
+          <t>28/09/2026 15:07</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 35j (02/11/2026)</t>
+          <t>Valide 34j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>35j</t>
+          <t>34j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 120j (26/01/2027)</t>
+          <t>Valide 119j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>27/09/2026 12:52</t>
+          <t>28/09/2026 15:07</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 54j (20/11/2026)</t>
+          <t>Valide 53j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>54j</t>
+          <t>53j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 35j (02/11/2026)</t>
+          <t>Valide 34j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>27/09/2026 12:52</t>
+          <t>28/09/2026 15:07</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 135j (09/02/2027)</t>
+          <t>Valide 134j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>135j</t>
+          <t>134j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 153j (28/02/2027)</t>
+          <t>Valide 152j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>27/09/2026 12:52</t>
+          <t>28/09/2026 15:07</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 133j (07/02/2027)</t>
+          <t>Valide 131j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>133j</t>
+          <t>131j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 297j (22/07/2027)</t>
+          <t>Valide 296j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>27/09/2026 12:52</t>
+          <t>28/09/2026 15:07</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 17j (14/10/2026)</t>
+          <t>Expire dans 16j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>17j</t>
+          <t>16j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>27/09/2026 12:52</t>
+          <t>28/09/2026 15:07</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 32j (29/10/2026)</t>
+          <t>Valide 31j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>32j</t>
+          <t>31j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 71j (07/12/2026)</t>
+          <t>Valide 70j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>27/09/2026 12:52</t>
+          <t>28/09/2026 15:07</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 32j (29/10/2026)</t>
+          <t>Valide 31j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>32j</t>
+          <t>31j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 71j (07/12/2026)</t>
+          <t>Valide 70j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>27/09/2026 12:52</t>
+          <t>28/09/2026 15:07</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 12j (09/10/2026)</t>
+          <t>Expire dans 11j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>12j</t>
+          <t>11j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 64j (30/11/2026)</t>
+          <t>Valide 63j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>27/09/2026 12:52</t>
+          <t>28/09/2026 15:07</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 12j (09/10/2026)</t>
+          <t>Expire dans 11j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>12j</t>
+          <t>11j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 64j (30/11/2026)</t>
+          <t>Valide 63j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>27/09/2026 12:52</t>
+          <t>28/09/2026 15:07</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 135j (09/02/2027)</t>
+          <t>Valide 134j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>135j</t>
+          <t>134j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 54j (20/11/2026)</t>
+          <t>Valide 52j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>27/09/2026 12:52</t>
+          <t>28/09/2026 15:07</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 135j (09/02/2027)</t>
+          <t>Valide 134j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>135j</t>
+          <t>134j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 54j (20/11/2026)</t>
+          <t>Valide 52j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>27/09/2026 12:52</t>
+          <t>28/09/2026 15:07</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 83j (19/12/2026)</t>
+          <t>Valide 82j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>83j</t>
+          <t>82j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 306j (31/07/2027)</t>
+          <t>Valide 305j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>27/09/2026 12:52</t>
+          <t>28/09/2026 15:07</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 83j (19/12/2026)</t>
+          <t>Valide 82j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>83j</t>
+          <t>82j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 306j (31/07/2027)</t>
+          <t>Valide 305j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>27/09/2026 12:52</t>
+          <t>28/09/2026 15:07</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,25 +2725,29 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 16j (13/10/2026)</t>
+          <t>Expire dans 15j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>16j</t>
+          <t>15j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 378j (10/10/2027)</t>
+          <t>Valide 376j (10/10/2027)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>27/09/2026 12:52</t>
-        </is>
-      </c>
-      <c r="P49" t="inlineStr"/>
+          <t>28/09/2026 15:07</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1" s="34">
       <c r="A50" s="3" t="inlineStr">

</xml_diff>

<commit_message>
chore: monitoring 29/09/2026 13:57
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 66j (04/12/2026)</t>
+          <t>Valide 65j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>66j</t>
+          <t>65j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 157j (05/03/2027)</t>
+          <t>Valide 156j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>28/09/2026 15:07</t>
+          <t>29/09/2026 13:52</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 312j (07/08/2027)</t>
+          <t>Valide 311j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>28/09/2026 15:07</t>
+          <t>29/09/2026 13:52</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 34j (02/11/2026)</t>
+          <t>Valide 33j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>34j</t>
+          <t>33j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 119j (26/01/2027)</t>
+          <t>Valide 118j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>28/09/2026 15:07</t>
+          <t>29/09/2026 13:52</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 53j (20/11/2026)</t>
+          <t>Valide 52j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>53j</t>
+          <t>52j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 34j (02/11/2026)</t>
+          <t>Valide 33j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>28/09/2026 15:07</t>
+          <t>29/09/2026 13:52</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 134j (09/02/2027)</t>
+          <t>Valide 133j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>134j</t>
+          <t>133j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 152j (28/02/2027)</t>
+          <t>Valide 151j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>28/09/2026 15:07</t>
+          <t>29/09/2026 13:52</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1590,12 +1590,12 @@
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 296j (22/07/2027)</t>
+          <t>Valide 295j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>28/09/2026 15:07</t>
+          <t>29/09/2026 13:52</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 16j (14/10/2026)</t>
+          <t>Expire dans 15j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>16j</t>
+          <t>15j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,10 +1665,14 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>28/09/2026 15:07</t>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr"/>
+          <t>29/09/2026 13:52</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
       <c r="R23" t="inlineStr">
         <is>
           <t>x</t>
@@ -1745,25 +1749,29 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 31j (29/10/2026)</t>
+          <t>Expire dans 30j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>31j</t>
+          <t>30j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 70j (07/12/2026)</t>
+          <t>Valide 69j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>28/09/2026 15:07</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr"/>
+          <t>29/09/2026 13:52</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1" s="34">
       <c r="A26" s="3" t="inlineStr">
@@ -1811,25 +1819,29 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 31j (29/10/2026)</t>
+          <t>Expire dans 30j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>31j</t>
+          <t>30j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 70j (07/12/2026)</t>
+          <t>Valide 69j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>28/09/2026 15:07</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr"/>
+          <t>29/09/2026 13:52</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="27" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A27" s="8" t="inlineStr">
@@ -1957,22 +1969,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 11j (09/10/2026)</t>
+          <t>Expire dans 10j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>11j</t>
+          <t>10j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 63j (30/11/2026)</t>
+          <t>Valide 62j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>28/09/2026 15:07</t>
+          <t>29/09/2026 13:52</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2019,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 11j (09/10/2026)</t>
+          <t>Expire dans 10j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>11j</t>
+          <t>10j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 63j (30/11/2026)</t>
+          <t>Valide 62j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>28/09/2026 15:07</t>
+          <t>29/09/2026 13:52</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,12 +2197,12 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 134j (09/02/2027)</t>
+          <t>Valide 133j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>134j</t>
+          <t>133j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
@@ -2200,7 +2212,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>28/09/2026 15:07</t>
+          <t>29/09/2026 13:52</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,12 +2259,12 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 134j (09/02/2027)</t>
+          <t>Valide 133j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>134j</t>
+          <t>133j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
@@ -2262,7 +2274,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>28/09/2026 15:07</t>
+          <t>29/09/2026 13:52</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2469,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 82j (19/12/2026)</t>
+          <t>Valide 81j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>82j</t>
+          <t>81j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 305j (31/07/2027)</t>
+          <t>Valide 304j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>28/09/2026 15:07</t>
+          <t>29/09/2026 13:52</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2523,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 82j (19/12/2026)</t>
+          <t>Valide 81j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>82j</t>
+          <t>81j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 305j (31/07/2027)</t>
+          <t>Valide 304j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>28/09/2026 15:07</t>
+          <t>29/09/2026 13:52</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,29 +2737,25 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 15j (13/10/2026)</t>
+          <t>Expire dans 14j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>15j</t>
+          <t>14j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 376j (10/10/2027)</t>
+          <t>Valide 375j (10/10/2027)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>28/09/2026 15:07</t>
-        </is>
-      </c>
-      <c r="P49" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>29/09/2026 13:52</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr"/>
     </row>
     <row r="50" ht="18" customHeight="1" s="34">
       <c r="A50" s="3" t="inlineStr">

</xml_diff>

<commit_message>
chore: monitoring 30/09/2026 13:32
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 65j (04/12/2026)</t>
+          <t>Valide 64j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>65j</t>
+          <t>64j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 156j (05/03/2027)</t>
+          <t>Valide 155j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>29/09/2026 13:52</t>
+          <t>30/09/2026 13:26</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 311j (07/08/2027)</t>
+          <t>Valide 310j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>29/09/2026 13:52</t>
+          <t>30/09/2026 13:26</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 33j (02/11/2026)</t>
+          <t>Valide 32j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>33j</t>
+          <t>32j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 118j (26/01/2027)</t>
+          <t>Valide 117j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>29/09/2026 13:52</t>
+          <t>30/09/2026 13:26</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 52j (20/11/2026)</t>
+          <t>Valide 51j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>52j</t>
+          <t>51j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 33j (02/11/2026)</t>
+          <t>Valide 32j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>29/09/2026 13:52</t>
+          <t>30/09/2026 13:26</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 133j (09/02/2027)</t>
+          <t>Valide 132j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>133j</t>
+          <t>132j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 151j (28/02/2027)</t>
+          <t>Valide 150j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>29/09/2026 13:52</t>
+          <t>30/09/2026 13:26</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 131j (07/02/2027)</t>
+          <t>Valide 130j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>131j</t>
+          <t>130j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 295j (22/07/2027)</t>
+          <t>Valide 294j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>29/09/2026 13:52</t>
+          <t>30/09/2026 13:26</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 15j (14/10/2026)</t>
+          <t>Expire dans 14j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>15j</t>
+          <t>14j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,14 +1665,10 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>29/09/2026 13:52</t>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>30/09/2026 13:26</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
           <t>x</t>
@@ -1749,29 +1745,25 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 30j (29/10/2026)</t>
+          <t>Expire dans 29j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>30j</t>
+          <t>29j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 69j (07/12/2026)</t>
+          <t>Valide 68j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>29/09/2026 13:52</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>30/09/2026 13:26</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr"/>
     </row>
     <row r="26" ht="18" customHeight="1" s="34">
       <c r="A26" s="3" t="inlineStr">
@@ -1819,29 +1811,25 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 30j (29/10/2026)</t>
+          <t>Expire dans 29j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>30j</t>
+          <t>29j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 69j (07/12/2026)</t>
+          <t>Valide 68j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>29/09/2026 13:52</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>30/09/2026 13:26</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A27" s="8" t="inlineStr">
@@ -1969,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 10j (09/10/2026)</t>
+          <t>Expire dans 9j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>10j</t>
+          <t>9j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 62j (30/11/2026)</t>
+          <t>Valide 61j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>29/09/2026 13:52</t>
+          <t>30/09/2026 13:26</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2019,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 10j (09/10/2026)</t>
+          <t>Expire dans 9j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>10j</t>
+          <t>9j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 62j (30/11/2026)</t>
+          <t>Valide 61j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>29/09/2026 13:52</t>
+          <t>30/09/2026 13:26</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2197,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 133j (09/02/2027)</t>
+          <t>Valide 132j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>133j</t>
+          <t>132j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 52j (20/11/2026)</t>
+          <t>Valide 51j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>29/09/2026 13:52</t>
+          <t>30/09/2026 13:26</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2259,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 133j (09/02/2027)</t>
+          <t>Valide 132j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>133j</t>
+          <t>132j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 52j (20/11/2026)</t>
+          <t>Valide 51j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>29/09/2026 13:52</t>
+          <t>30/09/2026 13:26</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2469,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 81j (19/12/2026)</t>
+          <t>Valide 80j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>81j</t>
+          <t>80j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 304j (31/07/2027)</t>
+          <t>Valide 303j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>29/09/2026 13:52</t>
+          <t>30/09/2026 13:26</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2523,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 81j (19/12/2026)</t>
+          <t>Valide 80j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>81j</t>
+          <t>80j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 304j (31/07/2027)</t>
+          <t>Valide 303j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>29/09/2026 13:52</t>
+          <t>30/09/2026 13:26</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2737,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 14j (13/10/2026)</t>
+          <t>Expire dans 13j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>14j</t>
+          <t>13j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 375j (10/10/2027)</t>
+          <t>Valide 374j (10/10/2027)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>29/09/2026 13:52</t>
+          <t>30/09/2026 13:26</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 01/10/2026 14:24
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 64j (04/12/2026)</t>
+          <t>Valide 63j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>64j</t>
+          <t>63j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 155j (05/03/2027)</t>
+          <t>Valide 154j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>30/09/2026 13:26</t>
+          <t>01/10/2026 14:19</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 310j (07/08/2027)</t>
+          <t>Valide 309j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>30/09/2026 13:26</t>
+          <t>01/10/2026 14:19</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 32j (02/11/2026)</t>
+          <t>Valide 31j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>32j</t>
+          <t>31j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 117j (26/01/2027)</t>
+          <t>Valide 116j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>30/09/2026 13:26</t>
+          <t>01/10/2026 14:19</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 51j (20/11/2026)</t>
+          <t>Valide 50j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>51j</t>
+          <t>50j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 32j (02/11/2026)</t>
+          <t>Valide 31j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>30/09/2026 13:26</t>
+          <t>01/10/2026 14:19</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 132j (09/02/2027)</t>
+          <t>Valide 131j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>132j</t>
+          <t>131j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 150j (28/02/2027)</t>
+          <t>Valide 149j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>30/09/2026 13:26</t>
+          <t>01/10/2026 14:19</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 130j (07/02/2027)</t>
+          <t>Valide 129j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>130j</t>
+          <t>129j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 294j (22/07/2027)</t>
+          <t>Valide 293j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>30/09/2026 13:26</t>
+          <t>01/10/2026 14:19</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 14j (14/10/2026)</t>
+          <t>Expire dans 13j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>14j</t>
+          <t>13j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>30/09/2026 13:26</t>
+          <t>01/10/2026 14:19</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 29j (29/10/2026)</t>
+          <t>Valide 89j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>29j</t>
+          <t>89j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 68j (07/12/2026)</t>
+          <t>Valide 67j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>30/09/2026 13:26</t>
+          <t>01/10/2026 14:19</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 29j (29/10/2026)</t>
+          <t>Valide 89j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>29j</t>
+          <t>89j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 68j (07/12/2026)</t>
+          <t>Valide 67j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>30/09/2026 13:26</t>
+          <t>01/10/2026 14:19</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 9j (09/10/2026)</t>
+          <t>Expire dans 8j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>9j</t>
+          <t>8j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 61j (30/11/2026)</t>
+          <t>Valide 60j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>30/09/2026 13:26</t>
+          <t>01/10/2026 14:19</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 9j (09/10/2026)</t>
+          <t>Expire dans 8j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>9j</t>
+          <t>8j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 61j (30/11/2026)</t>
+          <t>Valide 60j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>30/09/2026 13:26</t>
+          <t>01/10/2026 14:19</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 132j (09/02/2027)</t>
+          <t>Valide 131j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>132j</t>
+          <t>131j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 51j (20/11/2026)</t>
+          <t>Valide 50j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>30/09/2026 13:26</t>
+          <t>01/10/2026 14:19</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 132j (09/02/2027)</t>
+          <t>Valide 131j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>132j</t>
+          <t>131j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 51j (20/11/2026)</t>
+          <t>Valide 50j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>30/09/2026 13:26</t>
+          <t>01/10/2026 14:19</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 80j (19/12/2026)</t>
+          <t>Valide 79j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>80j</t>
+          <t>79j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 303j (31/07/2027)</t>
+          <t>Valide 302j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>30/09/2026 13:26</t>
+          <t>01/10/2026 14:19</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 80j (19/12/2026)</t>
+          <t>Valide 79j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>80j</t>
+          <t>79j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 303j (31/07/2027)</t>
+          <t>Valide 302j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>30/09/2026 13:26</t>
+          <t>01/10/2026 14:19</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 13j (13/10/2026)</t>
+          <t>Expire dans 12j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>13j</t>
+          <t>12j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 374j (10/10/2027)</t>
+          <t>Valide 373j (10/10/2027)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>30/09/2026 13:26</t>
+          <t>01/10/2026 14:19</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 02/10/2026 13:46
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 63j (04/12/2026)</t>
+          <t>Valide 62j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>63j</t>
+          <t>62j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 154j (05/03/2027)</t>
+          <t>Valide 153j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>01/10/2026 14:19</t>
+          <t>02/10/2026 13:41</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 128j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>128j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 309j (07/08/2027)</t>
+          <t>Valide 308j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>01/10/2026 14:19</t>
+          <t>02/10/2026 13:41</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,25 +1046,29 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 31j (02/11/2026)</t>
+          <t>Expire dans 30j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>31j</t>
+          <t>30j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 116j (26/01/2027)</t>
+          <t>Valide 115j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>01/10/2026 14:19</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr"/>
+          <t>02/10/2026 13:41</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="9" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A9" s="3" t="inlineStr">
@@ -1152,25 +1156,29 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 50j (20/11/2026)</t>
+          <t>Valide 49j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>50j</t>
+          <t>49j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 31j (02/11/2026)</t>
+          <t>Expire dans 30j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>01/10/2026 14:19</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr"/>
+          <t>02/10/2026 13:41</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="11" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A11" s="3" t="inlineStr">
@@ -1258,22 +1266,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 131j (09/02/2027)</t>
+          <t>Valide 130j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>131j</t>
+          <t>130j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 149j (28/02/2027)</t>
+          <t>Valide 148j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>01/10/2026 14:19</t>
+          <t>02/10/2026 13:41</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1588,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 129j (07/02/2027)</t>
+          <t>Valide 128j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>129j</t>
+          <t>128j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 293j (22/07/2027)</t>
+          <t>Valide 292j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>01/10/2026 14:19</t>
+          <t>02/10/2026 13:41</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1658,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 13j (14/10/2026)</t>
+          <t>Expire dans 12j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>13j</t>
+          <t>12j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1673,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>01/10/2026 14:19</t>
+          <t>02/10/2026 13:41</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1753,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 89j (29/12/2026)</t>
+          <t>Valide 88j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>89j</t>
+          <t>88j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 67j (07/12/2026)</t>
+          <t>Valide 66j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>01/10/2026 14:19</t>
+          <t>02/10/2026 13:41</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1819,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 89j (29/12/2026)</t>
+          <t>Valide 88j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>89j</t>
+          <t>88j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 67j (07/12/2026)</t>
+          <t>Valide 66j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>01/10/2026 14:19</t>
+          <t>02/10/2026 13:41</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,25 +1965,29 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 8j (09/10/2026)</t>
+          <t>Expire dans 7j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>8j</t>
+          <t>7j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 60j (30/11/2026)</t>
+          <t>Valide 59j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>01/10/2026 14:19</t>
-        </is>
-      </c>
-      <c r="P29" t="inlineStr"/>
+          <t>02/10/2026 13:41</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1" s="34">
       <c r="A30" s="3" t="inlineStr">
@@ -2007,25 +2019,29 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 8j (09/10/2026)</t>
+          <t>Expire dans 7j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>8j</t>
+          <t>7j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 60j (30/11/2026)</t>
+          <t>Valide 59j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>01/10/2026 14:19</t>
-        </is>
-      </c>
-      <c r="P30" t="inlineStr"/>
+          <t>02/10/2026 13:41</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="31" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A31" s="8" t="inlineStr">
@@ -2185,22 +2201,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 131j (09/02/2027)</t>
+          <t>Valide 130j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>131j</t>
+          <t>130j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 50j (20/11/2026)</t>
+          <t>Valide 49j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>01/10/2026 14:19</t>
+          <t>02/10/2026 13:41</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2263,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 131j (09/02/2027)</t>
+          <t>Valide 130j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>131j</t>
+          <t>130j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 50j (20/11/2026)</t>
+          <t>Valide 49j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>01/10/2026 14:19</t>
+          <t>02/10/2026 13:41</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2473,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 79j (19/12/2026)</t>
+          <t>Valide 78j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>79j</t>
+          <t>78j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 302j (31/07/2027)</t>
+          <t>Valide 301j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>01/10/2026 14:19</t>
+          <t>02/10/2026 13:41</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2527,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 79j (19/12/2026)</t>
+          <t>Valide 78j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>79j</t>
+          <t>78j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 302j (31/07/2027)</t>
+          <t>Valide 301j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>01/10/2026 14:19</t>
+          <t>02/10/2026 13:41</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2741,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 12j (13/10/2026)</t>
+          <t>Expire dans 11j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>12j</t>
+          <t>11j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 373j (10/10/2027)</t>
+          <t>Valide 372j (10/10/2027)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>01/10/2026 14:19</t>
+          <t>02/10/2026 13:41</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 03/10/2026 12:25
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 62j (04/12/2026)</t>
+          <t>Valide 61j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>62j</t>
+          <t>61j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 153j (05/03/2027)</t>
+          <t>Valide 152j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>02/10/2026 13:41</t>
+          <t>03/10/2026 12:20</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 128j (07/02/2027)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>128j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 308j (07/08/2027)</t>
+          <t>Valide 307j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>02/10/2026 13:41</t>
+          <t>03/10/2026 12:20</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,29 +1046,25 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 30j (02/11/2026)</t>
+          <t>Expire dans 29j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>30j</t>
+          <t>29j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 115j (26/01/2027)</t>
+          <t>Valide 114j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>02/10/2026 13:41</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>03/10/2026 12:20</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A9" s="3" t="inlineStr">
@@ -1156,29 +1152,25 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 49j (20/11/2026)</t>
+          <t>Valide 48j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>49j</t>
+          <t>48j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 30j (02/11/2026)</t>
+          <t>Expire dans 29j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>02/10/2026 13:41</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>03/10/2026 12:20</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A11" s="3" t="inlineStr">
@@ -1266,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 130j (09/02/2027)</t>
+          <t>Valide 129j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>130j</t>
+          <t>129j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 148j (28/02/2027)</t>
+          <t>Valide 147j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>02/10/2026 13:41</t>
+          <t>03/10/2026 12:20</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1588,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 128j (07/02/2027)</t>
+          <t>Valide 127j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>128j</t>
+          <t>127j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 292j (22/07/2027)</t>
+          <t>Valide 291j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>02/10/2026 13:41</t>
+          <t>03/10/2026 12:20</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1658,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 12j (14/10/2026)</t>
+          <t>Expire dans 11j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>12j</t>
+          <t>11j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1673,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>02/10/2026 13:41</t>
+          <t>03/10/2026 12:20</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1753,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 88j (29/12/2026)</t>
+          <t>Valide 87j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>88j</t>
+          <t>87j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 66j (07/12/2026)</t>
+          <t>Valide 65j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>02/10/2026 13:41</t>
+          <t>03/10/2026 12:20</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1819,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 88j (29/12/2026)</t>
+          <t>Valide 87j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>88j</t>
+          <t>87j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 66j (07/12/2026)</t>
+          <t>Valide 65j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>02/10/2026 13:41</t>
+          <t>03/10/2026 12:20</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1965,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 7j (09/10/2026)</t>
+          <t>Expire dans 6j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>7j</t>
+          <t>6j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 59j (30/11/2026)</t>
+          <t>Valide 58j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>02/10/2026 13:41</t>
+          <t>03/10/2026 12:20</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -2019,22 +2011,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 7j (09/10/2026)</t>
+          <t>Expire dans 6j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>7j</t>
+          <t>6j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 59j (30/11/2026)</t>
+          <t>Valide 58j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>02/10/2026 13:41</t>
+          <t>03/10/2026 12:20</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -2201,22 +2193,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 130j (09/02/2027)</t>
+          <t>Valide 129j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>130j</t>
+          <t>129j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 49j (20/11/2026)</t>
+          <t>Valide 48j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>02/10/2026 13:41</t>
+          <t>03/10/2026 12:20</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2263,22 +2255,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 130j (09/02/2027)</t>
+          <t>Valide 129j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>130j</t>
+          <t>129j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 49j (20/11/2026)</t>
+          <t>Valide 48j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>02/10/2026 13:41</t>
+          <t>03/10/2026 12:20</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2473,22 +2465,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 78j (19/12/2026)</t>
+          <t>Valide 77j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>78j</t>
+          <t>77j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 301j (31/07/2027)</t>
+          <t>Valide 300j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>02/10/2026 13:41</t>
+          <t>03/10/2026 12:20</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2527,22 +2519,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 78j (19/12/2026)</t>
+          <t>Valide 77j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>78j</t>
+          <t>77j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 301j (31/07/2027)</t>
+          <t>Valide 300j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>02/10/2026 13:41</t>
+          <t>03/10/2026 12:20</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2741,12 +2733,12 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 11j (13/10/2026)</t>
+          <t>Expire dans 10j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>11j</t>
+          <t>10j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
@@ -2756,7 +2748,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>02/10/2026 13:41</t>
+          <t>03/10/2026 12:20</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 04/10/2026 13:11
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 61j (04/12/2026)</t>
+          <t>Valide 60j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>61j</t>
+          <t>60j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 152j (05/03/2027)</t>
+          <t>Valide 151j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>03/10/2026 12:20</t>
+          <t>04/10/2026 13:06</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 307j (07/08/2027)</t>
+          <t>Valide 306j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>03/10/2026 12:20</t>
+          <t>04/10/2026 13:06</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 29j (02/11/2026)</t>
+          <t>Valide 89j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>29j</t>
+          <t>89j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 114j (26/01/2027)</t>
+          <t>Valide 113j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>03/10/2026 12:20</t>
+          <t>04/10/2026 13:06</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 48j (20/11/2026)</t>
+          <t>Valide 47j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>48j</t>
+          <t>47j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 29j (02/11/2026)</t>
+          <t>Expire dans 28j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>03/10/2026 12:20</t>
+          <t>04/10/2026 13:06</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 129j (09/02/2027)</t>
+          <t>Valide 128j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>129j</t>
+          <t>128j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 147j (28/02/2027)</t>
+          <t>Valide 146j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>03/10/2026 12:20</t>
+          <t>04/10/2026 13:06</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 127j (07/02/2027)</t>
+          <t>Valide 126j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>127j</t>
+          <t>126j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 291j (22/07/2027)</t>
+          <t>Valide 290j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>03/10/2026 12:20</t>
+          <t>04/10/2026 13:06</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 11j (14/10/2026)</t>
+          <t>Expire dans 10j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>11j</t>
+          <t>10j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>03/10/2026 12:20</t>
+          <t>04/10/2026 13:06</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 87j (29/12/2026)</t>
+          <t>Valide 86j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>87j</t>
+          <t>86j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 65j (07/12/2026)</t>
+          <t>Valide 64j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>03/10/2026 12:20</t>
+          <t>04/10/2026 13:06</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 87j (29/12/2026)</t>
+          <t>Valide 86j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>87j</t>
+          <t>86j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 65j (07/12/2026)</t>
+          <t>Valide 64j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>03/10/2026 12:20</t>
+          <t>04/10/2026 13:06</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 6j (09/10/2026)</t>
+          <t>Expire dans 5j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>6j</t>
+          <t>5j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 58j (30/11/2026)</t>
+          <t>Valide 57j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>03/10/2026 12:20</t>
+          <t>04/10/2026 13:06</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -2011,22 +2011,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 6j (09/10/2026)</t>
+          <t>Expire dans 5j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>6j</t>
+          <t>5j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 58j (30/11/2026)</t>
+          <t>Valide 57j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>03/10/2026 12:20</t>
+          <t>04/10/2026 13:06</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -2193,22 +2193,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 129j (09/02/2027)</t>
+          <t>Valide 128j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>129j</t>
+          <t>128j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 48j (20/11/2026)</t>
+          <t>Valide 47j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>03/10/2026 12:20</t>
+          <t>04/10/2026 13:06</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2255,22 +2255,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 129j (09/02/2027)</t>
+          <t>Valide 128j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>129j</t>
+          <t>128j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 48j (20/11/2026)</t>
+          <t>Valide 47j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>03/10/2026 12:20</t>
+          <t>04/10/2026 13:06</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2465,22 +2465,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 77j (19/12/2026)</t>
+          <t>Valide 76j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>77j</t>
+          <t>76j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 300j (31/07/2027)</t>
+          <t>Valide 299j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>03/10/2026 12:20</t>
+          <t>04/10/2026 13:06</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2519,22 +2519,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 77j (19/12/2026)</t>
+          <t>Valide 76j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>77j</t>
+          <t>76j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 300j (31/07/2027)</t>
+          <t>Valide 299j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>03/10/2026 12:20</t>
+          <t>04/10/2026 13:06</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2733,22 +2733,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 10j (13/10/2026)</t>
+          <t>Expire dans 9j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>10j</t>
+          <t>9j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 372j (10/10/2027)</t>
+          <t>Valide 370j (10/10/2027)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>03/10/2026 12:20</t>
+          <t>04/10/2026 13:06</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 05/10/2026 15:47
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 60j (04/12/2026)</t>
+          <t>Valide 59j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>60j</t>
+          <t>59j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 151j (05/03/2027)</t>
+          <t>Valide 150j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>04/10/2026 13:06</t>
+          <t>05/10/2026 15:42</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 306j (07/08/2027)</t>
+          <t>Valide 305j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>04/10/2026 13:06</t>
+          <t>05/10/2026 15:42</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 89j (01/01/2027)</t>
+          <t>Valide 88j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>89j</t>
+          <t>88j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 113j (26/01/2027)</t>
+          <t>Valide 112j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>04/10/2026 13:06</t>
+          <t>05/10/2026 15:42</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 47j (20/11/2026)</t>
+          <t>Valide 46j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>47j</t>
+          <t>46j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 28j (02/11/2026)</t>
+          <t>Expire dans 27j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>04/10/2026 13:06</t>
+          <t>05/10/2026 15:42</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 128j (09/02/2027)</t>
+          <t>Valide 127j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>128j</t>
+          <t>127j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 146j (28/02/2027)</t>
+          <t>Valide 145j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>04/10/2026 13:06</t>
+          <t>05/10/2026 15:42</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 126j (07/02/2027)</t>
+          <t>Valide 124j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>126j</t>
+          <t>124j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 290j (22/07/2027)</t>
+          <t>Valide 289j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>04/10/2026 13:06</t>
+          <t>05/10/2026 15:42</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 10j (14/10/2026)</t>
+          <t>Expire dans 9j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>10j</t>
+          <t>9j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>04/10/2026 13:06</t>
+          <t>05/10/2026 15:42</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 86j (29/12/2026)</t>
+          <t>Valide 85j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>86j</t>
+          <t>85j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 64j (07/12/2026)</t>
+          <t>Valide 63j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>04/10/2026 13:06</t>
+          <t>05/10/2026 15:42</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 86j (29/12/2026)</t>
+          <t>Valide 85j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>86j</t>
+          <t>85j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 64j (07/12/2026)</t>
+          <t>Valide 63j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>04/10/2026 13:06</t>
+          <t>05/10/2026 15:42</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 5j (09/10/2026)</t>
+          <t>Expire dans 4j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>5j</t>
+          <t>4j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 57j (30/11/2026)</t>
+          <t>Valide 55j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>04/10/2026 13:06</t>
+          <t>05/10/2026 15:42</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -2011,22 +2011,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 5j (09/10/2026)</t>
+          <t>Expire dans 4j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>5j</t>
+          <t>4j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 57j (30/11/2026)</t>
+          <t>Valide 55j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>04/10/2026 13:06</t>
+          <t>05/10/2026 15:42</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -2193,22 +2193,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 128j (09/02/2027)</t>
+          <t>Valide 127j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>128j</t>
+          <t>127j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 47j (20/11/2026)</t>
+          <t>Valide 45j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>04/10/2026 13:06</t>
+          <t>05/10/2026 15:42</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2255,22 +2255,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 128j (09/02/2027)</t>
+          <t>Valide 127j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>128j</t>
+          <t>127j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 47j (20/11/2026)</t>
+          <t>Valide 45j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>04/10/2026 13:06</t>
+          <t>05/10/2026 15:42</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2465,22 +2465,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 76j (19/12/2026)</t>
+          <t>Valide 75j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>76j</t>
+          <t>75j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 299j (31/07/2027)</t>
+          <t>Valide 298j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>04/10/2026 13:06</t>
+          <t>05/10/2026 15:42</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2519,22 +2519,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 76j (19/12/2026)</t>
+          <t>Valide 75j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>76j</t>
+          <t>75j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 299j (31/07/2027)</t>
+          <t>Valide 298j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>04/10/2026 13:06</t>
+          <t>05/10/2026 15:42</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2733,22 +2733,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 9j (13/10/2026)</t>
+          <t>Expire dans 8j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>9j</t>
+          <t>8j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 370j (10/10/2027)</t>
+          <t>Valide 369j (10/10/2027)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>04/10/2026 13:06</t>
+          <t>05/10/2026 15:42</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 06/10/2026 14:06
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 59j (04/12/2026)</t>
+          <t>Valide 58j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>59j</t>
+          <t>58j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 150j (05/03/2027)</t>
+          <t>Valide 149j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>05/10/2026 15:42</t>
+          <t>06/10/2026 14:01</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 305j (07/08/2027)</t>
+          <t>Valide 304j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>05/10/2026 15:42</t>
+          <t>06/10/2026 14:01</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 88j (01/01/2027)</t>
+          <t>Valide 87j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>88j</t>
+          <t>87j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 112j (26/01/2027)</t>
+          <t>Valide 111j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>05/10/2026 15:42</t>
+          <t>06/10/2026 14:01</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 46j (20/11/2026)</t>
+          <t>Valide 45j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>46j</t>
+          <t>45j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 27j (02/11/2026)</t>
+          <t>Expire dans 26j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>05/10/2026 15:42</t>
+          <t>06/10/2026 14:01</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 127j (09/02/2027)</t>
+          <t>Valide 126j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>127j</t>
+          <t>126j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 145j (28/02/2027)</t>
+          <t>Valide 144j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>05/10/2026 15:42</t>
+          <t>06/10/2026 14:01</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1590,12 +1590,12 @@
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 289j (22/07/2027)</t>
+          <t>Valide 288j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>05/10/2026 15:42</t>
+          <t>06/10/2026 14:01</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 9j (14/10/2026)</t>
+          <t>Expire dans 8j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>9j</t>
+          <t>8j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>05/10/2026 15:42</t>
+          <t>06/10/2026 14:01</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 85j (29/12/2026)</t>
+          <t>Valide 84j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>85j</t>
+          <t>84j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 63j (07/12/2026)</t>
+          <t>Valide 62j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>05/10/2026 15:42</t>
+          <t>06/10/2026 14:01</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 85j (29/12/2026)</t>
+          <t>Valide 84j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>85j</t>
+          <t>84j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 63j (07/12/2026)</t>
+          <t>Valide 62j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>05/10/2026 15:42</t>
+          <t>06/10/2026 14:01</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,12 +1957,12 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 4j (09/10/2026)</t>
+          <t>Expire dans 3j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>4j</t>
+          <t>3j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
@@ -1972,7 +1972,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>05/10/2026 15:42</t>
+          <t>06/10/2026 14:01</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -2011,12 +2011,12 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 4j (09/10/2026)</t>
+          <t>Expire dans 3j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>4j</t>
+          <t>3j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>05/10/2026 15:42</t>
+          <t>06/10/2026 14:01</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -2193,12 +2193,12 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 127j (09/02/2027)</t>
+          <t>Valide 126j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>127j</t>
+          <t>126j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>05/10/2026 15:42</t>
+          <t>06/10/2026 14:01</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2255,12 +2255,12 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 127j (09/02/2027)</t>
+          <t>Valide 126j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>127j</t>
+          <t>126j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
@@ -2270,7 +2270,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>05/10/2026 15:42</t>
+          <t>06/10/2026 14:01</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2465,22 +2465,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 75j (19/12/2026)</t>
+          <t>Valide 74j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>75j</t>
+          <t>74j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 298j (31/07/2027)</t>
+          <t>Valide 297j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>05/10/2026 15:42</t>
+          <t>06/10/2026 14:01</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2519,22 +2519,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 75j (19/12/2026)</t>
+          <t>Valide 74j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>75j</t>
+          <t>74j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 298j (31/07/2027)</t>
+          <t>Valide 297j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>05/10/2026 15:42</t>
+          <t>06/10/2026 14:01</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2733,25 +2733,29 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 8j (13/10/2026)</t>
+          <t>Expire dans 7j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>8j</t>
+          <t>7j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 369j (10/10/2027)</t>
+          <t>Valide 368j (10/10/2027)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>05/10/2026 15:42</t>
-        </is>
-      </c>
-      <c r="P49" t="inlineStr"/>
+          <t>06/10/2026 14:01</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1" s="34">
       <c r="A50" s="3" t="inlineStr">

</xml_diff>

<commit_message>
chore: monitoring 07/10/2026 14:24
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 58j (04/12/2026)</t>
+          <t>Valide 57j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>58j</t>
+          <t>57j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 149j (05/03/2027)</t>
+          <t>Valide 148j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>06/10/2026 14:01</t>
+          <t>07/10/2026 14:19</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 304j (07/08/2027)</t>
+          <t>Valide 303j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>06/10/2026 14:01</t>
+          <t>07/10/2026 14:19</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 87j (01/01/2027)</t>
+          <t>Valide 86j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>87j</t>
+          <t>86j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 111j (26/01/2027)</t>
+          <t>Valide 110j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>06/10/2026 14:01</t>
+          <t>07/10/2026 14:19</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 45j (20/11/2026)</t>
+          <t>Valide 44j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>45j</t>
+          <t>44j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 26j (02/11/2026)</t>
+          <t>Expire dans 25j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>06/10/2026 14:01</t>
+          <t>07/10/2026 14:19</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 126j (09/02/2027)</t>
+          <t>Valide 125j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>126j</t>
+          <t>125j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 144j (28/02/2027)</t>
+          <t>Valide 143j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>06/10/2026 14:01</t>
+          <t>07/10/2026 14:19</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 124j (07/02/2027)</t>
+          <t>Valide 123j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>124j</t>
+          <t>123j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 288j (22/07/2027)</t>
+          <t>Valide 287j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>06/10/2026 14:01</t>
+          <t>07/10/2026 14:19</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 8j (14/10/2026)</t>
+          <t>Valide 197j (23/04/2027)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>8j</t>
+          <t>197j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>06/10/2026 14:01</t>
+          <t>07/10/2026 14:19</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 84j (29/12/2026)</t>
+          <t>Valide 83j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>84j</t>
+          <t>83j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 62j (07/12/2026)</t>
+          <t>Valide 61j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>06/10/2026 14:01</t>
+          <t>07/10/2026 14:19</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 84j (29/12/2026)</t>
+          <t>Valide 83j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>84j</t>
+          <t>83j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 62j (07/12/2026)</t>
+          <t>Valide 61j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>06/10/2026 14:01</t>
+          <t>07/10/2026 14:19</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 3j (09/10/2026)</t>
+          <t>Expire dans 2j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>3j</t>
+          <t>2j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 55j (30/11/2026)</t>
+          <t>Valide 54j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>06/10/2026 14:01</t>
+          <t>07/10/2026 14:19</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -2011,22 +2011,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 3j (09/10/2026)</t>
+          <t>Expire dans 2j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>3j</t>
+          <t>2j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 55j (30/11/2026)</t>
+          <t>Valide 54j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>06/10/2026 14:01</t>
+          <t>07/10/2026 14:19</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -2193,22 +2193,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 126j (09/02/2027)</t>
+          <t>Valide 125j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>126j</t>
+          <t>125j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 45j (20/11/2026)</t>
+          <t>Valide 44j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>06/10/2026 14:01</t>
+          <t>07/10/2026 14:19</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2255,22 +2255,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 126j (09/02/2027)</t>
+          <t>Valide 125j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>126j</t>
+          <t>125j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 45j (20/11/2026)</t>
+          <t>Valide 44j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>06/10/2026 14:01</t>
+          <t>07/10/2026 14:19</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2465,22 +2465,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 74j (19/12/2026)</t>
+          <t>Valide 73j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>74j</t>
+          <t>73j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 297j (31/07/2027)</t>
+          <t>Valide 296j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>06/10/2026 14:01</t>
+          <t>07/10/2026 14:19</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2519,22 +2519,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 74j (19/12/2026)</t>
+          <t>Valide 73j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>74j</t>
+          <t>73j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 297j (31/07/2027)</t>
+          <t>Valide 296j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>06/10/2026 14:01</t>
+          <t>07/10/2026 14:19</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2733,29 +2733,25 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 7j (13/10/2026)</t>
+          <t>Valide 197j (23/04/2027)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>7j</t>
+          <t>197j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 368j (10/10/2027)</t>
+          <t>Valide 367j (10/10/2027)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>06/10/2026 14:01</t>
-        </is>
-      </c>
-      <c r="P49" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>07/10/2026 14:19</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr"/>
     </row>
     <row r="50" ht="18" customHeight="1" s="34">
       <c r="A50" s="3" t="inlineStr">

</xml_diff>

<commit_message>
chore: monitoring 08/10/2026 14:32
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 57j (04/12/2026)</t>
+          <t>Valide 56j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>57j</t>
+          <t>56j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 148j (05/03/2027)</t>
+          <t>Valide 147j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>07/10/2026 14:19</t>
+          <t>08/10/2026 14:27</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 121j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>121j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 303j (07/08/2027)</t>
+          <t>Valide 302j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>07/10/2026 14:19</t>
+          <t>08/10/2026 14:27</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 86j (01/01/2027)</t>
+          <t>Valide 85j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>86j</t>
+          <t>85j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 110j (26/01/2027)</t>
+          <t>Valide 109j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>07/10/2026 14:19</t>
+          <t>08/10/2026 14:27</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 44j (20/11/2026)</t>
+          <t>Valide 43j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>44j</t>
+          <t>43j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 25j (02/11/2026)</t>
+          <t>Expire dans 24j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>07/10/2026 14:19</t>
+          <t>08/10/2026 14:27</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 125j (09/02/2027)</t>
+          <t>Valide 124j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>125j</t>
+          <t>124j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 143j (28/02/2027)</t>
+          <t>Valide 142j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>07/10/2026 14:19</t>
+          <t>08/10/2026 14:27</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 123j (07/02/2027)</t>
+          <t>Valide 121j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>123j</t>
+          <t>121j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 287j (22/07/2027)</t>
+          <t>Valide 286j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>07/10/2026 14:19</t>
+          <t>08/10/2026 14:27</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 197j (23/04/2027)</t>
+          <t>Valide 196j (23/04/2027)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>197j</t>
+          <t>196j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>07/10/2026 14:19</t>
+          <t>08/10/2026 14:27</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 83j (29/12/2026)</t>
+          <t>Valide 82j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>83j</t>
+          <t>82j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 61j (07/12/2026)</t>
+          <t>Valide 60j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>07/10/2026 14:19</t>
+          <t>08/10/2026 14:27</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 83j (29/12/2026)</t>
+          <t>Valide 82j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>83j</t>
+          <t>82j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 61j (07/12/2026)</t>
+          <t>Valide 60j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>07/10/2026 14:19</t>
+          <t>08/10/2026 14:27</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 2j (09/10/2026)</t>
+          <t>Expire dans 1j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>2j</t>
+          <t>1j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 54j (30/11/2026)</t>
+          <t>Valide 53j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>07/10/2026 14:19</t>
+          <t>08/10/2026 14:27</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -2011,22 +2011,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 2j (09/10/2026)</t>
+          <t>Expire dans 1j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>2j</t>
+          <t>1j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 54j (30/11/2026)</t>
+          <t>Valide 53j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>07/10/2026 14:19</t>
+          <t>08/10/2026 14:27</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -2193,22 +2193,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 125j (09/02/2027)</t>
+          <t>Valide 124j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>125j</t>
+          <t>124j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 44j (20/11/2026)</t>
+          <t>Valide 43j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>07/10/2026 14:19</t>
+          <t>08/10/2026 14:27</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2255,22 +2255,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 125j (09/02/2027)</t>
+          <t>Valide 124j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>125j</t>
+          <t>124j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 44j (20/11/2026)</t>
+          <t>Valide 43j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>07/10/2026 14:19</t>
+          <t>08/10/2026 14:27</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2465,22 +2465,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 73j (19/12/2026)</t>
+          <t>Valide 72j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>73j</t>
+          <t>72j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 296j (31/07/2027)</t>
+          <t>Valide 295j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>07/10/2026 14:19</t>
+          <t>08/10/2026 14:27</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2519,22 +2519,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 73j (19/12/2026)</t>
+          <t>Valide 72j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>73j</t>
+          <t>72j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 296j (31/07/2027)</t>
+          <t>Valide 295j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>07/10/2026 14:19</t>
+          <t>08/10/2026 14:27</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2733,22 +2733,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 197j (23/04/2027)</t>
+          <t>Valide 196j (23/04/2027)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>197j</t>
+          <t>196j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 367j (10/10/2027)</t>
+          <t>Valide 366j (10/10/2027)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>07/10/2026 14:19</t>
+          <t>08/10/2026 14:27</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
Inventaire : retrait des 4 lignes lead-portage (projet arrete)
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Inventaire" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Config" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventaire" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventaire'!$A$2:$N$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventaire'!$A$2:$N$47</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -670,7 +670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R50"/>
+  <dimension ref="A1:R46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col width="18" customWidth="1" style="34" min="1" max="1"/>
@@ -860,7 +860,6 @@
           <t>08/10/2026 14:27</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A5" s="3" t="inlineStr">
@@ -994,7 +993,6 @@
           <t>08/10/2026 14:27</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1" s="34">
       <c r="A8" s="8" t="inlineStr">
@@ -1064,7 +1062,6 @@
           <t>08/10/2026 14:27</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A9" s="3" t="inlineStr">
@@ -1170,7 +1167,6 @@
           <t>08/10/2026 14:27</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A11" s="3" t="inlineStr">
@@ -1276,7 +1272,6 @@
           <t>08/10/2026 14:27</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A13" s="3" t="inlineStr">
@@ -1598,7 +1593,6 @@
           <t>08/10/2026 14:27</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr"/>
     </row>
     <row r="23" ht="18" customHeight="1" s="34">
       <c r="A23" s="8" t="inlineStr">
@@ -1668,7 +1662,6 @@
           <t>08/10/2026 14:27</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
           <t>x</t>
@@ -1763,7 +1756,6 @@
           <t>08/10/2026 14:27</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr"/>
     </row>
     <row r="26" ht="18" customHeight="1" s="34">
       <c r="A26" s="3" t="inlineStr">
@@ -1829,7 +1821,6 @@
           <t>08/10/2026 14:27</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A27" s="8" t="inlineStr">
@@ -1911,195 +1902,197 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>lead-portage.com</t>
-        </is>
-      </c>
-      <c r="C29" s="31" t="inlineStr">
-        <is>
-          <t>https://lead-portage.com</t>
-        </is>
-      </c>
+          <t>g2a-portage.com</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="n"/>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Gandi</t>
-        </is>
-      </c>
-      <c r="E29" s="9" t="inlineStr">
-        <is>
-          <t>Namecheap</t>
-        </is>
-      </c>
-      <c r="F29" s="9" t="inlineStr">
-        <is>
-          <t>LaBuonCom</t>
-        </is>
-      </c>
-      <c r="G29" s="9" t="inlineStr">
-        <is>
-          <t>ELITEETPASSION</t>
-        </is>
-      </c>
+          <t>Infomaniak</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="n"/>
+      <c r="F29" s="9" t="n"/>
+      <c r="G29" s="9" t="n"/>
       <c r="H29" s="11" t="n"/>
       <c r="I29" s="12" t="inlineStr">
         <is>
           <t>Patrick</t>
         </is>
       </c>
-      <c r="J29" s="9" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="K29" s="9" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="L29" s="9" t="inlineStr">
-        <is>
-          <t>Expire dans 1j (09/10/2026)</t>
-        </is>
-      </c>
-      <c r="M29" s="9" t="inlineStr">
-        <is>
-          <t>1j</t>
-        </is>
-      </c>
-      <c r="N29" s="9" t="inlineStr">
-        <is>
-          <t>Valide 53j (30/11/2026)</t>
-        </is>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>08/10/2026 14:27</t>
-        </is>
-      </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+      <c r="J29" s="9" t="n"/>
+      <c r="K29" s="9" t="n"/>
+      <c r="L29" s="9" t="n"/>
+      <c r="M29" s="9" t="n"/>
+      <c r="N29" s="9" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1" s="34">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Lead-Portage</t>
+          <t>SelNHelp</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>leadportage.com</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>https://lead-portage.com/</t>
-        </is>
-      </c>
+          <t>selnhelp.net</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="n"/>
       <c r="D30" s="4" t="n"/>
       <c r="E30" s="4" t="n"/>
       <c r="F30" s="4" t="n"/>
       <c r="G30" s="4" t="n"/>
       <c r="H30" s="6" t="n"/>
-      <c r="I30" s="7" t="n"/>
+      <c r="I30" s="7" t="inlineStr">
+        <is>
+          <t>Patrick</t>
+        </is>
+      </c>
       <c r="J30" s="4" t="n"/>
-      <c r="K30" s="4" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="L30" s="4" t="inlineStr">
-        <is>
-          <t>Expire dans 1j (09/10/2026)</t>
-        </is>
-      </c>
-      <c r="M30" s="4" t="inlineStr">
-        <is>
-          <t>1j</t>
-        </is>
-      </c>
-      <c r="N30" s="4" t="inlineStr">
-        <is>
-          <t>Valide 53j (30/11/2026)</t>
-        </is>
-      </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>08/10/2026 14:27</t>
-        </is>
-      </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+      <c r="K30" s="4" t="n"/>
+      <c r="L30" s="4" t="n"/>
+      <c r="M30" s="4" t="n"/>
+      <c r="N30" s="4" t="n"/>
     </row>
     <row r="31" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>Lead-Portage</t>
+          <t>SelNHelp</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>lead-portage.fr</t>
-        </is>
-      </c>
-      <c r="C31" s="10" t="n"/>
-      <c r="D31" s="9" t="n"/>
-      <c r="E31" s="9" t="n"/>
-      <c r="F31" s="9" t="n"/>
+          <t>selnhelp.fr</t>
+        </is>
+      </c>
+      <c r="C31" s="31" t="inlineStr">
+        <is>
+          <t>https://selnhelp.fr</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>AWS</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>Namecheap</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>LaBuonCom</t>
+        </is>
+      </c>
       <c r="G31" s="9" t="n"/>
       <c r="H31" s="11" t="n"/>
-      <c r="I31" s="12" t="n"/>
-      <c r="J31" s="9" t="n"/>
-      <c r="K31" s="9" t="n"/>
-      <c r="L31" s="9" t="n"/>
-      <c r="M31" s="9" t="n"/>
-      <c r="N31" s="9" t="n"/>
+      <c r="I31" s="12" t="inlineStr">
+        <is>
+          <t>Patrick</t>
+        </is>
+      </c>
+      <c r="J31" s="9" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="K31" s="9" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="L31" s="9" t="inlineStr">
+        <is>
+          <t>Valide 124j (09/02/2027)</t>
+        </is>
+      </c>
+      <c r="M31" s="9" t="inlineStr">
+        <is>
+          <t>124j</t>
+        </is>
+      </c>
+      <c r="N31" s="9" t="inlineStr">
+        <is>
+          <t>Valide 43j (20/11/2026)</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>08/10/2026 14:27</t>
+        </is>
+      </c>
     </row>
     <row r="32" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Lead-Portage</t>
+          <t>IDEC</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>leadportage.fr</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="n"/>
-      <c r="D32" s="4" t="n"/>
+          <t>idec91.fr</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>https://selnhelp.fr/</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>GANDI</t>
+        </is>
+      </c>
       <c r="E32" s="4" t="n"/>
       <c r="F32" s="4" t="n"/>
-      <c r="G32" s="4" t="n"/>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>ELITEETPASSION</t>
+        </is>
+      </c>
       <c r="H32" s="6" t="n"/>
-      <c r="I32" s="7" t="n"/>
+      <c r="I32" s="7" t="inlineStr">
+        <is>
+          <t>Patrick</t>
+        </is>
+      </c>
       <c r="J32" s="4" t="n"/>
-      <c r="K32" s="4" t="n"/>
-      <c r="L32" s="4" t="n"/>
-      <c r="M32" s="4" t="n"/>
-      <c r="N32" s="4" t="n"/>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>Valide 124j (09/02/2027)</t>
+        </is>
+      </c>
+      <c r="M32" s="4" t="inlineStr">
+        <is>
+          <t>124j</t>
+        </is>
+      </c>
+      <c r="N32" s="4" t="inlineStr">
+        <is>
+          <t>Valide 43j (20/11/2026)</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>08/10/2026 14:27</t>
+        </is>
+      </c>
     </row>
     <row r="33" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>Lead-Portage</t>
-        </is>
-      </c>
-      <c r="B33" s="9" t="inlineStr">
-        <is>
-          <t>g2a-portage.com</t>
-        </is>
-      </c>
-      <c r="C33" s="10" t="n"/>
-      <c r="D33" s="9" t="inlineStr">
-        <is>
-          <t>Infomaniak</t>
-        </is>
-      </c>
+          <t>GRELAT</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="n"/>
+      <c r="C33" s="13" t="n"/>
+      <c r="D33" s="9" t="n"/>
       <c r="E33" s="9" t="n"/>
       <c r="F33" s="9" t="n"/>
       <c r="G33" s="9" t="n"/>
@@ -2118,23 +2111,23 @@
     <row r="34" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>SelNHelp</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>selnhelp.net</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="n"/>
-      <c r="D34" s="4" t="n"/>
+          <t>GRASSET</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="n"/>
+      <c r="C34" s="14" t="n"/>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>IONOS</t>
+        </is>
+      </c>
       <c r="E34" s="4" t="n"/>
       <c r="F34" s="4" t="n"/>
       <c r="G34" s="4" t="n"/>
       <c r="H34" s="6" t="n"/>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>Patrick</t>
+          <t>Cesar / Axel</t>
         </is>
       </c>
       <c r="J34" s="4" t="n"/>
@@ -2146,34 +2139,14 @@
     <row r="35" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>SelNHelp</t>
-        </is>
-      </c>
-      <c r="B35" s="9" t="inlineStr">
-        <is>
-          <t>selnhelp.fr</t>
-        </is>
-      </c>
-      <c r="C35" s="31" t="inlineStr">
-        <is>
-          <t>https://selnhelp.fr</t>
-        </is>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
-        <is>
-          <t>AWS</t>
-        </is>
-      </c>
-      <c r="E35" s="9" t="inlineStr">
-        <is>
-          <t>Namecheap</t>
-        </is>
-      </c>
-      <c r="F35" s="9" t="inlineStr">
-        <is>
-          <t>LaBuonCom</t>
-        </is>
-      </c>
+          <t>SPI PONTAULT</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="n"/>
+      <c r="C35" s="13" t="n"/>
+      <c r="D35" s="9" t="n"/>
+      <c r="E35" s="9" t="n"/>
+      <c r="F35" s="9" t="n"/>
       <c r="G35" s="9" t="n"/>
       <c r="H35" s="11" t="n"/>
       <c r="I35" s="12" t="inlineStr">
@@ -2181,64 +2154,30 @@
           <t>Patrick</t>
         </is>
       </c>
-      <c r="J35" s="9" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="K35" s="9" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="L35" s="9" t="inlineStr">
-        <is>
-          <t>Valide 124j (09/02/2027)</t>
-        </is>
-      </c>
-      <c r="M35" s="9" t="inlineStr">
-        <is>
-          <t>124j</t>
-        </is>
-      </c>
-      <c r="N35" s="9" t="inlineStr">
-        <is>
-          <t>Valide 43j (20/11/2026)</t>
-        </is>
-      </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>08/10/2026 14:27</t>
-        </is>
-      </c>
-      <c r="P35" t="inlineStr"/>
+      <c r="J35" s="9" t="n"/>
+      <c r="K35" s="9" t="n"/>
+      <c r="L35" s="9" t="n"/>
+      <c r="M35" s="9" t="n"/>
+      <c r="N35" s="9" t="n"/>
     </row>
     <row r="36" ht="18" customHeight="1" s="34">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>IDEC</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>idec91.fr</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>https://selnhelp.fr/</t>
-        </is>
-      </c>
+          <t>Elite Et Passion</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="n"/>
+      <c r="C36" s="14" t="n"/>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>GANDI</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="E36" s="4" t="n"/>
       <c r="F36" s="4" t="n"/>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>ELITEETPASSION</t>
+          <t>ALBYS</t>
         </is>
       </c>
       <c r="H36" s="6" t="n"/>
@@ -2248,49 +2187,35 @@
         </is>
       </c>
       <c r="J36" s="4" t="n"/>
-      <c r="K36" s="4" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="L36" s="4" t="inlineStr">
-        <is>
-          <t>Valide 124j (09/02/2027)</t>
-        </is>
-      </c>
-      <c r="M36" s="4" t="inlineStr">
-        <is>
-          <t>124j</t>
-        </is>
-      </c>
-      <c r="N36" s="4" t="inlineStr">
-        <is>
-          <t>Valide 43j (20/11/2026)</t>
-        </is>
-      </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>08/10/2026 14:27</t>
-        </is>
-      </c>
-      <c r="P36" t="inlineStr"/>
+      <c r="K36" s="4" t="n"/>
+      <c r="L36" s="4" t="n"/>
+      <c r="M36" s="4" t="n"/>
+      <c r="N36" s="4" t="n"/>
     </row>
     <row r="37" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>GRELAT</t>
+          <t>Fichet Group</t>
         </is>
       </c>
       <c r="B37" s="9" t="n"/>
       <c r="C37" s="13" t="n"/>
-      <c r="D37" s="9" t="n"/>
+      <c r="D37" s="9" t="inlineStr">
+        <is>
+          <t>AWS</t>
+        </is>
+      </c>
       <c r="E37" s="9" t="n"/>
       <c r="F37" s="9" t="n"/>
-      <c r="G37" s="9" t="n"/>
+      <c r="G37" s="9" t="inlineStr">
+        <is>
+          <t>ALBYS</t>
+        </is>
+      </c>
       <c r="H37" s="11" t="n"/>
       <c r="I37" s="12" t="inlineStr">
         <is>
-          <t>Patrick</t>
+          <t>Cesar / Axel / cédric</t>
         </is>
       </c>
       <c r="J37" s="9" t="n"/>
@@ -2302,75 +2227,145 @@
     <row r="38" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>GRASSET</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="n"/>
-      <c r="C38" s="14" t="n"/>
+          <t xml:space="preserve"> ISYTEM</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>isytem.com</t>
+        </is>
+      </c>
+      <c r="C38" s="32" t="inlineStr">
+        <is>
+          <t>https://isytem.com</t>
+        </is>
+      </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>IONOS</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="n"/>
-      <c r="F38" s="4" t="n"/>
-      <c r="G38" s="4" t="n"/>
+          <t>GANDI</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>Namecheap</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>LaBuonCom</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>ELITEETPASSION</t>
+        </is>
+      </c>
       <c r="H38" s="6" t="n"/>
-      <c r="I38" s="7" t="inlineStr">
-        <is>
-          <t>Cesar / Axel</t>
-        </is>
-      </c>
-      <c r="J38" s="4" t="n"/>
-      <c r="K38" s="4" t="n"/>
-      <c r="L38" s="4" t="n"/>
-      <c r="M38" s="4" t="n"/>
-      <c r="N38" s="4" t="n"/>
+      <c r="I38" s="7" t="n"/>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="K38" s="4" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>Valide 72j (19/12/2026)</t>
+        </is>
+      </c>
+      <c r="M38" s="4" t="inlineStr">
+        <is>
+          <t>72j</t>
+        </is>
+      </c>
+      <c r="N38" s="4" t="inlineStr">
+        <is>
+          <t>Valide 295j (31/07/2027)</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>08/10/2026 14:27</t>
+        </is>
+      </c>
     </row>
     <row r="39" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>SPI PONTAULT</t>
-        </is>
-      </c>
-      <c r="B39" s="9" t="n"/>
-      <c r="C39" s="13" t="n"/>
-      <c r="D39" s="9" t="n"/>
+          <t xml:space="preserve"> ISYTEM</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>isytem.fr</t>
+        </is>
+      </c>
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>https://isytem.com/</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>GANDI</t>
+        </is>
+      </c>
       <c r="E39" s="9" t="n"/>
       <c r="F39" s="9" t="n"/>
       <c r="G39" s="9" t="n"/>
       <c r="H39" s="11" t="n"/>
-      <c r="I39" s="12" t="inlineStr">
-        <is>
-          <t>Patrick</t>
-        </is>
-      </c>
+      <c r="I39" s="12" t="n"/>
       <c r="J39" s="9" t="n"/>
-      <c r="K39" s="9" t="n"/>
-      <c r="L39" s="9" t="n"/>
-      <c r="M39" s="9" t="n"/>
-      <c r="N39" s="9" t="n"/>
+      <c r="K39" s="9" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="L39" s="9" t="inlineStr">
+        <is>
+          <t>Valide 72j (19/12/2026)</t>
+        </is>
+      </c>
+      <c r="M39" s="9" t="inlineStr">
+        <is>
+          <t>72j</t>
+        </is>
+      </c>
+      <c r="N39" s="9" t="inlineStr">
+        <is>
+          <t>Valide 295j (31/07/2027)</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>08/10/2026 14:27</t>
+        </is>
+      </c>
     </row>
     <row r="40" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Elite Et Passion</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="n"/>
-      <c r="C40" s="14" t="n"/>
+          <t xml:space="preserve"> ISYTEM</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>isytem.net</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="n"/>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>GANDI</t>
         </is>
       </c>
       <c r="E40" s="4" t="n"/>
       <c r="F40" s="4" t="n"/>
-      <c r="G40" s="4" t="inlineStr">
-        <is>
-          <t>ALBYS</t>
-        </is>
-      </c>
+      <c r="G40" s="4" t="n"/>
       <c r="H40" s="6" t="n"/>
       <c r="I40" s="7" t="inlineStr">
         <is>
@@ -2386,14 +2381,18 @@
     <row r="41" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>Fichet Group</t>
-        </is>
-      </c>
-      <c r="B41" s="9" t="n"/>
-      <c r="C41" s="13" t="n"/>
+          <t>CS2DI</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>cs2di.com</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="n"/>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>google</t>
         </is>
       </c>
       <c r="E41" s="9" t="n"/>
@@ -2406,7 +2405,7 @@
       <c r="H41" s="11" t="n"/>
       <c r="I41" s="12" t="inlineStr">
         <is>
-          <t>Cesar / Axel / cédric</t>
+          <t>Patrick</t>
         </is>
       </c>
       <c r="J41" s="9" t="n"/>
@@ -2418,153 +2417,69 @@
     <row r="42" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ISYTEM</t>
+          <t>HOLDJUST</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>isytem.com</t>
-        </is>
-      </c>
-      <c r="C42" s="32" t="inlineStr">
-        <is>
-          <t>https://isytem.com</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>GANDI</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>Namecheap</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>LaBuonCom</t>
-        </is>
-      </c>
-      <c r="G42" s="4" t="inlineStr">
-        <is>
-          <t>ELITEETPASSION</t>
-        </is>
-      </c>
+          <t>Holdjust.com</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="n"/>
+      <c r="D42" s="4" t="n"/>
+      <c r="E42" s="4" t="n"/>
+      <c r="F42" s="4" t="n"/>
+      <c r="G42" s="4" t="n"/>
       <c r="H42" s="6" t="n"/>
       <c r="I42" s="7" t="n"/>
-      <c r="J42" s="4" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="K42" s="4" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="L42" s="4" t="inlineStr">
-        <is>
-          <t>Valide 72j (19/12/2026)</t>
-        </is>
-      </c>
-      <c r="M42" s="4" t="inlineStr">
-        <is>
-          <t>72j</t>
-        </is>
-      </c>
-      <c r="N42" s="4" t="inlineStr">
-        <is>
-          <t>Valide 295j (31/07/2027)</t>
-        </is>
-      </c>
-      <c r="O42" t="inlineStr">
-        <is>
-          <t>08/10/2026 14:27</t>
-        </is>
-      </c>
-      <c r="P42" t="inlineStr"/>
+      <c r="J42" s="4" t="n"/>
+      <c r="K42" s="4" t="n"/>
+      <c r="L42" s="4" t="n"/>
+      <c r="M42" s="4" t="n"/>
+      <c r="N42" s="4" t="n"/>
     </row>
     <row r="43" ht="18" customHeight="1" s="34">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ISYTEM</t>
+          <t>HOLDJUST</t>
         </is>
       </c>
       <c r="B43" s="9" t="inlineStr">
         <is>
-          <t>isytem.fr</t>
-        </is>
-      </c>
-      <c r="C43" s="10" t="inlineStr">
-        <is>
-          <t>https://isytem.com/</t>
-        </is>
-      </c>
-      <c r="D43" s="9" t="inlineStr">
-        <is>
-          <t>GANDI</t>
-        </is>
-      </c>
+          <t>holdjust.fr</t>
+        </is>
+      </c>
+      <c r="C43" s="31" t="n"/>
+      <c r="D43" s="9" t="n"/>
       <c r="E43" s="9" t="n"/>
       <c r="F43" s="9" t="n"/>
       <c r="G43" s="9" t="n"/>
       <c r="H43" s="11" t="n"/>
       <c r="I43" s="12" t="n"/>
       <c r="J43" s="9" t="n"/>
-      <c r="K43" s="9" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="L43" s="9" t="inlineStr">
-        <is>
-          <t>Valide 72j (19/12/2026)</t>
-        </is>
-      </c>
-      <c r="M43" s="9" t="inlineStr">
-        <is>
-          <t>72j</t>
-        </is>
-      </c>
-      <c r="N43" s="9" t="inlineStr">
-        <is>
-          <t>Valide 295j (31/07/2027)</t>
-        </is>
-      </c>
-      <c r="O43" t="inlineStr">
-        <is>
-          <t>08/10/2026 14:27</t>
-        </is>
-      </c>
-      <c r="P43" t="inlineStr"/>
+      <c r="K43" s="9" t="n"/>
+      <c r="L43" s="9" t="n"/>
+      <c r="M43" s="9" t="n"/>
+      <c r="N43" s="9" t="n"/>
     </row>
     <row r="44" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ISYTEM</t>
+          <t>HOLDJUST</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>isytem.net</t>
+          <t>holdjust.net</t>
         </is>
       </c>
       <c r="C44" s="5" t="n"/>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>GANDI</t>
-        </is>
-      </c>
+      <c r="D44" s="4" t="n"/>
       <c r="E44" s="4" t="n"/>
       <c r="F44" s="4" t="n"/>
       <c r="G44" s="4" t="n"/>
       <c r="H44" s="6" t="n"/>
-      <c r="I44" s="7" t="inlineStr">
-        <is>
-          <t>Patrick</t>
-        </is>
-      </c>
+      <c r="I44" s="7" t="n"/>
       <c r="J44" s="4" t="n"/>
       <c r="K44" s="4" t="n"/>
       <c r="L44" s="4" t="n"/>
@@ -2574,22 +2489,34 @@
     <row r="45" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>CS2DI</t>
+          <t>DRAVEIL HANDBALL</t>
         </is>
       </c>
       <c r="B45" s="9" t="inlineStr">
         <is>
-          <t>cs2di.com</t>
-        </is>
-      </c>
-      <c r="C45" s="10" t="n"/>
+          <t>draveil-handball.fr</t>
+        </is>
+      </c>
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>https://draveil-handball.fr</t>
+        </is>
+      </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>google</t>
-        </is>
-      </c>
-      <c r="E45" s="9" t="n"/>
-      <c r="F45" s="9" t="n"/>
+          <t>Gandi</t>
+        </is>
+      </c>
+      <c r="E45" s="9" t="inlineStr">
+        <is>
+          <t>Namecheap</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="inlineStr">
+        <is>
+          <t>LaBuonCom</t>
+        </is>
+      </c>
       <c r="G45" s="9" t="inlineStr">
         <is>
           <t>ALBYS</t>
@@ -2598,27 +2525,48 @@
       <c r="H45" s="11" t="n"/>
       <c r="I45" s="12" t="inlineStr">
         <is>
-          <t>Patrick</t>
-        </is>
-      </c>
-      <c r="J45" s="9" t="n"/>
-      <c r="K45" s="9" t="n"/>
-      <c r="L45" s="9" t="n"/>
-      <c r="M45" s="9" t="n"/>
-      <c r="N45" s="9" t="n"/>
+          <t>Axel</t>
+        </is>
+      </c>
+      <c r="J45" s="9" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="K45" s="9" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="L45" s="9" t="inlineStr">
+        <is>
+          <t>Valide 196j (23/04/2027)</t>
+        </is>
+      </c>
+      <c r="M45" s="9" t="inlineStr">
+        <is>
+          <t>196j</t>
+        </is>
+      </c>
+      <c r="N45" s="9" t="inlineStr">
+        <is>
+          <t>Valide 366j (10/10/2027)</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>08/10/2026 14:27</t>
+        </is>
+      </c>
     </row>
     <row r="46" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>HOLDJUST</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>Holdjust.com</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="n"/>
+          <t>PREMIUM-TRADING</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="n"/>
+      <c r="C46" s="14" t="n"/>
       <c r="D46" s="4" t="n"/>
       <c r="E46" s="4" t="n"/>
       <c r="F46" s="4" t="n"/>
@@ -2631,151 +2579,13 @@
       <c r="M46" s="4" t="n"/>
       <c r="N46" s="4" t="n"/>
     </row>
-    <row r="47" hidden="1" ht="18" customHeight="1" s="34">
-      <c r="A47" s="8" t="inlineStr">
-        <is>
-          <t>HOLDJUST</t>
-        </is>
-      </c>
-      <c r="B47" s="9" t="inlineStr">
-        <is>
-          <t>holdjust.fr</t>
-        </is>
-      </c>
-      <c r="C47" s="31" t="n"/>
-      <c r="D47" s="9" t="n"/>
-      <c r="E47" s="9" t="n"/>
-      <c r="F47" s="9" t="n"/>
-      <c r="G47" s="9" t="n"/>
-      <c r="H47" s="11" t="n"/>
-      <c r="I47" s="12" t="n"/>
-      <c r="J47" s="9" t="n"/>
-      <c r="K47" s="9" t="n"/>
-      <c r="L47" s="9" t="n"/>
-      <c r="M47" s="9" t="n"/>
-      <c r="N47" s="9" t="n"/>
-    </row>
-    <row r="48" hidden="1" ht="18" customHeight="1" s="34">
-      <c r="A48" s="3" t="inlineStr">
-        <is>
-          <t>HOLDJUST</t>
-        </is>
-      </c>
-      <c r="B48" s="4" t="inlineStr">
-        <is>
-          <t>holdjust.net</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="n"/>
-      <c r="D48" s="4" t="n"/>
-      <c r="E48" s="4" t="n"/>
-      <c r="F48" s="4" t="n"/>
-      <c r="G48" s="4" t="n"/>
-      <c r="H48" s="6" t="n"/>
-      <c r="I48" s="7" t="n"/>
-      <c r="J48" s="4" t="n"/>
-      <c r="K48" s="4" t="n"/>
-      <c r="L48" s="4" t="n"/>
-      <c r="M48" s="4" t="n"/>
-      <c r="N48" s="4" t="n"/>
-    </row>
-    <row r="49" hidden="1" ht="18" customHeight="1" s="34">
-      <c r="A49" s="8" t="inlineStr">
-        <is>
-          <t>DRAVEIL HANDBALL</t>
-        </is>
-      </c>
-      <c r="B49" s="9" t="inlineStr">
-        <is>
-          <t>draveil-handball.fr</t>
-        </is>
-      </c>
-      <c r="C49" s="10" t="inlineStr">
-        <is>
-          <t>https://draveil-handball.fr</t>
-        </is>
-      </c>
-      <c r="D49" s="9" t="inlineStr">
-        <is>
-          <t>Gandi</t>
-        </is>
-      </c>
-      <c r="E49" s="9" t="inlineStr">
-        <is>
-          <t>Namecheap</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="inlineStr">
-        <is>
-          <t>LaBuonCom</t>
-        </is>
-      </c>
-      <c r="G49" s="9" t="inlineStr">
-        <is>
-          <t>ALBYS</t>
-        </is>
-      </c>
-      <c r="H49" s="11" t="n"/>
-      <c r="I49" s="12" t="inlineStr">
-        <is>
-          <t>Axel</t>
-        </is>
-      </c>
-      <c r="J49" s="9" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="K49" s="9" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="L49" s="9" t="inlineStr">
-        <is>
-          <t>Valide 196j (23/04/2027)</t>
-        </is>
-      </c>
-      <c r="M49" s="9" t="inlineStr">
-        <is>
-          <t>196j</t>
-        </is>
-      </c>
-      <c r="N49" s="9" t="inlineStr">
-        <is>
-          <t>Valide 366j (10/10/2027)</t>
-        </is>
-      </c>
-      <c r="O49" t="inlineStr">
-        <is>
-          <t>08/10/2026 14:27</t>
-        </is>
-      </c>
-      <c r="P49" t="inlineStr"/>
-    </row>
-    <row r="50" ht="18" customHeight="1" s="34">
-      <c r="A50" s="3" t="inlineStr">
-        <is>
-          <t>PREMIUM-TRADING</t>
-        </is>
-      </c>
-      <c r="B50" s="4" t="n"/>
-      <c r="C50" s="14" t="n"/>
-      <c r="D50" s="4" t="n"/>
-      <c r="E50" s="4" t="n"/>
-      <c r="F50" s="4" t="n"/>
-      <c r="G50" s="4" t="n"/>
-      <c r="H50" s="6" t="n"/>
-      <c r="I50" s="7" t="n"/>
-      <c r="J50" s="4" t="n"/>
-      <c r="K50" s="4" t="n"/>
-      <c r="L50" s="4" t="n"/>
-      <c r="M50" s="4" t="n"/>
-      <c r="N50" s="4" t="n"/>
-    </row>
+    <row r="47" hidden="1" s="34"/>
+    <row r="48" hidden="1" s="34"/>
+    <row r="49" hidden="1" s="34"/>
+    <row r="50" s="34"/>
     <row r="51" hidden="1" ht="18" customHeight="1" s="34"/>
   </sheetData>
-  <autoFilter ref="A2:N51">
+  <autoFilter ref="A2:N47">
     <filterColumn colId="11" hiddenButton="0" showButton="1">
       <customFilters>
         <customFilter val=" " operator="notEqual"/>
@@ -2791,9 +2601,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: monitoring 09/10/2026 14:18
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventaire" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Inventaire" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Config" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventaire'!$A$2:$N$47</definedName>
@@ -842,24 +842,25 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 56j (04/12/2026)</t>
+          <t>Valide 55j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>56j</t>
+          <t>55j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 147j (05/03/2027)</t>
+          <t>Valide 146j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>08/10/2026 14:27</t>
-        </is>
-      </c>
+          <t>09/10/2026 14:14</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A5" s="3" t="inlineStr">
@@ -975,24 +976,25 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 121j (07/02/2027)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>121j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 302j (07/08/2027)</t>
+          <t>Valide 301j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>08/10/2026 14:27</t>
-        </is>
-      </c>
+          <t>09/10/2026 14:14</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1" s="34">
       <c r="A8" s="8" t="inlineStr">
@@ -1044,24 +1046,25 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 85j (01/01/2027)</t>
+          <t>Valide 84j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>85j</t>
+          <t>84j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 109j (26/01/2027)</t>
+          <t>Valide 108j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>08/10/2026 14:27</t>
-        </is>
-      </c>
+          <t>09/10/2026 14:14</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A9" s="3" t="inlineStr">
@@ -1149,24 +1152,25 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 43j (20/11/2026)</t>
+          <t>Valide 42j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>43j</t>
+          <t>42j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 24j (02/11/2026)</t>
+          <t>Expire dans 23j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>08/10/2026 14:27</t>
-        </is>
-      </c>
+          <t>09/10/2026 14:14</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A11" s="3" t="inlineStr">
@@ -1254,24 +1258,25 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 124j (09/02/2027)</t>
+          <t>Valide 123j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>124j</t>
+          <t>123j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 142j (28/02/2027)</t>
+          <t>Valide 141j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>08/10/2026 14:27</t>
-        </is>
-      </c>
+          <t>09/10/2026 14:14</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A13" s="3" t="inlineStr">
@@ -1585,14 +1590,15 @@
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 286j (22/07/2027)</t>
+          <t>Valide 285j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>08/10/2026 14:27</t>
-        </is>
-      </c>
+          <t>09/10/2026 14:14</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr"/>
     </row>
     <row r="23" ht="18" customHeight="1" s="34">
       <c r="A23" s="8" t="inlineStr">
@@ -1644,24 +1650,25 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 196j (23/04/2027)</t>
+          <t>Valide 195j (23/04/2027)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>196j</t>
+          <t>195j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Whois command returned no output</t>
+          <t>Valide 381j (25/10/2027)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>08/10/2026 14:27</t>
-        </is>
-      </c>
+          <t>09/10/2026 14:14</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
           <t>x</t>
@@ -1738,24 +1745,25 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 82j (29/12/2026)</t>
+          <t>Valide 81j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>82j</t>
+          <t>81j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 60j (07/12/2026)</t>
+          <t>Valide 59j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>08/10/2026 14:27</t>
-        </is>
-      </c>
+          <t>09/10/2026 14:14</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr"/>
     </row>
     <row r="26" ht="18" customHeight="1" s="34">
       <c r="A26" s="3" t="inlineStr">
@@ -1803,24 +1811,25 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 82j (29/12/2026)</t>
+          <t>Valide 81j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>82j</t>
+          <t>81j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 60j (07/12/2026)</t>
+          <t>Valide 59j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>08/10/2026 14:27</t>
-        </is>
-      </c>
+          <t>09/10/2026 14:14</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A27" s="8" t="inlineStr">
@@ -2004,24 +2013,25 @@
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t>Valide 124j (09/02/2027)</t>
+          <t>Valide 123j (09/02/2027)</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>124j</t>
+          <t>123j</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
-          <t>Valide 43j (20/11/2026)</t>
+          <t>Valide 42j (20/11/2026)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>08/10/2026 14:27</t>
-        </is>
-      </c>
+          <t>09/10/2026 14:14</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr"/>
     </row>
     <row r="32" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A32" s="3" t="inlineStr">
@@ -2065,24 +2075,25 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Valide 124j (09/02/2027)</t>
+          <t>Valide 123j (09/02/2027)</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>124j</t>
+          <t>123j</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Valide 43j (20/11/2026)</t>
+          <t>Valide 42j (20/11/2026)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>08/10/2026 14:27</t>
-        </is>
-      </c>
+          <t>09/10/2026 14:14</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr"/>
     </row>
     <row r="33" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A33" s="8" t="inlineStr">
@@ -2274,24 +2285,25 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Valide 72j (19/12/2026)</t>
+          <t>Valide 71j (19/12/2026)</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>72j</t>
+          <t>71j</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>Valide 295j (31/07/2027)</t>
+          <t>Valide 294j (31/07/2027)</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>08/10/2026 14:27</t>
-        </is>
-      </c>
+          <t>09/10/2026 14:14</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr"/>
     </row>
     <row r="39" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A39" s="8" t="inlineStr">
@@ -2327,24 +2339,25 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t>Valide 72j (19/12/2026)</t>
+          <t>Valide 71j (19/12/2026)</t>
         </is>
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>72j</t>
+          <t>71j</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
         <is>
-          <t>Valide 295j (31/07/2027)</t>
+          <t>Valide 294j (31/07/2027)</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>08/10/2026 14:27</t>
-        </is>
-      </c>
+          <t>09/10/2026 14:14</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr"/>
     </row>
     <row r="40" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A40" s="3" t="inlineStr">
@@ -2540,24 +2553,25 @@
       </c>
       <c r="L45" s="9" t="inlineStr">
         <is>
-          <t>Valide 196j (23/04/2027)</t>
+          <t>Valide 195j (23/04/2027)</t>
         </is>
       </c>
       <c r="M45" s="9" t="inlineStr">
         <is>
-          <t>196j</t>
+          <t>195j</t>
         </is>
       </c>
       <c r="N45" s="9" t="inlineStr">
         <is>
-          <t>Valide 366j (10/10/2027)</t>
+          <t>Valide 365j (10/10/2027)</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>08/10/2026 14:27</t>
-        </is>
-      </c>
+          <t>09/10/2026 14:14</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr"/>
     </row>
     <row r="46" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A46" s="3" t="inlineStr">

</xml_diff>

<commit_message>
chore: monitoring 10/10/2026 13:29
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 55j (04/12/2026)</t>
+          <t>Valide 54j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>55j</t>
+          <t>54j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 146j (05/03/2027)</t>
+          <t>Valide 145j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>09/10/2026 14:14</t>
+          <t>10/10/2026 13:24</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 120j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>120j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 301j (07/08/2027)</t>
+          <t>Valide 300j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>09/10/2026 14:14</t>
+          <t>10/10/2026 13:24</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 84j (01/01/2027)</t>
+          <t>Valide 83j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>84j</t>
+          <t>83j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 108j (26/01/2027)</t>
+          <t>Valide 107j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>09/10/2026 14:14</t>
+          <t>10/10/2026 13:24</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 42j (20/11/2026)</t>
+          <t>Valide 41j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>42j</t>
+          <t>41j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 23j (02/11/2026)</t>
+          <t>Expire dans 22j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>09/10/2026 14:14</t>
+          <t>10/10/2026 13:24</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 123j (09/02/2027)</t>
+          <t>Valide 122j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>123j</t>
+          <t>122j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 141j (28/02/2027)</t>
+          <t>Valide 140j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>09/10/2026 14:14</t>
+          <t>10/10/2026 13:24</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 121j (07/02/2027)</t>
+          <t>Valide 120j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>121j</t>
+          <t>120j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 285j (22/07/2027)</t>
+          <t>Valide 284j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>09/10/2026 14:14</t>
+          <t>10/10/2026 13:24</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 195j (23/04/2027)</t>
+          <t>Valide 194j (23/04/2027)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>195j</t>
+          <t>194j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Valide 381j (25/10/2027)</t>
+          <t>Valide 380j (25/10/2027)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>09/10/2026 14:14</t>
+          <t>10/10/2026 13:24</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 81j (29/12/2026)</t>
+          <t>Valide 80j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>81j</t>
+          <t>80j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 59j (07/12/2026)</t>
+          <t>Valide 58j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>09/10/2026 14:14</t>
+          <t>10/10/2026 13:24</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 81j (29/12/2026)</t>
+          <t>Valide 80j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>81j</t>
+          <t>80j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 59j (07/12/2026)</t>
+          <t>Valide 58j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>09/10/2026 14:14</t>
+          <t>10/10/2026 13:24</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2013,22 +2013,22 @@
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t>Valide 123j (09/02/2027)</t>
+          <t>Valide 122j (09/02/2027)</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>123j</t>
+          <t>122j</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
-          <t>Valide 42j (20/11/2026)</t>
+          <t>Valide 41j (20/11/2026)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>09/10/2026 14:14</t>
+          <t>10/10/2026 13:24</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
@@ -2075,22 +2075,22 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Valide 123j (09/02/2027)</t>
+          <t>Valide 122j (09/02/2027)</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>123j</t>
+          <t>122j</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Valide 42j (20/11/2026)</t>
+          <t>Valide 41j (20/11/2026)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>09/10/2026 14:14</t>
+          <t>10/10/2026 13:24</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
@@ -2285,22 +2285,22 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Valide 71j (19/12/2026)</t>
+          <t>Valide 70j (19/12/2026)</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>71j</t>
+          <t>70j</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>Valide 294j (31/07/2027)</t>
+          <t>Valide 293j (31/07/2027)</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>09/10/2026 14:14</t>
+          <t>10/10/2026 13:24</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
@@ -2339,22 +2339,22 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t>Valide 71j (19/12/2026)</t>
+          <t>Valide 70j (19/12/2026)</t>
         </is>
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>71j</t>
+          <t>70j</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
         <is>
-          <t>Valide 294j (31/07/2027)</t>
+          <t>Valide 293j (31/07/2027)</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>09/10/2026 14:14</t>
+          <t>10/10/2026 13:24</t>
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
@@ -2553,22 +2553,22 @@
       </c>
       <c r="L45" s="9" t="inlineStr">
         <is>
-          <t>Valide 195j (23/04/2027)</t>
+          <t>Valide 194j (23/04/2027)</t>
         </is>
       </c>
       <c r="M45" s="9" t="inlineStr">
         <is>
-          <t>195j</t>
+          <t>194j</t>
         </is>
       </c>
       <c r="N45" s="9" t="inlineStr">
         <is>
-          <t>Valide 365j (10/10/2027)</t>
+          <t>Valide 364j (10/10/2027)</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>09/10/2026 14:14</t>
+          <t>10/10/2026 13:24</t>
         </is>
       </c>
       <c r="P45" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 11/10/2026 13:56
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 54j (04/12/2026)</t>
+          <t>Valide 53j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>54j</t>
+          <t>53j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 145j (05/03/2027)</t>
+          <t>Valide 144j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>10/10/2026 13:24</t>
+          <t>11/10/2026 13:51</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 120j (07/02/2027)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>120j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 300j (07/08/2027)</t>
+          <t>Valide 299j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>10/10/2026 13:24</t>
+          <t>11/10/2026 13:51</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 83j (01/01/2027)</t>
+          <t>Valide 82j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>83j</t>
+          <t>82j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 107j (26/01/2027)</t>
+          <t>Valide 106j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>10/10/2026 13:24</t>
+          <t>11/10/2026 13:51</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 41j (20/11/2026)</t>
+          <t>Valide 40j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>41j</t>
+          <t>40j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 22j (02/11/2026)</t>
+          <t>Expire dans 21j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>10/10/2026 13:24</t>
+          <t>11/10/2026 13:51</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 122j (09/02/2027)</t>
+          <t>Valide 121j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>122j</t>
+          <t>121j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 140j (28/02/2027)</t>
+          <t>Valide 139j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>10/10/2026 13:24</t>
+          <t>11/10/2026 13:51</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 120j (07/02/2027)</t>
+          <t>Valide 119j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>120j</t>
+          <t>119j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 284j (22/07/2027)</t>
+          <t>Valide 283j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>10/10/2026 13:24</t>
+          <t>11/10/2026 13:51</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 194j (23/04/2027)</t>
+          <t>Valide 193j (23/04/2027)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>194j</t>
+          <t>193j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Valide 380j (25/10/2027)</t>
+          <t>Valide 379j (25/10/2027)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>10/10/2026 13:24</t>
+          <t>11/10/2026 13:51</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 80j (29/12/2026)</t>
+          <t>Valide 79j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>80j</t>
+          <t>79j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 58j (07/12/2026)</t>
+          <t>Valide 57j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>10/10/2026 13:24</t>
+          <t>11/10/2026 13:51</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 80j (29/12/2026)</t>
+          <t>Valide 79j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>80j</t>
+          <t>79j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 58j (07/12/2026)</t>
+          <t>Valide 57j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>10/10/2026 13:24</t>
+          <t>11/10/2026 13:51</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2013,22 +2013,22 @@
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t>Valide 122j (09/02/2027)</t>
+          <t>Valide 121j (09/02/2027)</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>122j</t>
+          <t>121j</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
-          <t>Valide 41j (20/11/2026)</t>
+          <t>Valide 40j (20/11/2026)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>10/10/2026 13:24</t>
+          <t>11/10/2026 13:51</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
@@ -2075,22 +2075,22 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Valide 122j (09/02/2027)</t>
+          <t>Valide 121j (09/02/2027)</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>122j</t>
+          <t>121j</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Valide 41j (20/11/2026)</t>
+          <t>Valide 40j (20/11/2026)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>10/10/2026 13:24</t>
+          <t>11/10/2026 13:51</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
@@ -2285,22 +2285,22 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Valide 70j (19/12/2026)</t>
+          <t>Valide 69j (19/12/2026)</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>70j</t>
+          <t>69j</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>Valide 293j (31/07/2027)</t>
+          <t>Valide 292j (31/07/2027)</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>10/10/2026 13:24</t>
+          <t>11/10/2026 13:51</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
@@ -2339,22 +2339,22 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t>Valide 70j (19/12/2026)</t>
+          <t>Valide 69j (19/12/2026)</t>
         </is>
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>70j</t>
+          <t>69j</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
         <is>
-          <t>Valide 293j (31/07/2027)</t>
+          <t>Valide 292j (31/07/2027)</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>10/10/2026 13:24</t>
+          <t>11/10/2026 13:51</t>
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
@@ -2553,22 +2553,22 @@
       </c>
       <c r="L45" s="9" t="inlineStr">
         <is>
-          <t>Valide 194j (23/04/2027)</t>
+          <t>Valide 193j (23/04/2027)</t>
         </is>
       </c>
       <c r="M45" s="9" t="inlineStr">
         <is>
-          <t>194j</t>
+          <t>193j</t>
         </is>
       </c>
       <c r="N45" s="9" t="inlineStr">
         <is>
-          <t>Valide 364j (10/10/2027)</t>
+          <t>Valide 363j (10/10/2027)</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>10/10/2026 13:24</t>
+          <t>11/10/2026 13:51</t>
         </is>
       </c>
       <c r="P45" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 12/10/2026 16:39
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 53j (04/12/2026)</t>
+          <t>Valide 52j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>53j</t>
+          <t>52j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 144j (05/03/2027)</t>
+          <t>Valide 143j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>11/10/2026 13:51</t>
+          <t>12/10/2026 16:35</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 117j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>117j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 299j (07/08/2027)</t>
+          <t>Valide 298j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>11/10/2026 13:51</t>
+          <t>12/10/2026 16:35</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 82j (01/01/2027)</t>
+          <t>Valide 80j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>82j</t>
+          <t>80j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 106j (26/01/2027)</t>
+          <t>Valide 105j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>11/10/2026 13:51</t>
+          <t>12/10/2026 16:35</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 40j (20/11/2026)</t>
+          <t>Valide 39j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>40j</t>
+          <t>39j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 21j (02/11/2026)</t>
+          <t>Expire dans 20j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>11/10/2026 13:51</t>
+          <t>12/10/2026 16:35</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 121j (09/02/2027)</t>
+          <t>Valide 120j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>121j</t>
+          <t>120j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 139j (28/02/2027)</t>
+          <t>Valide 138j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>11/10/2026 13:51</t>
+          <t>12/10/2026 16:35</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 119j (07/02/2027)</t>
+          <t>Valide 117j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>119j</t>
+          <t>117j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 283j (22/07/2027)</t>
+          <t>Valide 282j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>11/10/2026 13:51</t>
+          <t>12/10/2026 16:35</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 193j (23/04/2027)</t>
+          <t>Valide 192j (23/04/2027)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>193j</t>
+          <t>192j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Valide 379j (25/10/2027)</t>
+          <t>Valide 378j (25/10/2027)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>11/10/2026 13:51</t>
+          <t>12/10/2026 16:35</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 79j (29/12/2026)</t>
+          <t>Valide 78j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>79j</t>
+          <t>78j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 57j (07/12/2026)</t>
+          <t>Valide 56j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>11/10/2026 13:51</t>
+          <t>12/10/2026 16:35</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 79j (29/12/2026)</t>
+          <t>Valide 78j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>79j</t>
+          <t>78j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 57j (07/12/2026)</t>
+          <t>Valide 56j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>11/10/2026 13:51</t>
+          <t>12/10/2026 16:35</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2013,22 +2013,22 @@
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t>Valide 121j (09/02/2027)</t>
+          <t>Valide 120j (09/02/2027)</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>121j</t>
+          <t>120j</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
-          <t>Valide 40j (20/11/2026)</t>
+          <t>Valide 38j (20/11/2026)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>11/10/2026 13:51</t>
+          <t>12/10/2026 16:35</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
@@ -2075,22 +2075,22 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Valide 121j (09/02/2027)</t>
+          <t>Valide 120j (09/02/2027)</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>121j</t>
+          <t>120j</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Valide 40j (20/11/2026)</t>
+          <t>Valide 38j (20/11/2026)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>11/10/2026 13:51</t>
+          <t>12/10/2026 16:35</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
@@ -2285,22 +2285,22 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Valide 69j (19/12/2026)</t>
+          <t>Valide 68j (19/12/2026)</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>69j</t>
+          <t>68j</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>Valide 292j (31/07/2027)</t>
+          <t>Valide 291j (31/07/2027)</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>11/10/2026 13:51</t>
+          <t>12/10/2026 16:35</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
@@ -2339,22 +2339,22 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t>Valide 69j (19/12/2026)</t>
+          <t>Valide 68j (19/12/2026)</t>
         </is>
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>69j</t>
+          <t>68j</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
         <is>
-          <t>Valide 292j (31/07/2027)</t>
+          <t>Valide 291j (31/07/2027)</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>11/10/2026 13:51</t>
+          <t>12/10/2026 16:35</t>
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
@@ -2553,22 +2553,22 @@
       </c>
       <c r="L45" s="9" t="inlineStr">
         <is>
-          <t>Valide 193j (23/04/2027)</t>
+          <t>Valide 192j (23/04/2027)</t>
         </is>
       </c>
       <c r="M45" s="9" t="inlineStr">
         <is>
-          <t>193j</t>
+          <t>192j</t>
         </is>
       </c>
       <c r="N45" s="9" t="inlineStr">
         <is>
-          <t>Valide 363j (10/10/2027)</t>
+          <t>Valide 362j (10/10/2027)</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>11/10/2026 13:51</t>
+          <t>12/10/2026 16:35</t>
         </is>
       </c>
       <c r="P45" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 13/10/2026 14:57
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 52j (04/12/2026)</t>
+          <t>Valide 51j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>52j</t>
+          <t>51j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 143j (05/03/2027)</t>
+          <t>Valide 142j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>12/10/2026 16:35</t>
+          <t>13/10/2026 14:52</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 117j (07/02/2027)</t>
+          <t>Valide 116j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>117j</t>
+          <t>116j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 298j (07/08/2027)</t>
+          <t>Valide 297j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>12/10/2026 16:35</t>
+          <t>13/10/2026 14:52</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1056,12 +1056,12 @@
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 105j (26/01/2027)</t>
+          <t>Valide 104j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>12/10/2026 16:35</t>
+          <t>13/10/2026 14:52</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 39j (20/11/2026)</t>
+          <t>Valide 38j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>39j</t>
+          <t>38j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 20j (02/11/2026)</t>
+          <t>Expire dans 19j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>12/10/2026 16:35</t>
+          <t>13/10/2026 14:52</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 120j (09/02/2027)</t>
+          <t>Valide 119j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>120j</t>
+          <t>119j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 138j (28/02/2027)</t>
+          <t>Valide 137j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>12/10/2026 16:35</t>
+          <t>13/10/2026 14:52</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 117j (07/02/2027)</t>
+          <t>Valide 116j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>117j</t>
+          <t>116j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 282j (22/07/2027)</t>
+          <t>Valide 281j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>12/10/2026 16:35</t>
+          <t>13/10/2026 14:52</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 192j (23/04/2027)</t>
+          <t>Valide 191j (23/04/2027)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>192j</t>
+          <t>191j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Valide 378j (25/10/2027)</t>
+          <t>Valide 377j (25/10/2027)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>12/10/2026 16:35</t>
+          <t>13/10/2026 14:52</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 78j (29/12/2026)</t>
+          <t>Valide 77j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>78j</t>
+          <t>77j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 56j (07/12/2026)</t>
+          <t>Valide 55j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>12/10/2026 16:35</t>
+          <t>13/10/2026 14:52</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 78j (29/12/2026)</t>
+          <t>Valide 77j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>78j</t>
+          <t>77j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 56j (07/12/2026)</t>
+          <t>Valide 55j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>12/10/2026 16:35</t>
+          <t>13/10/2026 14:52</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2013,22 +2013,22 @@
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t>Valide 120j (09/02/2027)</t>
+          <t>Valide 119j (09/02/2027)</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>120j</t>
+          <t>119j</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
-          <t>Valide 38j (20/11/2026)</t>
+          <t>Valide 37j (20/11/2026)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>12/10/2026 16:35</t>
+          <t>13/10/2026 14:52</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
@@ -2075,22 +2075,22 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Valide 120j (09/02/2027)</t>
+          <t>Valide 119j (09/02/2027)</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>120j</t>
+          <t>119j</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Valide 38j (20/11/2026)</t>
+          <t>Valide 37j (20/11/2026)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>12/10/2026 16:35</t>
+          <t>13/10/2026 14:52</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
@@ -2285,22 +2285,22 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Valide 68j (19/12/2026)</t>
+          <t>Valide 67j (19/12/2026)</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>68j</t>
+          <t>67j</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>Valide 291j (31/07/2027)</t>
+          <t>Valide 290j (31/07/2027)</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>12/10/2026 16:35</t>
+          <t>13/10/2026 14:52</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
@@ -2339,22 +2339,22 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t>Valide 68j (19/12/2026)</t>
+          <t>Valide 67j (19/12/2026)</t>
         </is>
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>68j</t>
+          <t>67j</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
         <is>
-          <t>Valide 291j (31/07/2027)</t>
+          <t>Valide 290j (31/07/2027)</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>12/10/2026 16:35</t>
+          <t>13/10/2026 14:52</t>
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
@@ -2553,22 +2553,22 @@
       </c>
       <c r="L45" s="9" t="inlineStr">
         <is>
-          <t>Valide 192j (23/04/2027)</t>
+          <t>Valide 191j (23/04/2027)</t>
         </is>
       </c>
       <c r="M45" s="9" t="inlineStr">
         <is>
-          <t>192j</t>
+          <t>191j</t>
         </is>
       </c>
       <c r="N45" s="9" t="inlineStr">
         <is>
-          <t>Valide 362j (10/10/2027)</t>
+          <t>Valide 361j (10/10/2027)</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>12/10/2026 16:35</t>
+          <t>13/10/2026 14:52</t>
         </is>
       </c>
       <c r="P45" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 14/10/2026 12:48
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 51j (04/12/2026)</t>
+          <t>Valide 50j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>51j</t>
+          <t>50j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 142j (05/03/2027)</t>
+          <t>Valide 141j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>13/10/2026 14:52</t>
+          <t>14/10/2026 12:43</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 116j (07/02/2027)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>116j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 297j (07/08/2027)</t>
+          <t>Valide 296j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>13/10/2026 14:52</t>
+          <t>14/10/2026 12:43</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 80j (01/01/2027)</t>
+          <t>Valide 79j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>80j</t>
+          <t>79j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 104j (26/01/2027)</t>
+          <t>Valide 103j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>13/10/2026 14:52</t>
+          <t>14/10/2026 12:43</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 38j (20/11/2026)</t>
+          <t>Valide 37j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>38j</t>
+          <t>37j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 19j (02/11/2026)</t>
+          <t>Expire dans 18j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>13/10/2026 14:52</t>
+          <t>14/10/2026 12:43</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 119j (09/02/2027)</t>
+          <t>Valide 118j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>119j</t>
+          <t>118j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 137j (28/02/2027)</t>
+          <t>Valide 136j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>13/10/2026 14:52</t>
+          <t>14/10/2026 12:43</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1590,12 +1590,12 @@
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 281j (22/07/2027)</t>
+          <t>Valide 280j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>13/10/2026 14:52</t>
+          <t>14/10/2026 12:43</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 191j (23/04/2027)</t>
+          <t>Valide 190j (23/04/2027)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>191j</t>
+          <t>190j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Valide 377j (25/10/2027)</t>
+          <t>Valide 376j (25/10/2027)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>13/10/2026 14:52</t>
+          <t>14/10/2026 12:43</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 77j (29/12/2026)</t>
+          <t>Valide 76j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>77j</t>
+          <t>76j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 55j (07/12/2026)</t>
+          <t>Valide 54j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>13/10/2026 14:52</t>
+          <t>14/10/2026 12:43</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 77j (29/12/2026)</t>
+          <t>Valide 76j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>77j</t>
+          <t>76j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 55j (07/12/2026)</t>
+          <t>Valide 54j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>13/10/2026 14:52</t>
+          <t>14/10/2026 12:43</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2013,12 +2013,12 @@
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t>Valide 119j (09/02/2027)</t>
+          <t>Valide 118j (09/02/2027)</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>119j</t>
+          <t>118j</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
@@ -2028,7 +2028,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>13/10/2026 14:52</t>
+          <t>14/10/2026 12:43</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
@@ -2075,12 +2075,12 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Valide 119j (09/02/2027)</t>
+          <t>Valide 118j (09/02/2027)</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>119j</t>
+          <t>118j</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
@@ -2090,7 +2090,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>13/10/2026 14:52</t>
+          <t>14/10/2026 12:43</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
@@ -2285,22 +2285,22 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Valide 67j (19/12/2026)</t>
+          <t>Valide 66j (19/12/2026)</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>67j</t>
+          <t>66j</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>Valide 290j (31/07/2027)</t>
+          <t>Valide 289j (31/07/2027)</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>13/10/2026 14:52</t>
+          <t>14/10/2026 12:43</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
@@ -2339,22 +2339,22 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t>Valide 67j (19/12/2026)</t>
+          <t>Valide 66j (19/12/2026)</t>
         </is>
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>67j</t>
+          <t>66j</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
         <is>
-          <t>Valide 290j (31/07/2027)</t>
+          <t>Valide 289j (31/07/2027)</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>13/10/2026 14:52</t>
+          <t>14/10/2026 12:43</t>
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
@@ -2553,12 +2553,12 @@
       </c>
       <c r="L45" s="9" t="inlineStr">
         <is>
-          <t>Valide 191j (23/04/2027)</t>
+          <t>Valide 190j (23/04/2027)</t>
         </is>
       </c>
       <c r="M45" s="9" t="inlineStr">
         <is>
-          <t>191j</t>
+          <t>190j</t>
         </is>
       </c>
       <c r="N45" s="9" t="inlineStr">
@@ -2568,7 +2568,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>13/10/2026 14:52</t>
+          <t>14/10/2026 12:43</t>
         </is>
       </c>
       <c r="P45" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 15/10/2026 12:36
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 50j (04/12/2026)</t>
+          <t>Valide 49j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>50j</t>
+          <t>49j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 141j (05/03/2027)</t>
+          <t>Valide 140j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>14/10/2026 12:43</t>
+          <t>15/10/2026 12:31</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 296j (07/08/2027)</t>
+          <t>Valide 295j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>14/10/2026 12:43</t>
+          <t>15/10/2026 12:31</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 79j (01/01/2027)</t>
+          <t>Valide 78j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>79j</t>
+          <t>78j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 103j (26/01/2027)</t>
+          <t>Valide 102j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>14/10/2026 12:43</t>
+          <t>15/10/2026 12:31</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 37j (20/11/2026)</t>
+          <t>Valide 36j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>37j</t>
+          <t>36j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 18j (02/11/2026)</t>
+          <t>Expire dans 17j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>14/10/2026 12:43</t>
+          <t>15/10/2026 12:31</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 118j (09/02/2027)</t>
+          <t>Valide 117j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>118j</t>
+          <t>117j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 136j (28/02/2027)</t>
+          <t>Valide 135j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>14/10/2026 12:43</t>
+          <t>15/10/2026 12:31</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 116j (07/02/2027)</t>
+          <t>Valide 115j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>116j</t>
+          <t>115j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 280j (22/07/2027)</t>
+          <t>Valide 279j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>14/10/2026 12:43</t>
+          <t>15/10/2026 12:31</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1660,12 +1660,12 @@
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Valide 376j (25/10/2027)</t>
+          <t>Valide 375j (25/10/2027)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>14/10/2026 12:43</t>
+          <t>15/10/2026 12:31</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 76j (29/12/2026)</t>
+          <t>Valide 75j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>76j</t>
+          <t>75j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 54j (07/12/2026)</t>
+          <t>Valide 53j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>14/10/2026 12:43</t>
+          <t>15/10/2026 12:31</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 76j (29/12/2026)</t>
+          <t>Valide 75j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>76j</t>
+          <t>75j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 54j (07/12/2026)</t>
+          <t>Valide 53j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>14/10/2026 12:43</t>
+          <t>15/10/2026 12:31</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2013,22 +2013,22 @@
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t>Valide 118j (09/02/2027)</t>
+          <t>Valide 117j (09/02/2027)</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>118j</t>
+          <t>117j</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
-          <t>Valide 37j (20/11/2026)</t>
+          <t>Valide 36j (20/11/2026)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>14/10/2026 12:43</t>
+          <t>15/10/2026 12:31</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
@@ -2075,22 +2075,22 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Valide 118j (09/02/2027)</t>
+          <t>Valide 117j (09/02/2027)</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>118j</t>
+          <t>117j</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Valide 37j (20/11/2026)</t>
+          <t>Valide 36j (20/11/2026)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>14/10/2026 12:43</t>
+          <t>15/10/2026 12:31</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
@@ -2285,22 +2285,22 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Valide 66j (19/12/2026)</t>
+          <t>Valide 65j (19/12/2026)</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>66j</t>
+          <t>65j</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>Valide 289j (31/07/2027)</t>
+          <t>Valide 288j (31/07/2027)</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>14/10/2026 12:43</t>
+          <t>15/10/2026 12:31</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
@@ -2339,22 +2339,22 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t>Valide 66j (19/12/2026)</t>
+          <t>Valide 65j (19/12/2026)</t>
         </is>
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>66j</t>
+          <t>65j</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
         <is>
-          <t>Valide 289j (31/07/2027)</t>
+          <t>Valide 288j (31/07/2027)</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>14/10/2026 12:43</t>
+          <t>15/10/2026 12:31</t>
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
@@ -2563,12 +2563,12 @@
       </c>
       <c r="N45" s="9" t="inlineStr">
         <is>
-          <t>Valide 361j (10/10/2027)</t>
+          <t>Valide 360j (10/10/2027)</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>14/10/2026 12:43</t>
+          <t>15/10/2026 12:31</t>
         </is>
       </c>
       <c r="P45" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 16/10/2026 12:15
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 49j (04/12/2026)</t>
+          <t>Valide 48j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>49j</t>
+          <t>48j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 140j (05/03/2027)</t>
+          <t>Valide 139j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>15/10/2026 12:31</t>
+          <t>16/10/2026 12:10</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 114j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>114j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 295j (07/08/2027)</t>
+          <t>Valide 294j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>15/10/2026 12:31</t>
+          <t>16/10/2026 12:10</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 78j (01/01/2027)</t>
+          <t>Valide 77j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>78j</t>
+          <t>77j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 102j (26/01/2027)</t>
+          <t>Valide 101j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>15/10/2026 12:31</t>
+          <t>16/10/2026 12:10</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,12 +1152,12 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 36j (20/11/2026)</t>
+          <t>Valide 35j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>36j</t>
+          <t>35j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>15/10/2026 12:31</t>
+          <t>16/10/2026 12:10</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 117j (09/02/2027)</t>
+          <t>Valide 116j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>117j</t>
+          <t>116j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 135j (28/02/2027)</t>
+          <t>Valide 134j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>15/10/2026 12:31</t>
+          <t>16/10/2026 12:10</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 115j (07/02/2027)</t>
+          <t>Valide 114j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>115j</t>
+          <t>114j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 279j (22/07/2027)</t>
+          <t>Valide 278j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>15/10/2026 12:31</t>
+          <t>16/10/2026 12:10</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 190j (23/04/2027)</t>
+          <t>Valide 189j (23/04/2027)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>190j</t>
+          <t>189j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Valide 375j (25/10/2027)</t>
+          <t>Valide 374j (25/10/2027)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>15/10/2026 12:31</t>
+          <t>16/10/2026 12:10</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 75j (29/12/2026)</t>
+          <t>Valide 74j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>75j</t>
+          <t>74j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 53j (07/12/2026)</t>
+          <t>Valide 52j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>15/10/2026 12:31</t>
+          <t>16/10/2026 12:10</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 75j (29/12/2026)</t>
+          <t>Valide 74j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>75j</t>
+          <t>74j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 53j (07/12/2026)</t>
+          <t>Valide 52j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>15/10/2026 12:31</t>
+          <t>16/10/2026 12:10</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2013,22 +2013,22 @@
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t>Valide 117j (09/02/2027)</t>
+          <t>Valide 116j (09/02/2027)</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>117j</t>
+          <t>116j</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
-          <t>Valide 36j (20/11/2026)</t>
+          <t>Valide 35j (20/11/2026)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>15/10/2026 12:31</t>
+          <t>16/10/2026 12:10</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
@@ -2075,22 +2075,22 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Valide 117j (09/02/2027)</t>
+          <t>Valide 116j (09/02/2027)</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>117j</t>
+          <t>116j</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Valide 36j (20/11/2026)</t>
+          <t>Valide 35j (20/11/2026)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>15/10/2026 12:31</t>
+          <t>16/10/2026 12:10</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
@@ -2285,22 +2285,22 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Valide 65j (19/12/2026)</t>
+          <t>Valide 64j (19/12/2026)</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>65j</t>
+          <t>64j</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>Valide 288j (31/07/2027)</t>
+          <t>Valide 287j (31/07/2027)</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>15/10/2026 12:31</t>
+          <t>16/10/2026 12:10</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
@@ -2339,22 +2339,22 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t>Valide 65j (19/12/2026)</t>
+          <t>Valide 64j (19/12/2026)</t>
         </is>
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>65j</t>
+          <t>64j</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
         <is>
-          <t>Valide 288j (31/07/2027)</t>
+          <t>Valide 287j (31/07/2027)</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>15/10/2026 12:31</t>
+          <t>16/10/2026 12:10</t>
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
@@ -2553,22 +2553,22 @@
       </c>
       <c r="L45" s="9" t="inlineStr">
         <is>
-          <t>Valide 190j (23/04/2027)</t>
+          <t>Valide 189j (23/04/2027)</t>
         </is>
       </c>
       <c r="M45" s="9" t="inlineStr">
         <is>
-          <t>190j</t>
+          <t>189j</t>
         </is>
       </c>
       <c r="N45" s="9" t="inlineStr">
         <is>
-          <t>Valide 360j (10/10/2027)</t>
+          <t>Valide 359j (10/10/2027)</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>15/10/2026 12:31</t>
+          <t>16/10/2026 12:10</t>
         </is>
       </c>
       <c r="P45" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 17/10/2026 11:33
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 48j (04/12/2026)</t>
+          <t>Valide 47j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>48j</t>
+          <t>47j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 139j (05/03/2027)</t>
+          <t>Valide 138j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>16/10/2026 12:10</t>
+          <t>17/10/2026 11:28</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 114j (07/02/2027)</t>
+          <t>Valide 113j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>114j</t>
+          <t>113j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 294j (07/08/2027)</t>
+          <t>Valide 293j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>16/10/2026 12:10</t>
+          <t>17/10/2026 11:28</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 77j (01/01/2027)</t>
+          <t>Valide 76j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>77j</t>
+          <t>76j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 101j (26/01/2027)</t>
+          <t>Valide 100j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>16/10/2026 12:10</t>
+          <t>17/10/2026 11:28</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 35j (20/11/2026)</t>
+          <t>Valide 34j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>35j</t>
+          <t>34j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 17j (02/11/2026)</t>
+          <t>Expire dans 16j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>16/10/2026 12:10</t>
+          <t>17/10/2026 11:28</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 116j (09/02/2027)</t>
+          <t>Valide 115j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>116j</t>
+          <t>115j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 134j (28/02/2027)</t>
+          <t>Valide 133j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>16/10/2026 12:10</t>
+          <t>17/10/2026 11:28</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 114j (07/02/2027)</t>
+          <t>Valide 113j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>114j</t>
+          <t>113j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 278j (22/07/2027)</t>
+          <t>Valide 277j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>16/10/2026 12:10</t>
+          <t>17/10/2026 11:28</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 189j (23/04/2027)</t>
+          <t>Valide 188j (23/04/2027)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>189j</t>
+          <t>188j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Valide 374j (25/10/2027)</t>
+          <t>Valide 373j (25/10/2027)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>16/10/2026 12:10</t>
+          <t>17/10/2026 11:28</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 74j (29/12/2026)</t>
+          <t>Valide 73j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>74j</t>
+          <t>73j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 52j (07/12/2026)</t>
+          <t>Valide 51j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>16/10/2026 12:10</t>
+          <t>17/10/2026 11:28</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 74j (29/12/2026)</t>
+          <t>Valide 73j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>74j</t>
+          <t>73j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 52j (07/12/2026)</t>
+          <t>Valide 51j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>16/10/2026 12:10</t>
+          <t>17/10/2026 11:28</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2013,22 +2013,22 @@
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t>Valide 116j (09/02/2027)</t>
+          <t>Valide 115j (09/02/2027)</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>116j</t>
+          <t>115j</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
-          <t>Valide 35j (20/11/2026)</t>
+          <t>Valide 399j (20/11/2027)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>16/10/2026 12:10</t>
+          <t>17/10/2026 11:28</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
@@ -2075,22 +2075,22 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Valide 116j (09/02/2027)</t>
+          <t>Valide 115j (09/02/2027)</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>116j</t>
+          <t>115j</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Valide 35j (20/11/2026)</t>
+          <t>Valide 399j (20/11/2027)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>16/10/2026 12:10</t>
+          <t>17/10/2026 11:28</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
@@ -2285,22 +2285,22 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Valide 64j (19/12/2026)</t>
+          <t>Valide 63j (19/12/2026)</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>64j</t>
+          <t>63j</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>Valide 287j (31/07/2027)</t>
+          <t>Valide 286j (31/07/2027)</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>16/10/2026 12:10</t>
+          <t>17/10/2026 11:28</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
@@ -2339,22 +2339,22 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t>Valide 64j (19/12/2026)</t>
+          <t>Valide 63j (19/12/2026)</t>
         </is>
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>64j</t>
+          <t>63j</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
         <is>
-          <t>Valide 287j (31/07/2027)</t>
+          <t>Valide 286j (31/07/2027)</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>16/10/2026 12:10</t>
+          <t>17/10/2026 11:28</t>
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
@@ -2553,22 +2553,22 @@
       </c>
       <c r="L45" s="9" t="inlineStr">
         <is>
-          <t>Valide 189j (23/04/2027)</t>
+          <t>Valide 188j (23/04/2027)</t>
         </is>
       </c>
       <c r="M45" s="9" t="inlineStr">
         <is>
-          <t>189j</t>
+          <t>188j</t>
         </is>
       </c>
       <c r="N45" s="9" t="inlineStr">
         <is>
-          <t>Valide 359j (10/10/2027)</t>
+          <t>Valide 358j (10/10/2027)</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>16/10/2026 12:10</t>
+          <t>17/10/2026 11:28</t>
         </is>
       </c>
       <c r="P45" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 18/10/2026 12:03
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 47j (04/12/2026)</t>
+          <t>Valide 46j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>47j</t>
+          <t>46j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 138j (05/03/2027)</t>
+          <t>Valide 137j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>17/10/2026 11:28</t>
+          <t>18/10/2026 11:58</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 113j (07/02/2027)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>113j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 293j (07/08/2027)</t>
+          <t>Valide 292j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>17/10/2026 11:28</t>
+          <t>18/10/2026 11:58</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 76j (01/01/2027)</t>
+          <t>Valide 75j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>76j</t>
+          <t>75j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 100j (26/01/2027)</t>
+          <t>Valide 99j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>17/10/2026 11:28</t>
+          <t>18/10/2026 11:58</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,25 +1152,29 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 34j (20/11/2026)</t>
+          <t>Valide 33j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>34j</t>
+          <t>33j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 16j (02/11/2026)</t>
+          <t>Expire dans 15j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>17/10/2026 11:28</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr"/>
+          <t>18/10/2026 11:58</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="11" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A11" s="3" t="inlineStr">
@@ -1258,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 115j (09/02/2027)</t>
+          <t>Valide 114j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>115j</t>
+          <t>114j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 133j (28/02/2027)</t>
+          <t>Valide 132j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>17/10/2026 11:28</t>
+          <t>18/10/2026 11:58</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1584,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 113j (07/02/2027)</t>
+          <t>Valide 112j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>113j</t>
+          <t>112j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 277j (22/07/2027)</t>
+          <t>Valide 276j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>17/10/2026 11:28</t>
+          <t>18/10/2026 11:58</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,22 +1654,22 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 188j (23/04/2027)</t>
+          <t>Valide 187j (23/04/2027)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>188j</t>
+          <t>187j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Valide 373j (25/10/2027)</t>
+          <t>Valide 372j (25/10/2027)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>17/10/2026 11:28</t>
+          <t>18/10/2026 11:58</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1749,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 73j (29/12/2026)</t>
+          <t>Valide 72j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>73j</t>
+          <t>72j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 51j (07/12/2026)</t>
+          <t>Valide 50j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>17/10/2026 11:28</t>
+          <t>18/10/2026 11:58</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1815,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 73j (29/12/2026)</t>
+          <t>Valide 72j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>73j</t>
+          <t>72j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 51j (07/12/2026)</t>
+          <t>Valide 50j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>17/10/2026 11:28</t>
+          <t>18/10/2026 11:58</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2013,22 +2017,22 @@
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t>Valide 115j (09/02/2027)</t>
+          <t>Valide 114j (09/02/2027)</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>115j</t>
+          <t>114j</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
-          <t>Valide 399j (20/11/2027)</t>
+          <t>Valide 398j (20/11/2027)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>17/10/2026 11:28</t>
+          <t>18/10/2026 11:58</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
@@ -2075,22 +2079,22 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Valide 115j (09/02/2027)</t>
+          <t>Valide 114j (09/02/2027)</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>115j</t>
+          <t>114j</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Valide 399j (20/11/2027)</t>
+          <t>Valide 398j (20/11/2027)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>17/10/2026 11:28</t>
+          <t>18/10/2026 11:58</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
@@ -2285,22 +2289,22 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Valide 63j (19/12/2026)</t>
+          <t>Valide 62j (19/12/2026)</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>63j</t>
+          <t>62j</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>Valide 286j (31/07/2027)</t>
+          <t>Valide 285j (31/07/2027)</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>17/10/2026 11:28</t>
+          <t>18/10/2026 11:58</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
@@ -2339,22 +2343,22 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t>Valide 63j (19/12/2026)</t>
+          <t>Valide 62j (19/12/2026)</t>
         </is>
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>63j</t>
+          <t>62j</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
         <is>
-          <t>Valide 286j (31/07/2027)</t>
+          <t>Valide 285j (31/07/2027)</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>17/10/2026 11:28</t>
+          <t>18/10/2026 11:58</t>
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
@@ -2553,22 +2557,22 @@
       </c>
       <c r="L45" s="9" t="inlineStr">
         <is>
-          <t>Valide 188j (23/04/2027)</t>
+          <t>Valide 187j (23/04/2027)</t>
         </is>
       </c>
       <c r="M45" s="9" t="inlineStr">
         <is>
-          <t>188j</t>
+          <t>187j</t>
         </is>
       </c>
       <c r="N45" s="9" t="inlineStr">
         <is>
-          <t>Valide 358j (10/10/2027)</t>
+          <t>Valide 357j (10/10/2027)</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>17/10/2026 11:28</t>
+          <t>18/10/2026 11:58</t>
         </is>
       </c>
       <c r="P45" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 19/10/2026 14:32
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 46j (04/12/2026)</t>
+          <t>Valide 45j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>46j</t>
+          <t>45j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 137j (05/03/2027)</t>
+          <t>Valide 136j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>18/10/2026 11:58</t>
+          <t>19/10/2026 14:27</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 110j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>110j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 292j (07/08/2027)</t>
+          <t>Valide 291j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>18/10/2026 11:58</t>
+          <t>19/10/2026 14:27</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 75j (01/01/2027)</t>
+          <t>Valide 74j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>75j</t>
+          <t>74j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 99j (26/01/2027)</t>
+          <t>Valide 98j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>18/10/2026 11:58</t>
+          <t>19/10/2026 14:27</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,29 +1152,25 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 33j (20/11/2026)</t>
+          <t>Valide 32j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>33j</t>
+          <t>32j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 15j (02/11/2026)</t>
+          <t>Expire dans 13j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>18/10/2026 11:58</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>19/10/2026 14:27</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A11" s="3" t="inlineStr">
@@ -1262,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 114j (09/02/2027)</t>
+          <t>Valide 113j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>114j</t>
+          <t>113j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 132j (28/02/2027)</t>
+          <t>Valide 131j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>18/10/2026 11:58</t>
+          <t>19/10/2026 14:27</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1584,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 112j (07/02/2027)</t>
+          <t>Valide 110j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>112j</t>
+          <t>110j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 276j (22/07/2027)</t>
+          <t>Valide 275j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>18/10/2026 11:58</t>
+          <t>19/10/2026 14:27</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1654,22 +1650,22 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 187j (23/04/2027)</t>
+          <t>Valide 185j (23/04/2027)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>187j</t>
+          <t>185j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Valide 372j (25/10/2027)</t>
+          <t>Valide 371j (25/10/2027)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>18/10/2026 11:58</t>
+          <t>19/10/2026 14:27</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1749,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 72j (29/12/2026)</t>
+          <t>Valide 71j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>72j</t>
+          <t>71j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 50j (07/12/2026)</t>
+          <t>Valide 49j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>18/10/2026 11:58</t>
+          <t>19/10/2026 14:27</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1815,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 72j (29/12/2026)</t>
+          <t>Valide 71j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>72j</t>
+          <t>71j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 50j (07/12/2026)</t>
+          <t>Valide 49j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>18/10/2026 11:58</t>
+          <t>19/10/2026 14:27</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2017,22 +2013,22 @@
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t>Valide 114j (09/02/2027)</t>
+          <t>Valide 113j (09/02/2027)</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>114j</t>
+          <t>113j</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
-          <t>Valide 398j (20/11/2027)</t>
+          <t>Valide 397j (20/11/2027)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>18/10/2026 11:58</t>
+          <t>19/10/2026 14:27</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
@@ -2079,22 +2075,22 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Valide 114j (09/02/2027)</t>
+          <t>Valide 113j (09/02/2027)</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>114j</t>
+          <t>113j</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Valide 398j (20/11/2027)</t>
+          <t>Valide 397j (20/11/2027)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>18/10/2026 11:58</t>
+          <t>19/10/2026 14:27</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
@@ -2289,22 +2285,22 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Valide 62j (19/12/2026)</t>
+          <t>Valide 61j (19/12/2026)</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>62j</t>
+          <t>61j</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>Valide 285j (31/07/2027)</t>
+          <t>Valide 284j (31/07/2027)</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>18/10/2026 11:58</t>
+          <t>19/10/2026 14:27</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
@@ -2343,22 +2339,22 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t>Valide 62j (19/12/2026)</t>
+          <t>Valide 61j (19/12/2026)</t>
         </is>
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>62j</t>
+          <t>61j</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
         <is>
-          <t>Valide 285j (31/07/2027)</t>
+          <t>Valide 284j (31/07/2027)</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>18/10/2026 11:58</t>
+          <t>19/10/2026 14:27</t>
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
@@ -2557,22 +2553,22 @@
       </c>
       <c r="L45" s="9" t="inlineStr">
         <is>
-          <t>Valide 187j (23/04/2027)</t>
+          <t>Valide 185j (23/04/2027)</t>
         </is>
       </c>
       <c r="M45" s="9" t="inlineStr">
         <is>
-          <t>187j</t>
+          <t>185j</t>
         </is>
       </c>
       <c r="N45" s="9" t="inlineStr">
         <is>
-          <t>Valide 357j (10/10/2027)</t>
+          <t>Valide 355j (10/10/2027)</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>18/10/2026 11:58</t>
+          <t>19/10/2026 14:27</t>
         </is>
       </c>
       <c r="P45" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 20/10/2026 12:40
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 45j (04/12/2026)</t>
+          <t>Valide 44j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>45j</t>
+          <t>44j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 136j (05/03/2027)</t>
+          <t>Valide 135j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>19/10/2026 14:27</t>
+          <t>20/10/2026 12:36</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 291j (07/08/2027)</t>
+          <t>Valide 290j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>19/10/2026 14:27</t>
+          <t>20/10/2026 12:36</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 74j (01/01/2027)</t>
+          <t>Valide 73j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>74j</t>
+          <t>73j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 98j (26/01/2027)</t>
+          <t>Valide 97j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>19/10/2026 14:27</t>
+          <t>20/10/2026 12:36</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 32j (20/11/2026)</t>
+          <t>Valide 31j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>32j</t>
+          <t>31j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 13j (02/11/2026)</t>
+          <t>Expire dans 12j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>19/10/2026 14:27</t>
+          <t>20/10/2026 12:36</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 113j (09/02/2027)</t>
+          <t>Valide 112j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>113j</t>
+          <t>112j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 131j (28/02/2027)</t>
+          <t>Valide 130j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>19/10/2026 14:27</t>
+          <t>20/10/2026 12:36</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1590,12 +1590,12 @@
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 275j (22/07/2027)</t>
+          <t>Valide 274j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>19/10/2026 14:27</t>
+          <t>20/10/2026 12:36</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1660,12 +1660,12 @@
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Valide 371j (25/10/2027)</t>
+          <t>Valide 370j (25/10/2027)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>19/10/2026 14:27</t>
+          <t>20/10/2026 12:36</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 71j (29/12/2026)</t>
+          <t>Valide 70j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>71j</t>
+          <t>70j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 49j (07/12/2026)</t>
+          <t>Valide 48j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>19/10/2026 14:27</t>
+          <t>20/10/2026 12:36</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 71j (29/12/2026)</t>
+          <t>Valide 70j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>71j</t>
+          <t>70j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 49j (07/12/2026)</t>
+          <t>Valide 48j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>19/10/2026 14:27</t>
+          <t>20/10/2026 12:36</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2013,22 +2013,22 @@
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t>Valide 113j (09/02/2027)</t>
+          <t>Valide 112j (09/02/2027)</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>113j</t>
+          <t>112j</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
-          <t>Valide 397j (20/11/2027)</t>
+          <t>Valide 396j (20/11/2027)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>19/10/2026 14:27</t>
+          <t>20/10/2026 12:36</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
@@ -2075,22 +2075,22 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Valide 113j (09/02/2027)</t>
+          <t>Valide 112j (09/02/2027)</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>113j</t>
+          <t>112j</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Valide 397j (20/11/2027)</t>
+          <t>Valide 396j (20/11/2027)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>19/10/2026 14:27</t>
+          <t>20/10/2026 12:36</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
@@ -2285,22 +2285,22 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Valide 61j (19/12/2026)</t>
+          <t>Valide 60j (19/12/2026)</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>61j</t>
+          <t>60j</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>Valide 284j (31/07/2027)</t>
+          <t>Valide 283j (31/07/2027)</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>19/10/2026 14:27</t>
+          <t>20/10/2026 12:36</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
@@ -2339,22 +2339,22 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t>Valide 61j (19/12/2026)</t>
+          <t>Valide 60j (19/12/2026)</t>
         </is>
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>61j</t>
+          <t>60j</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
         <is>
-          <t>Valide 284j (31/07/2027)</t>
+          <t>Valide 283j (31/07/2027)</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>19/10/2026 14:27</t>
+          <t>20/10/2026 12:36</t>
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
@@ -2568,7 +2568,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>19/10/2026 14:27</t>
+          <t>20/10/2026 12:36</t>
         </is>
       </c>
       <c r="P45" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 21/10/2026 12:52
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 44j (04/12/2026)</t>
+          <t>Valide 43j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>44j</t>
+          <t>43j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 135j (05/03/2027)</t>
+          <t>Valide 134j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>20/10/2026 12:36</t>
+          <t>21/10/2026 12:47</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 110j (07/02/2027)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>110j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 290j (07/08/2027)</t>
+          <t>Valide 289j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>20/10/2026 12:36</t>
+          <t>21/10/2026 12:47</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 73j (01/01/2027)</t>
+          <t>Valide 72j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>73j</t>
+          <t>72j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 97j (26/01/2027)</t>
+          <t>Valide 96j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>20/10/2026 12:36</t>
+          <t>21/10/2026 12:47</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,25 +1152,29 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 31j (20/11/2026)</t>
+          <t>Expire dans 30j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>31j</t>
+          <t>30j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 12j (02/11/2026)</t>
+          <t>Expire dans 11j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>20/10/2026 12:36</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr"/>
+          <t>21/10/2026 12:47</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="11" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A11" s="3" t="inlineStr">
@@ -1258,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 112j (09/02/2027)</t>
+          <t>Valide 111j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>112j</t>
+          <t>111j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 130j (28/02/2027)</t>
+          <t>Valide 129j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>20/10/2026 12:36</t>
+          <t>21/10/2026 12:47</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1584,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 110j (07/02/2027)</t>
+          <t>Valide 109j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>110j</t>
+          <t>109j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 274j (22/07/2027)</t>
+          <t>Valide 273j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>20/10/2026 12:36</t>
+          <t>21/10/2026 12:47</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,22 +1654,22 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 185j (23/04/2027)</t>
+          <t>Valide 183j (23/04/2027)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>185j</t>
+          <t>183j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Valide 370j (25/10/2027)</t>
+          <t>Valide 369j (25/10/2027)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>20/10/2026 12:36</t>
+          <t>21/10/2026 12:47</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1749,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 70j (29/12/2026)</t>
+          <t>Valide 69j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>70j</t>
+          <t>69j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 48j (07/12/2026)</t>
+          <t>Valide 47j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>20/10/2026 12:36</t>
+          <t>21/10/2026 12:47</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1815,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 70j (29/12/2026)</t>
+          <t>Valide 69j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>70j</t>
+          <t>69j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 48j (07/12/2026)</t>
+          <t>Valide 47j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>20/10/2026 12:36</t>
+          <t>21/10/2026 12:47</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2013,22 +2017,22 @@
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t>Valide 112j (09/02/2027)</t>
+          <t>Valide 111j (09/02/2027)</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>112j</t>
+          <t>111j</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
-          <t>Valide 396j (20/11/2027)</t>
+          <t>Valide 395j (20/11/2027)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>20/10/2026 12:36</t>
+          <t>21/10/2026 12:47</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
@@ -2075,22 +2079,22 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Valide 112j (09/02/2027)</t>
+          <t>Valide 111j (09/02/2027)</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>112j</t>
+          <t>111j</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Valide 396j (20/11/2027)</t>
+          <t>Valide 395j (20/11/2027)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>20/10/2026 12:36</t>
+          <t>21/10/2026 12:47</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
@@ -2285,22 +2289,22 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Valide 60j (19/12/2026)</t>
+          <t>Valide 59j (19/12/2026)</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>60j</t>
+          <t>59j</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>Valide 283j (31/07/2027)</t>
+          <t>Valide 282j (31/07/2027)</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>20/10/2026 12:36</t>
+          <t>21/10/2026 12:47</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
@@ -2339,22 +2343,22 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t>Valide 60j (19/12/2026)</t>
+          <t>Valide 59j (19/12/2026)</t>
         </is>
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>60j</t>
+          <t>59j</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
         <is>
-          <t>Valide 283j (31/07/2027)</t>
+          <t>Valide 282j (31/07/2027)</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>20/10/2026 12:36</t>
+          <t>21/10/2026 12:47</t>
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
@@ -2553,22 +2557,22 @@
       </c>
       <c r="L45" s="9" t="inlineStr">
         <is>
-          <t>Valide 185j (23/04/2027)</t>
+          <t>Valide 183j (23/04/2027)</t>
         </is>
       </c>
       <c r="M45" s="9" t="inlineStr">
         <is>
-          <t>185j</t>
+          <t>183j</t>
         </is>
       </c>
       <c r="N45" s="9" t="inlineStr">
         <is>
-          <t>Valide 355j (10/10/2027)</t>
+          <t>Valide 354j (10/10/2027)</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>20/10/2026 12:36</t>
+          <t>21/10/2026 12:47</t>
         </is>
       </c>
       <c r="P45" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 22/10/2026 12:55
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 43j (04/12/2026)</t>
+          <t>Valide 42j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>43j</t>
+          <t>42j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 134j (05/03/2027)</t>
+          <t>Valide 133j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>21/10/2026 12:47</t>
+          <t>22/10/2026 12:50</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 289j (07/08/2027)</t>
+          <t>Valide 288j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>21/10/2026 12:47</t>
+          <t>22/10/2026 12:50</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 72j (01/01/2027)</t>
+          <t>Valide 71j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>72j</t>
+          <t>71j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 96j (26/01/2027)</t>
+          <t>Valide 95j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>21/10/2026 12:47</t>
+          <t>22/10/2026 12:50</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,29 +1152,25 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 30j (20/11/2026)</t>
+          <t>Valide 197j (07/05/2027)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>30j</t>
+          <t>197j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 11j (02/11/2026)</t>
+          <t>Expire dans 10j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>21/10/2026 12:47</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>22/10/2026 12:50</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A11" s="3" t="inlineStr">
@@ -1262,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 111j (09/02/2027)</t>
+          <t>Valide 110j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>111j</t>
+          <t>110j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 129j (28/02/2027)</t>
+          <t>Valide 128j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>21/10/2026 12:47</t>
+          <t>22/10/2026 12:50</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1584,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 109j (07/02/2027)</t>
+          <t>Valide 108j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>109j</t>
+          <t>108j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 273j (22/07/2027)</t>
+          <t>Valide 272j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>21/10/2026 12:47</t>
+          <t>22/10/2026 12:50</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1654,22 +1650,22 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 183j (23/04/2027)</t>
+          <t>Valide 182j (23/04/2027)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>183j</t>
+          <t>182j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Valide 369j (25/10/2027)</t>
+          <t>Valide 368j (25/10/2027)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>21/10/2026 12:47</t>
+          <t>22/10/2026 12:50</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1749,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 69j (29/12/2026)</t>
+          <t>Valide 68j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>69j</t>
+          <t>68j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 47j (07/12/2026)</t>
+          <t>Valide 46j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>21/10/2026 12:47</t>
+          <t>22/10/2026 12:50</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1815,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 69j (29/12/2026)</t>
+          <t>Valide 68j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>69j</t>
+          <t>68j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 47j (07/12/2026)</t>
+          <t>Valide 46j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>21/10/2026 12:47</t>
+          <t>22/10/2026 12:50</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2017,22 +2013,22 @@
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t>Valide 111j (09/02/2027)</t>
+          <t>Valide 110j (09/02/2027)</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>111j</t>
+          <t>110j</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
-          <t>Valide 395j (20/11/2027)</t>
+          <t>Valide 394j (20/11/2027)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>21/10/2026 12:47</t>
+          <t>22/10/2026 12:50</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
@@ -2079,22 +2075,22 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Valide 111j (09/02/2027)</t>
+          <t>Valide 110j (09/02/2027)</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>111j</t>
+          <t>110j</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Valide 395j (20/11/2027)</t>
+          <t>Valide 394j (20/11/2027)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>21/10/2026 12:47</t>
+          <t>22/10/2026 12:50</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
@@ -2289,22 +2285,22 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Valide 59j (19/12/2026)</t>
+          <t>Valide 58j (19/12/2026)</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>59j</t>
+          <t>58j</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>Valide 282j (31/07/2027)</t>
+          <t>Valide 281j (31/07/2027)</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>21/10/2026 12:47</t>
+          <t>22/10/2026 12:50</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
@@ -2343,22 +2339,22 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t>Valide 59j (19/12/2026)</t>
+          <t>Valide 58j (19/12/2026)</t>
         </is>
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>59j</t>
+          <t>58j</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
         <is>
-          <t>Valide 282j (31/07/2027)</t>
+          <t>Valide 281j (31/07/2027)</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>21/10/2026 12:47</t>
+          <t>22/10/2026 12:50</t>
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
@@ -2557,22 +2553,22 @@
       </c>
       <c r="L45" s="9" t="inlineStr">
         <is>
-          <t>Valide 183j (23/04/2027)</t>
+          <t>Valide 182j (23/04/2027)</t>
         </is>
       </c>
       <c r="M45" s="9" t="inlineStr">
         <is>
-          <t>183j</t>
+          <t>182j</t>
         </is>
       </c>
       <c r="N45" s="9" t="inlineStr">
         <is>
-          <t>Valide 354j (10/10/2027)</t>
+          <t>Valide 353j (10/10/2027)</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>21/10/2026 12:47</t>
+          <t>22/10/2026 12:50</t>
         </is>
       </c>
       <c r="P45" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 23/10/2026 12:34
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 42j (04/12/2026)</t>
+          <t>Valide 41j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>42j</t>
+          <t>41j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 133j (05/03/2027)</t>
+          <t>Valide 132j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>22/10/2026 12:50</t>
+          <t>23/10/2026 12:29</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 288j (07/08/2027)</t>
+          <t>Valide 287j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>22/10/2026 12:50</t>
+          <t>23/10/2026 12:29</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 71j (01/01/2027)</t>
+          <t>Valide 70j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>71j</t>
+          <t>70j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 95j (26/01/2027)</t>
+          <t>Valide 94j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>22/10/2026 12:50</t>
+          <t>23/10/2026 12:29</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 197j (07/05/2027)</t>
+          <t>Valide 196j (07/05/2027)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>197j</t>
+          <t>196j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 10j (02/11/2026)</t>
+          <t>Expire dans 9j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>22/10/2026 12:50</t>
+          <t>23/10/2026 12:29</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 110j (09/02/2027)</t>
+          <t>Valide 109j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>110j</t>
+          <t>109j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 128j (28/02/2027)</t>
+          <t>Valide 127j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>22/10/2026 12:50</t>
+          <t>23/10/2026 12:29</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 108j (07/02/2027)</t>
+          <t>Valide 107j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>108j</t>
+          <t>107j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 272j (22/07/2027)</t>
+          <t>Valide 271j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>22/10/2026 12:50</t>
+          <t>23/10/2026 12:29</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1660,12 +1660,12 @@
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Valide 368j (25/10/2027)</t>
+          <t>Valide 367j (25/10/2027)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>22/10/2026 12:50</t>
+          <t>23/10/2026 12:29</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 68j (29/12/2026)</t>
+          <t>Valide 67j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>68j</t>
+          <t>67j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 46j (07/12/2026)</t>
+          <t>Valide 45j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>22/10/2026 12:50</t>
+          <t>23/10/2026 12:29</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 68j (29/12/2026)</t>
+          <t>Valide 67j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>68j</t>
+          <t>67j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 46j (07/12/2026)</t>
+          <t>Valide 45j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>22/10/2026 12:50</t>
+          <t>23/10/2026 12:29</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2013,22 +2013,22 @@
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t>Valide 110j (09/02/2027)</t>
+          <t>Valide 109j (09/02/2027)</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>110j</t>
+          <t>109j</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
-          <t>Valide 394j (20/11/2027)</t>
+          <t>Valide 393j (20/11/2027)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>22/10/2026 12:50</t>
+          <t>23/10/2026 12:29</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
@@ -2075,22 +2075,22 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Valide 110j (09/02/2027)</t>
+          <t>Valide 109j (09/02/2027)</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>110j</t>
+          <t>109j</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Valide 394j (20/11/2027)</t>
+          <t>Valide 393j (20/11/2027)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>22/10/2026 12:50</t>
+          <t>23/10/2026 12:29</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
@@ -2285,22 +2285,22 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Valide 58j (19/12/2026)</t>
+          <t>Valide 57j (19/12/2026)</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>58j</t>
+          <t>57j</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>Valide 281j (31/07/2027)</t>
+          <t>Valide 280j (31/07/2027)</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>22/10/2026 12:50</t>
+          <t>23/10/2026 12:29</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
@@ -2339,22 +2339,22 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t>Valide 58j (19/12/2026)</t>
+          <t>Valide 57j (19/12/2026)</t>
         </is>
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>58j</t>
+          <t>57j</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
         <is>
-          <t>Valide 281j (31/07/2027)</t>
+          <t>Valide 280j (31/07/2027)</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>22/10/2026 12:50</t>
+          <t>23/10/2026 12:29</t>
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
@@ -2563,12 +2563,12 @@
       </c>
       <c r="N45" s="9" t="inlineStr">
         <is>
-          <t>Valide 353j (10/10/2027)</t>
+          <t>Valide 352j (10/10/2027)</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>22/10/2026 12:50</t>
+          <t>23/10/2026 12:29</t>
         </is>
       </c>
       <c r="P45" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 24/10/2026 11:58
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 41j (04/12/2026)</t>
+          <t>Valide 40j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>41j</t>
+          <t>40j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 132j (05/03/2027)</t>
+          <t>Valide 131j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>23/10/2026 12:29</t>
+          <t>24/10/2026 11:53</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 106j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>106j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 287j (07/08/2027)</t>
+          <t>Valide 286j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>23/10/2026 12:29</t>
+          <t>24/10/2026 11:53</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 70j (01/01/2027)</t>
+          <t>Valide 69j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>70j</t>
+          <t>69j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 94j (26/01/2027)</t>
+          <t>Valide 93j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>23/10/2026 12:29</t>
+          <t>24/10/2026 11:53</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,12 +1152,12 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 196j (07/05/2027)</t>
+          <t>Valide 195j (07/05/2027)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>196j</t>
+          <t>195j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>23/10/2026 12:29</t>
+          <t>24/10/2026 11:53</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 109j (09/02/2027)</t>
+          <t>Valide 108j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>109j</t>
+          <t>108j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 127j (28/02/2027)</t>
+          <t>Valide 126j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>23/10/2026 12:29</t>
+          <t>24/10/2026 11:53</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 107j (07/02/2027)</t>
+          <t>Valide 106j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>107j</t>
+          <t>106j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 271j (22/07/2027)</t>
+          <t>Valide 270j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>23/10/2026 12:29</t>
+          <t>24/10/2026 11:53</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 182j (23/04/2027)</t>
+          <t>Valide 181j (23/04/2027)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>182j</t>
+          <t>181j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Valide 367j (25/10/2027)</t>
+          <t>Valide 366j (25/10/2027)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>23/10/2026 12:29</t>
+          <t>24/10/2026 11:53</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 67j (29/12/2026)</t>
+          <t>Valide 66j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>67j</t>
+          <t>66j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 45j (07/12/2026)</t>
+          <t>Valide 44j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>23/10/2026 12:29</t>
+          <t>24/10/2026 11:53</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 67j (29/12/2026)</t>
+          <t>Valide 66j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>67j</t>
+          <t>66j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 45j (07/12/2026)</t>
+          <t>Valide 44j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>23/10/2026 12:29</t>
+          <t>24/10/2026 11:53</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2013,22 +2013,22 @@
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t>Valide 109j (09/02/2027)</t>
+          <t>Valide 108j (09/02/2027)</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>109j</t>
+          <t>108j</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
-          <t>Valide 393j (20/11/2027)</t>
+          <t>Valide 392j (20/11/2027)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>23/10/2026 12:29</t>
+          <t>24/10/2026 11:53</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
@@ -2075,22 +2075,22 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Valide 109j (09/02/2027)</t>
+          <t>Valide 108j (09/02/2027)</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>109j</t>
+          <t>108j</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Valide 393j (20/11/2027)</t>
+          <t>Valide 392j (20/11/2027)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>23/10/2026 12:29</t>
+          <t>24/10/2026 11:53</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
@@ -2285,22 +2285,22 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Valide 57j (19/12/2026)</t>
+          <t>Valide 56j (19/12/2026)</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>57j</t>
+          <t>56j</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>Valide 280j (31/07/2027)</t>
+          <t>Valide 279j (31/07/2027)</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>23/10/2026 12:29</t>
+          <t>24/10/2026 11:53</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
@@ -2339,22 +2339,22 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t>Valide 57j (19/12/2026)</t>
+          <t>Valide 56j (19/12/2026)</t>
         </is>
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>57j</t>
+          <t>56j</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
         <is>
-          <t>Valide 280j (31/07/2027)</t>
+          <t>Valide 279j (31/07/2027)</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>23/10/2026 12:29</t>
+          <t>24/10/2026 11:53</t>
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
@@ -2553,22 +2553,22 @@
       </c>
       <c r="L45" s="9" t="inlineStr">
         <is>
-          <t>Valide 182j (23/04/2027)</t>
+          <t>Valide 181j (23/04/2027)</t>
         </is>
       </c>
       <c r="M45" s="9" t="inlineStr">
         <is>
-          <t>182j</t>
+          <t>181j</t>
         </is>
       </c>
       <c r="N45" s="9" t="inlineStr">
         <is>
-          <t>Valide 352j (10/10/2027)</t>
+          <t>Valide 351j (10/10/2027)</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>23/10/2026 12:29</t>
+          <t>24/10/2026 11:53</t>
         </is>
       </c>
       <c r="P45" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 25/10/2026 12:29
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 40j (04/12/2026)</t>
+          <t>Valide 39j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>40j</t>
+          <t>39j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 131j (05/03/2027)</t>
+          <t>Valide 130j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>24/10/2026 11:53</t>
+          <t>25/10/2026 12:24</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 106j (07/02/2027)</t>
+          <t>Valide 105j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>106j</t>
+          <t>105j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 286j (07/08/2027)</t>
+          <t>Valide 285j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>24/10/2026 11:53</t>
+          <t>25/10/2026 12:24</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 69j (01/01/2027)</t>
+          <t>Valide 68j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>69j</t>
+          <t>68j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 93j (26/01/2027)</t>
+          <t>Valide 92j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>24/10/2026 11:53</t>
+          <t>25/10/2026 12:24</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,25 +1152,29 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 195j (07/05/2027)</t>
+          <t>Valide 194j (07/05/2027)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>195j</t>
+          <t>194j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 9j (02/11/2026)</t>
+          <t>Expire dans 7j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>24/10/2026 11:53</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr"/>
+          <t>25/10/2026 12:24</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="11" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A11" s="3" t="inlineStr">
@@ -1258,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 108j (09/02/2027)</t>
+          <t>Valide 107j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>108j</t>
+          <t>107j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 126j (28/02/2027)</t>
+          <t>Valide 125j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>24/10/2026 11:53</t>
+          <t>25/10/2026 12:24</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1584,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 106j (07/02/2027)</t>
+          <t>Valide 105j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>106j</t>
+          <t>105j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 270j (22/07/2027)</t>
+          <t>Valide 269j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>24/10/2026 11:53</t>
+          <t>25/10/2026 12:24</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,22 +1654,22 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 181j (23/04/2027)</t>
+          <t>Valide 180j (23/04/2027)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>181j</t>
+          <t>180j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Valide 366j (25/10/2027)</t>
+          <t>Valide 365j (25/10/2027)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>24/10/2026 11:53</t>
+          <t>25/10/2026 12:24</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1749,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 66j (29/12/2026)</t>
+          <t>Valide 65j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>66j</t>
+          <t>65j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 44j (07/12/2026)</t>
+          <t>Valide 43j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>24/10/2026 11:53</t>
+          <t>25/10/2026 12:24</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1815,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 66j (29/12/2026)</t>
+          <t>Valide 65j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>66j</t>
+          <t>65j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 44j (07/12/2026)</t>
+          <t>Valide 43j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>24/10/2026 11:53</t>
+          <t>25/10/2026 12:24</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2013,22 +2017,22 @@
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t>Valide 108j (09/02/2027)</t>
+          <t>Valide 107j (09/02/2027)</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>108j</t>
+          <t>107j</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
-          <t>Valide 392j (20/11/2027)</t>
+          <t>Valide 391j (20/11/2027)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>24/10/2026 11:53</t>
+          <t>25/10/2026 12:24</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
@@ -2075,22 +2079,22 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Valide 108j (09/02/2027)</t>
+          <t>Valide 107j (09/02/2027)</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>108j</t>
+          <t>107j</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Valide 392j (20/11/2027)</t>
+          <t>Valide 391j (20/11/2027)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>24/10/2026 11:53</t>
+          <t>25/10/2026 12:24</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
@@ -2285,22 +2289,22 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Valide 56j (19/12/2026)</t>
+          <t>Valide 55j (19/12/2026)</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>56j</t>
+          <t>55j</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>Valide 279j (31/07/2027)</t>
+          <t>Valide 278j (31/07/2027)</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>24/10/2026 11:53</t>
+          <t>25/10/2026 12:24</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
@@ -2339,22 +2343,22 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t>Valide 56j (19/12/2026)</t>
+          <t>Valide 55j (19/12/2026)</t>
         </is>
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>56j</t>
+          <t>55j</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
         <is>
-          <t>Valide 279j (31/07/2027)</t>
+          <t>Valide 278j (31/07/2027)</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>24/10/2026 11:53</t>
+          <t>25/10/2026 12:24</t>
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
@@ -2553,22 +2557,22 @@
       </c>
       <c r="L45" s="9" t="inlineStr">
         <is>
-          <t>Valide 181j (23/04/2027)</t>
+          <t>Valide 180j (23/04/2027)</t>
         </is>
       </c>
       <c r="M45" s="9" t="inlineStr">
         <is>
-          <t>181j</t>
+          <t>180j</t>
         </is>
       </c>
       <c r="N45" s="9" t="inlineStr">
         <is>
-          <t>Valide 351j (10/10/2027)</t>
+          <t>Valide 350j (10/10/2027)</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>24/10/2026 11:53</t>
+          <t>25/10/2026 12:24</t>
         </is>
       </c>
       <c r="P45" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 26/10/2026 14:05
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 39j (04/12/2026)</t>
+          <t>Valide 38j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>39j</t>
+          <t>38j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 130j (05/03/2027)</t>
+          <t>Valide 129j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>25/10/2026 12:24</t>
+          <t>26/10/2026 14:01</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 105j (07/02/2027)</t>
+          <t>Valide 104j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>105j</t>
+          <t>104j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 285j (07/08/2027)</t>
+          <t>Valide 284j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>25/10/2026 12:24</t>
+          <t>26/10/2026 14:01</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 68j (01/01/2027)</t>
+          <t>Valide 67j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>68j</t>
+          <t>67j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 92j (26/01/2027)</t>
+          <t>Valide 91j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>25/10/2026 12:24</t>
+          <t>26/10/2026 14:01</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 194j (07/05/2027)</t>
+          <t>Valide 193j (07/05/2027)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>194j</t>
+          <t>193j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 7j (02/11/2026)</t>
+          <t>Expire dans 6j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>25/10/2026 12:24</t>
+          <t>26/10/2026 14:01</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1262,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 107j (09/02/2027)</t>
+          <t>Valide 106j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>107j</t>
+          <t>106j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 125j (28/02/2027)</t>
+          <t>Valide 124j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>25/10/2026 12:24</t>
+          <t>26/10/2026 14:01</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1584,22 +1584,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 105j (07/02/2027)</t>
+          <t>Valide 104j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>105j</t>
+          <t>104j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 269j (22/07/2027)</t>
+          <t>Valide 268j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>25/10/2026 12:24</t>
+          <t>26/10/2026 14:01</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1654,22 +1654,22 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 180j (23/04/2027)</t>
+          <t>Valide 178j (23/04/2027)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>180j</t>
+          <t>178j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Valide 365j (25/10/2027)</t>
+          <t>Valide 364j (25/10/2027)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>25/10/2026 12:24</t>
+          <t>26/10/2026 14:01</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1749,22 +1749,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 65j (29/12/2026)</t>
+          <t>Valide 64j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>65j</t>
+          <t>64j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 43j (07/12/2026)</t>
+          <t>Valide 42j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>25/10/2026 12:24</t>
+          <t>26/10/2026 14:01</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 65j (29/12/2026)</t>
+          <t>Valide 64j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>65j</t>
+          <t>64j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 43j (07/12/2026)</t>
+          <t>Valide 42j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>25/10/2026 12:24</t>
+          <t>26/10/2026 14:01</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2017,22 +2017,22 @@
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t>Valide 107j (09/02/2027)</t>
+          <t>Valide 106j (09/02/2027)</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>107j</t>
+          <t>106j</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
-          <t>Valide 391j (20/11/2027)</t>
+          <t>Valide 390j (20/11/2027)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>25/10/2026 12:24</t>
+          <t>26/10/2026 14:01</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
@@ -2079,22 +2079,22 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Valide 107j (09/02/2027)</t>
+          <t>Valide 106j (09/02/2027)</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>107j</t>
+          <t>106j</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Valide 391j (20/11/2027)</t>
+          <t>Valide 390j (20/11/2027)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>25/10/2026 12:24</t>
+          <t>26/10/2026 14:01</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
@@ -2289,22 +2289,22 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Valide 55j (19/12/2026)</t>
+          <t>Valide 54j (19/12/2026)</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>55j</t>
+          <t>54j</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>Valide 278j (31/07/2027)</t>
+          <t>Valide 277j (31/07/2027)</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>25/10/2026 12:24</t>
+          <t>26/10/2026 14:01</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
@@ -2343,22 +2343,22 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t>Valide 55j (19/12/2026)</t>
+          <t>Valide 54j (19/12/2026)</t>
         </is>
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>55j</t>
+          <t>54j</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
         <is>
-          <t>Valide 278j (31/07/2027)</t>
+          <t>Valide 277j (31/07/2027)</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>25/10/2026 12:24</t>
+          <t>26/10/2026 14:01</t>
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
@@ -2557,22 +2557,22 @@
       </c>
       <c r="L45" s="9" t="inlineStr">
         <is>
-          <t>Valide 180j (23/04/2027)</t>
+          <t>Valide 178j (23/04/2027)</t>
         </is>
       </c>
       <c r="M45" s="9" t="inlineStr">
         <is>
-          <t>180j</t>
+          <t>178j</t>
         </is>
       </c>
       <c r="N45" s="9" t="inlineStr">
         <is>
-          <t>Valide 350j (10/10/2027)</t>
+          <t>Valide 348j (10/10/2027)</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>25/10/2026 12:24</t>
+          <t>26/10/2026 14:01</t>
         </is>
       </c>
       <c r="P45" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 27/10/2026 13:07
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 38j (04/12/2026)</t>
+          <t>Valide 37j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>38j</t>
+          <t>37j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 129j (05/03/2027)</t>
+          <t>Valide 128j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>26/10/2026 14:01</t>
+          <t>27/10/2026 13:03</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 104j (07/02/2027)</t>
+          <t>Valide 103j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>104j</t>
+          <t>103j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 284j (07/08/2027)</t>
+          <t>Valide 283j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>26/10/2026 14:01</t>
+          <t>27/10/2026 13:03</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 67j (01/01/2027)</t>
+          <t>Valide 66j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>67j</t>
+          <t>66j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 91j (26/01/2027)</t>
+          <t>Valide 90j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>26/10/2026 14:01</t>
+          <t>27/10/2026 13:03</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 193j (07/05/2027)</t>
+          <t>Valide 192j (07/05/2027)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>193j</t>
+          <t>192j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 6j (02/11/2026)</t>
+          <t>Expire dans 5j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>26/10/2026 14:01</t>
+          <t>27/10/2026 13:03</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1262,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 106j (09/02/2027)</t>
+          <t>Valide 105j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>106j</t>
+          <t>105j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 124j (28/02/2027)</t>
+          <t>Valide 123j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>26/10/2026 14:01</t>
+          <t>27/10/2026 13:03</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1584,22 +1584,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 104j (07/02/2027)</t>
+          <t>Valide 103j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>104j</t>
+          <t>103j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 268j (22/07/2027)</t>
+          <t>Valide 267j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>26/10/2026 14:01</t>
+          <t>27/10/2026 13:03</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1654,22 +1654,22 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 178j (23/04/2027)</t>
+          <t>Valide 177j (23/04/2027)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>178j</t>
+          <t>177j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Valide 364j (25/10/2027)</t>
+          <t>Valide 363j (25/10/2027)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>26/10/2026 14:01</t>
+          <t>27/10/2026 13:03</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1749,22 +1749,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 64j (29/12/2026)</t>
+          <t>Valide 63j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>64j</t>
+          <t>63j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 42j (07/12/2026)</t>
+          <t>Valide 41j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>26/10/2026 14:01</t>
+          <t>27/10/2026 13:03</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 64j (29/12/2026)</t>
+          <t>Valide 63j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>64j</t>
+          <t>63j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 42j (07/12/2026)</t>
+          <t>Valide 41j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>26/10/2026 14:01</t>
+          <t>27/10/2026 13:03</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2017,22 +2017,22 @@
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t>Valide 106j (09/02/2027)</t>
+          <t>Valide 105j (09/02/2027)</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>106j</t>
+          <t>105j</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
-          <t>Valide 390j (20/11/2027)</t>
+          <t>Valide 389j (20/11/2027)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>26/10/2026 14:01</t>
+          <t>27/10/2026 13:03</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
@@ -2079,22 +2079,22 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Valide 106j (09/02/2027)</t>
+          <t>Valide 105j (09/02/2027)</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>106j</t>
+          <t>105j</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Valide 390j (20/11/2027)</t>
+          <t>Valide 389j (20/11/2027)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>26/10/2026 14:01</t>
+          <t>27/10/2026 13:03</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
@@ -2289,22 +2289,22 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Valide 54j (19/12/2026)</t>
+          <t>Valide 89j (24/01/2027)</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>54j</t>
+          <t>89j</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>Valide 277j (31/07/2027)</t>
+          <t>Valide 276j (31/07/2027)</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>26/10/2026 14:01</t>
+          <t>27/10/2026 13:03</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
@@ -2343,22 +2343,22 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t>Valide 54j (19/12/2026)</t>
+          <t>Valide 89j (24/01/2027)</t>
         </is>
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>54j</t>
+          <t>89j</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
         <is>
-          <t>Valide 277j (31/07/2027)</t>
+          <t>Valide 276j (31/07/2027)</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>26/10/2026 14:01</t>
+          <t>27/10/2026 13:03</t>
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
@@ -2557,12 +2557,12 @@
       </c>
       <c r="L45" s="9" t="inlineStr">
         <is>
-          <t>Valide 178j (23/04/2027)</t>
+          <t>Valide 177j (23/04/2027)</t>
         </is>
       </c>
       <c r="M45" s="9" t="inlineStr">
         <is>
-          <t>178j</t>
+          <t>177j</t>
         </is>
       </c>
       <c r="N45" s="9" t="inlineStr">
@@ -2572,7 +2572,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>26/10/2026 14:01</t>
+          <t>27/10/2026 13:03</t>
         </is>
       </c>
       <c r="P45" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 28/10/2026 13:58
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 37j (04/12/2026)</t>
+          <t>Valide 36j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>37j</t>
+          <t>36j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 128j (05/03/2027)</t>
+          <t>Valide 127j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>27/10/2026 13:03</t>
+          <t>28/10/2026 13:53</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 103j (07/02/2027)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>103j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 283j (07/08/2027)</t>
+          <t>Valide 282j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>27/10/2026 13:03</t>
+          <t>28/10/2026 13:53</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 66j (01/01/2027)</t>
+          <t>Valide 65j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>66j</t>
+          <t>65j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 90j (26/01/2027)</t>
+          <t>Valide 89j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>27/10/2026 13:03</t>
+          <t>28/10/2026 13:53</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,29 +1152,25 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 192j (07/05/2027)</t>
+          <t>Valide 191j (07/05/2027)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>192j</t>
+          <t>191j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 5j (02/11/2026)</t>
+          <t>Expire dans 4j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>27/10/2026 13:03</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>28/10/2026 13:53</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A11" s="3" t="inlineStr">
@@ -1262,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 105j (09/02/2027)</t>
+          <t>Valide 104j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>105j</t>
+          <t>104j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 123j (28/02/2027)</t>
+          <t>Valide 122j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>27/10/2026 13:03</t>
+          <t>28/10/2026 13:53</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1584,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 103j (07/02/2027)</t>
+          <t>Valide 102j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>103j</t>
+          <t>102j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 267j (22/07/2027)</t>
+          <t>Valide 266j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>27/10/2026 13:03</t>
+          <t>28/10/2026 13:53</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1654,22 +1650,22 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 177j (23/04/2027)</t>
+          <t>Valide 176j (23/04/2027)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>177j</t>
+          <t>176j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Valide 363j (25/10/2027)</t>
+          <t>Valide 362j (25/10/2027)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>27/10/2026 13:03</t>
+          <t>28/10/2026 13:53</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1749,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 63j (29/12/2026)</t>
+          <t>Valide 62j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>63j</t>
+          <t>62j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 41j (07/12/2026)</t>
+          <t>Valide 40j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>27/10/2026 13:03</t>
+          <t>28/10/2026 13:53</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1815,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 63j (29/12/2026)</t>
+          <t>Valide 62j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>63j</t>
+          <t>62j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 41j (07/12/2026)</t>
+          <t>Valide 40j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>27/10/2026 13:03</t>
+          <t>28/10/2026 13:53</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2017,22 +2013,22 @@
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t>Valide 105j (09/02/2027)</t>
+          <t>Valide 104j (09/02/2027)</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>105j</t>
+          <t>104j</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
-          <t>Valide 389j (20/11/2027)</t>
+          <t>Valide 388j (20/11/2027)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>27/10/2026 13:03</t>
+          <t>28/10/2026 13:53</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
@@ -2079,22 +2075,22 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Valide 105j (09/02/2027)</t>
+          <t>Valide 104j (09/02/2027)</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>105j</t>
+          <t>104j</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Valide 389j (20/11/2027)</t>
+          <t>Valide 388j (20/11/2027)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>27/10/2026 13:03</t>
+          <t>28/10/2026 13:53</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
@@ -2289,22 +2285,22 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Valide 89j (24/01/2027)</t>
+          <t>Valide 87j (24/01/2027)</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>89j</t>
+          <t>87j</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>Valide 276j (31/07/2027)</t>
+          <t>Valide 275j (31/07/2027)</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>27/10/2026 13:03</t>
+          <t>28/10/2026 13:53</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
@@ -2343,22 +2339,22 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t>Valide 89j (24/01/2027)</t>
+          <t>Valide 87j (24/01/2027)</t>
         </is>
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>89j</t>
+          <t>87j</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
         <is>
-          <t>Valide 276j (31/07/2027)</t>
+          <t>Valide 275j (31/07/2027)</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>27/10/2026 13:03</t>
+          <t>28/10/2026 13:53</t>
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
@@ -2557,22 +2553,22 @@
       </c>
       <c r="L45" s="9" t="inlineStr">
         <is>
-          <t>Valide 177j (23/04/2027)</t>
+          <t>Valide 176j (23/04/2027)</t>
         </is>
       </c>
       <c r="M45" s="9" t="inlineStr">
         <is>
-          <t>177j</t>
+          <t>176j</t>
         </is>
       </c>
       <c r="N45" s="9" t="inlineStr">
         <is>
-          <t>Valide 348j (10/10/2027)</t>
+          <t>Valide 346j (10/10/2027)</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>27/10/2026 13:03</t>
+          <t>28/10/2026 13:53</t>
         </is>
       </c>
       <c r="P45" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 29/10/2026 14:03
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 36j (04/12/2026)</t>
+          <t>Valide 35j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>36j</t>
+          <t>35j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 127j (05/03/2027)</t>
+          <t>Valide 126j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>28/10/2026 13:53</t>
+          <t>29/10/2026 13:59</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 101j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>101j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 282j (07/08/2027)</t>
+          <t>Valide 281j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>28/10/2026 13:53</t>
+          <t>29/10/2026 13:59</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 65j (01/01/2027)</t>
+          <t>Valide 64j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>65j</t>
+          <t>64j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 89j (26/01/2027)</t>
+          <t>Valide 88j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>28/10/2026 13:53</t>
+          <t>29/10/2026 13:59</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 191j (07/05/2027)</t>
+          <t>Valide 190j (07/05/2027)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>191j</t>
+          <t>190j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 4j (02/11/2026)</t>
+          <t>Expire dans 3j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>28/10/2026 13:53</t>
+          <t>29/10/2026 13:59</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 104j (09/02/2027)</t>
+          <t>Valide 103j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>104j</t>
+          <t>103j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 122j (28/02/2027)</t>
+          <t>Valide 121j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>28/10/2026 13:53</t>
+          <t>29/10/2026 13:59</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 102j (07/02/2027)</t>
+          <t>Valide 101j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>102j</t>
+          <t>101j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 266j (22/07/2027)</t>
+          <t>Valide 265j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>28/10/2026 13:53</t>
+          <t>29/10/2026 13:59</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 176j (23/04/2027)</t>
+          <t>Valide 175j (23/04/2027)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>176j</t>
+          <t>175j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Valide 362j (25/10/2027)</t>
+          <t>Valide 361j (25/10/2027)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>28/10/2026 13:53</t>
+          <t>29/10/2026 13:59</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 62j (29/12/2026)</t>
+          <t>Valide 61j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>62j</t>
+          <t>61j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 40j (07/12/2026)</t>
+          <t>Valide 39j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>28/10/2026 13:53</t>
+          <t>29/10/2026 13:59</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 62j (29/12/2026)</t>
+          <t>Valide 61j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>62j</t>
+          <t>61j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 40j (07/12/2026)</t>
+          <t>Valide 39j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>28/10/2026 13:53</t>
+          <t>29/10/2026 13:59</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2013,22 +2013,22 @@
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t>Valide 104j (09/02/2027)</t>
+          <t>Valide 103j (09/02/2027)</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>104j</t>
+          <t>103j</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
-          <t>Valide 388j (20/11/2027)</t>
+          <t>Valide 387j (20/11/2027)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>28/10/2026 13:53</t>
+          <t>29/10/2026 13:59</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
@@ -2075,22 +2075,22 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Valide 104j (09/02/2027)</t>
+          <t>Valide 103j (09/02/2027)</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>104j</t>
+          <t>103j</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Valide 388j (20/11/2027)</t>
+          <t>Valide 387j (20/11/2027)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>28/10/2026 13:53</t>
+          <t>29/10/2026 13:59</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
@@ -2285,22 +2285,22 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Valide 87j (24/01/2027)</t>
+          <t>Valide 86j (24/01/2027)</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>87j</t>
+          <t>86j</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>Valide 275j (31/07/2027)</t>
+          <t>Valide 274j (31/07/2027)</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>28/10/2026 13:53</t>
+          <t>29/10/2026 13:59</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
@@ -2339,22 +2339,22 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t>Valide 87j (24/01/2027)</t>
+          <t>Valide 86j (24/01/2027)</t>
         </is>
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>87j</t>
+          <t>86j</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
         <is>
-          <t>Valide 275j (31/07/2027)</t>
+          <t>Valide 274j (31/07/2027)</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>28/10/2026 13:53</t>
+          <t>29/10/2026 13:59</t>
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
@@ -2553,22 +2553,22 @@
       </c>
       <c r="L45" s="9" t="inlineStr">
         <is>
-          <t>Valide 176j (23/04/2027)</t>
+          <t>Valide 175j (23/04/2027)</t>
         </is>
       </c>
       <c r="M45" s="9" t="inlineStr">
         <is>
-          <t>176j</t>
+          <t>175j</t>
         </is>
       </c>
       <c r="N45" s="9" t="inlineStr">
         <is>
-          <t>Valide 346j (10/10/2027)</t>
+          <t>Valide 345j (10/10/2027)</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>28/10/2026 13:53</t>
+          <t>29/10/2026 13:59</t>
         </is>
       </c>
       <c r="P45" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 30/10/2026 13:59
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 35j (04/12/2026)</t>
+          <t>Valide 34j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>35j</t>
+          <t>34j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 126j (05/03/2027)</t>
+          <t>Valide 125j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>29/10/2026 13:59</t>
+          <t>30/10/2026 13:54</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 101j (07/02/2027)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>101j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 281j (07/08/2027)</t>
+          <t>Valide 280j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>29/10/2026 13:59</t>
+          <t>30/10/2026 13:54</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 64j (01/01/2027)</t>
+          <t>Valide 63j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>64j</t>
+          <t>63j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 88j (26/01/2027)</t>
+          <t>Valide 87j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>29/10/2026 13:59</t>
+          <t>30/10/2026 13:54</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 190j (07/05/2027)</t>
+          <t>Valide 189j (07/05/2027)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>190j</t>
+          <t>189j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 3j (02/11/2026)</t>
+          <t>Expire dans 2j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>29/10/2026 13:59</t>
+          <t>30/10/2026 13:54</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 103j (09/02/2027)</t>
+          <t>Valide 102j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>103j</t>
+          <t>102j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 121j (28/02/2027)</t>
+          <t>Valide 120j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>29/10/2026 13:59</t>
+          <t>30/10/2026 13:54</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 101j (07/02/2027)</t>
+          <t>Valide 100j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>101j</t>
+          <t>100j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 265j (22/07/2027)</t>
+          <t>Valide 264j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>29/10/2026 13:59</t>
+          <t>30/10/2026 13:54</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 175j (23/04/2027)</t>
+          <t>Valide 174j (23/04/2027)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>175j</t>
+          <t>174j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Valide 361j (25/10/2027)</t>
+          <t>Valide 360j (25/10/2027)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>29/10/2026 13:59</t>
+          <t>30/10/2026 13:54</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 61j (29/12/2026)</t>
+          <t>Valide 60j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>61j</t>
+          <t>60j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 39j (07/12/2026)</t>
+          <t>Valide 38j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>29/10/2026 13:59</t>
+          <t>30/10/2026 13:54</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 61j (29/12/2026)</t>
+          <t>Valide 60j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>61j</t>
+          <t>60j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 39j (07/12/2026)</t>
+          <t>Valide 38j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>29/10/2026 13:59</t>
+          <t>30/10/2026 13:54</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2013,22 +2013,22 @@
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t>Valide 103j (09/02/2027)</t>
+          <t>Valide 102j (09/02/2027)</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>103j</t>
+          <t>102j</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
-          <t>Valide 387j (20/11/2027)</t>
+          <t>Valide 386j (20/11/2027)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>29/10/2026 13:59</t>
+          <t>30/10/2026 13:54</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
@@ -2075,22 +2075,22 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Valide 103j (09/02/2027)</t>
+          <t>Valide 102j (09/02/2027)</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>103j</t>
+          <t>102j</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Valide 387j (20/11/2027)</t>
+          <t>Valide 386j (20/11/2027)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>29/10/2026 13:59</t>
+          <t>30/10/2026 13:54</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
@@ -2285,22 +2285,22 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Valide 86j (24/01/2027)</t>
+          <t>Valide 85j (24/01/2027)</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>86j</t>
+          <t>85j</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>Valide 274j (31/07/2027)</t>
+          <t>Valide 273j (31/07/2027)</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>29/10/2026 13:59</t>
+          <t>30/10/2026 13:54</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
@@ -2339,22 +2339,22 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t>Valide 86j (24/01/2027)</t>
+          <t>Valide 85j (24/01/2027)</t>
         </is>
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>86j</t>
+          <t>85j</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
         <is>
-          <t>Valide 274j (31/07/2027)</t>
+          <t>Valide 273j (31/07/2027)</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>29/10/2026 13:59</t>
+          <t>30/10/2026 13:54</t>
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
@@ -2553,22 +2553,22 @@
       </c>
       <c r="L45" s="9" t="inlineStr">
         <is>
-          <t>Valide 175j (23/04/2027)</t>
+          <t>Valide 174j (23/04/2027)</t>
         </is>
       </c>
       <c r="M45" s="9" t="inlineStr">
         <is>
-          <t>175j</t>
+          <t>174j</t>
         </is>
       </c>
       <c r="N45" s="9" t="inlineStr">
         <is>
-          <t>Valide 345j (10/10/2027)</t>
+          <t>Valide 344j (10/10/2027)</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>29/10/2026 13:59</t>
+          <t>30/10/2026 13:54</t>
         </is>
       </c>
       <c r="P45" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 31/10/2026 13:31
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 34j (04/12/2026)</t>
+          <t>Valide 33j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>34j</t>
+          <t>33j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 125j (05/03/2027)</t>
+          <t>Valide 124j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>30/10/2026 13:54</t>
+          <t>31/10/2026 13:27</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 280j (07/08/2027)</t>
+          <t>Valide 279j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>30/10/2026 13:54</t>
+          <t>31/10/2026 13:27</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 63j (01/01/2027)</t>
+          <t>Valide 62j (01/01/2027)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>63j</t>
+          <t>62j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 87j (26/01/2027)</t>
+          <t>Valide 86j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>30/10/2026 13:54</t>
+          <t>31/10/2026 13:27</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 189j (07/05/2027)</t>
+          <t>Valide 188j (07/05/2027)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>189j</t>
+          <t>188j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 2j (02/11/2026)</t>
+          <t>Expire dans 1j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>30/10/2026 13:54</t>
+          <t>31/10/2026 13:27</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 102j (09/02/2027)</t>
+          <t>Valide 101j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>102j</t>
+          <t>101j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 120j (28/02/2027)</t>
+          <t>Valide 119j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>30/10/2026 13:54</t>
+          <t>31/10/2026 13:27</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 100j (07/02/2027)</t>
+          <t>Valide 99j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>100j</t>
+          <t>99j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 264j (22/07/2027)</t>
+          <t>Valide 263j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>30/10/2026 13:54</t>
+          <t>31/10/2026 13:27</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 174j (23/04/2027)</t>
+          <t>Valide 173j (23/04/2027)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>174j</t>
+          <t>173j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Valide 360j (25/10/2027)</t>
+          <t>Valide 359j (25/10/2027)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>30/10/2026 13:54</t>
+          <t>31/10/2026 13:27</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 60j (29/12/2026)</t>
+          <t>Valide 59j (29/12/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>60j</t>
+          <t>59j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 38j (07/12/2026)</t>
+          <t>Valide 37j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>30/10/2026 13:54</t>
+          <t>31/10/2026 13:27</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 60j (29/12/2026)</t>
+          <t>Valide 59j (29/12/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>60j</t>
+          <t>59j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 38j (07/12/2026)</t>
+          <t>Valide 37j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>30/10/2026 13:54</t>
+          <t>31/10/2026 13:27</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2013,22 +2013,22 @@
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t>Valide 102j (09/02/2027)</t>
+          <t>Valide 101j (09/02/2027)</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>102j</t>
+          <t>101j</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
-          <t>Valide 386j (20/11/2027)</t>
+          <t>Valide 385j (20/11/2027)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>30/10/2026 13:54</t>
+          <t>31/10/2026 13:27</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
@@ -2075,22 +2075,22 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Valide 102j (09/02/2027)</t>
+          <t>Valide 101j (09/02/2027)</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>102j</t>
+          <t>101j</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Valide 386j (20/11/2027)</t>
+          <t>Valide 385j (20/11/2027)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>30/10/2026 13:54</t>
+          <t>31/10/2026 13:27</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
@@ -2285,22 +2285,22 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Valide 85j (24/01/2027)</t>
+          <t>Valide 84j (24/01/2027)</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>85j</t>
+          <t>84j</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>Valide 273j (31/07/2027)</t>
+          <t>Valide 272j (31/07/2027)</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>30/10/2026 13:54</t>
+          <t>31/10/2026 13:27</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
@@ -2339,22 +2339,22 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t>Valide 85j (24/01/2027)</t>
+          <t>Valide 84j (24/01/2027)</t>
         </is>
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>85j</t>
+          <t>84j</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
         <is>
-          <t>Valide 273j (31/07/2027)</t>
+          <t>Valide 272j (31/07/2027)</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>30/10/2026 13:54</t>
+          <t>31/10/2026 13:27</t>
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
@@ -2553,22 +2553,22 @@
       </c>
       <c r="L45" s="9" t="inlineStr">
         <is>
-          <t>Valide 174j (23/04/2027)</t>
+          <t>Valide 173j (23/04/2027)</t>
         </is>
       </c>
       <c r="M45" s="9" t="inlineStr">
         <is>
-          <t>174j</t>
+          <t>173j</t>
         </is>
       </c>
       <c r="N45" s="9" t="inlineStr">
         <is>
-          <t>Valide 344j (10/10/2027)</t>
+          <t>Valide 343j (10/10/2027)</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>30/10/2026 13:54</t>
+          <t>31/10/2026 13:27</t>
         </is>
       </c>
       <c r="P45" t="inlineStr"/>

</xml_diff>